<commit_message>
Populate audited FY22-FY26 financial statements
</commit_message>
<xml_diff>
--- a/model/QinetiQ_Valuation_Model.xlsx
+++ b/model/QinetiQ_Valuation_Model.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R039025a319fb4843"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Rd8f33f0530cc4244"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="Ra66c41abe4bb4de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R5beea3abd3a445d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Ra3345494570043f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R92b077f90bdd4e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Rff30a548cec844a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="R5da24cc9b4ec4e37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R2816ebf5f4cd4f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R1e935455497a41f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,14 +17,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="dd-mmm-yyyy"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0;(#,##0.0);-"/>
     <x:numFmt numFmtId="202" formatCode="0.0%;(0.0%);-"/>
     <x:numFmt numFmtId="203" formatCode="0.0x"/>
     <x:numFmt numFmtId="204" formatCode="0.00;(0.00);0.00"/>
+    <x:numFmt numFmtId="205" formatCode="0.00;(0.00);-"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -91,8 +92,30 @@
       <x:color rgb="FF666666"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -119,8 +142,28 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="10">
     <x:border/>
     <x:border>
       <x:bottom style="medium">
@@ -168,11 +211,16 @@
         <x:color rgb="FFFFFFFF"/>
       </x:right>
     </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="84">
+  <x:cellXfs count="129">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -344,6 +392,137 @@
     </x:xf>
     <x:xf numFmtId="204" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="9" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="14" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="14" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="14" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="12" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="12" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="9" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="15" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -825,7 +1004,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="D10" s="1" t="str">
-        <x:v>0.1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
@@ -889,7 +1068,7 @@
         <x:v>Current stage</x:v>
       </x:c>
       <x:c r="D12" s="1" t="str">
-        <x:v>Historical data collection</x:v>
+        <x:v>Audited historical statements complete</x:v>
       </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
@@ -9459,13 +9638,13 @@
   <x:cols>
     <x:col min="1" max="1" width="3" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="3" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="47" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="38" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -9558,7 +9737,7 @@
       <x:c r="A4" s="1"/>
       <x:c r="B4" s="1"/>
       <x:c r="C4" s="28" t="str">
-        <x:v>Populate FY22-FY26 from the audited annual reports; £m except EPS</x:v>
+        <x:v>Audited FY22-FY26 consolidated actuals; £m except EPS</x:v>
       </x:c>
       <x:c r="D4" s="1"/>
       <x:c r="E4" s="1"/>
@@ -9690,14 +9869,24 @@
       <x:c r="C8" s="52" t="str">
         <x:v>Revenue</x:v>
       </x:c>
-      <x:c r="D8" s="81"/>
-      <x:c r="E8" s="81"/>
-      <x:c r="F8" s="81"/>
-      <x:c r="G8" s="81"/>
-      <x:c r="H8" s="81"/>
+      <x:c r="D8" s="113" t="n">
+        <x:v>1320.4</x:v>
+      </x:c>
+      <x:c r="E8" s="113" t="n">
+        <x:v>1580.7</x:v>
+      </x:c>
+      <x:c r="F8" s="113" t="n">
+        <x:v>1912.1</x:v>
+      </x:c>
+      <x:c r="G8" s="113" t="n">
+        <x:v>1931.6</x:v>
+      </x:c>
+      <x:c r="H8" s="113" t="n">
+        <x:v>1922.6</x:v>
+      </x:c>
       <x:c r="I8" s="1"/>
       <x:c r="J8" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K8" s="1"/>
       <x:c r="L8" s="1"/>
@@ -9722,14 +9911,24 @@
       <x:c r="C9" s="52" t="str">
         <x:v>Other income</x:v>
       </x:c>
-      <x:c r="D9" s="81"/>
-      <x:c r="E9" s="81"/>
-      <x:c r="F9" s="81"/>
-      <x:c r="G9" s="81"/>
-      <x:c r="H9" s="81"/>
+      <x:c r="D9" s="113" t="n">
+        <x:v>16.7</x:v>
+      </x:c>
+      <x:c r="E9" s="113" t="n">
+        <x:v>49.6</x:v>
+      </x:c>
+      <x:c r="F9" s="113" t="n">
+        <x:v>42.2</x:v>
+      </x:c>
+      <x:c r="G9" s="113" t="n">
+        <x:v>39.2</x:v>
+      </x:c>
+      <x:c r="H9" s="113" t="n">
+        <x:v>30.1</x:v>
+      </x:c>
       <x:c r="I9" s="1"/>
       <x:c r="J9" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K9" s="1"/>
       <x:c r="L9" s="1"/>
@@ -9754,14 +9953,24 @@
       <x:c r="C10" s="52" t="str">
         <x:v>EBITDA</x:v>
       </x:c>
-      <x:c r="D10" s="81"/>
-      <x:c r="E10" s="81"/>
-      <x:c r="F10" s="81"/>
-      <x:c r="G10" s="81"/>
-      <x:c r="H10" s="81"/>
+      <x:c r="D10" s="113" t="n">
+        <x:v>187.7</x:v>
+      </x:c>
+      <x:c r="E10" s="113" t="n">
+        <x:v>247.4</x:v>
+      </x:c>
+      <x:c r="F10" s="113" t="n">
+        <x:v>283.9</x:v>
+      </x:c>
+      <x:c r="G10" s="113" t="n">
+        <x:v>164.9</x:v>
+      </x:c>
+      <x:c r="H10" s="113" t="n">
+        <x:v>289.9</x:v>
+      </x:c>
       <x:c r="I10" s="1"/>
       <x:c r="J10" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K10" s="1"/>
       <x:c r="L10" s="1"/>
@@ -9784,16 +9993,26 @@
       <x:c r="A11" s="1"/>
       <x:c r="B11" s="1"/>
       <x:c r="C11" s="52" t="str">
-        <x:v>Depreciation and amortisation</x:v>
-      </x:c>
-      <x:c r="D11" s="81"/>
-      <x:c r="E11" s="81"/>
-      <x:c r="F11" s="81"/>
-      <x:c r="G11" s="81"/>
-      <x:c r="H11" s="81"/>
+        <x:v>D&amp;A and non-current asset impairments</x:v>
+      </x:c>
+      <x:c r="D11" s="113" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E11" s="113" t="n">
+        <x:v>74.6</x:v>
+      </x:c>
+      <x:c r="F11" s="113" t="n">
+        <x:v>91.4</x:v>
+      </x:c>
+      <x:c r="G11" s="113" t="n">
+        <x:v>255.4</x:v>
+      </x:c>
+      <x:c r="H11" s="113" t="n">
+        <x:v>120.1</x:v>
+      </x:c>
       <x:c r="I11" s="1"/>
       <x:c r="J11" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K11" s="1"/>
       <x:c r="L11" s="1"/>
@@ -9815,17 +10034,32 @@
     <x:row r="12">
       <x:c r="A12" s="1"/>
       <x:c r="B12" s="1"/>
-      <x:c r="C12" s="52" t="str">
+      <x:c r="C12" s="97" t="str">
         <x:v>Statutory operating profit/(loss)</x:v>
       </x:c>
-      <x:c r="D12" s="81"/>
-      <x:c r="E12" s="81"/>
-      <x:c r="F12" s="81"/>
-      <x:c r="G12" s="81"/>
-      <x:c r="H12" s="81"/>
+      <x:c r="D12" s="114" t="n">
+        <x:f>D10-D11</x:f>
+        <x:v>123.69999999999999</x:v>
+      </x:c>
+      <x:c r="E12" s="114" t="n">
+        <x:f>E10-E11</x:f>
+        <x:v>172.8</x:v>
+      </x:c>
+      <x:c r="F12" s="114" t="n">
+        <x:f>F10-F11</x:f>
+        <x:v>192.49999999999997</x:v>
+      </x:c>
+      <x:c r="G12" s="114" t="n">
+        <x:f>G10-G11</x:f>
+        <x:v>-90.5</x:v>
+      </x:c>
+      <x:c r="H12" s="114" t="n">
+        <x:f>H10-H11</x:f>
+        <x:v>169.79999999999998</x:v>
+      </x:c>
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K12" s="1"/>
       <x:c r="L12" s="1"/>
@@ -9848,16 +10082,26 @@
       <x:c r="A13" s="1"/>
       <x:c r="B13" s="1"/>
       <x:c r="C13" s="52" t="str">
-        <x:v>Underlying operating profit</x:v>
-      </x:c>
-      <x:c r="D13" s="81"/>
-      <x:c r="E13" s="81"/>
-      <x:c r="F13" s="81"/>
-      <x:c r="G13" s="81"/>
-      <x:c r="H13" s="81"/>
+        <x:v>Underlying operating profit (incl. RDEC)</x:v>
+      </x:c>
+      <x:c r="D13" s="113" t="n">
+        <x:v>143.6</x:v>
+      </x:c>
+      <x:c r="E13" s="113" t="n">
+        <x:v>196.3</x:v>
+      </x:c>
+      <x:c r="F13" s="113" t="n">
+        <x:v>242.4</x:v>
+      </x:c>
+      <x:c r="G13" s="113" t="n">
+        <x:v>215.4</x:v>
+      </x:c>
+      <x:c r="H13" s="113" t="n">
+        <x:v>247.2</x:v>
+      </x:c>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K13" s="1"/>
       <x:c r="L13" s="1"/>
@@ -9880,16 +10124,26 @@
       <x:c r="A14" s="1"/>
       <x:c r="B14" s="1"/>
       <x:c r="C14" s="52" t="str">
-        <x:v>Net finance expense</x:v>
-      </x:c>
-      <x:c r="D14" s="81"/>
-      <x:c r="E14" s="81"/>
-      <x:c r="F14" s="81"/>
-      <x:c r="G14" s="81"/>
-      <x:c r="H14" s="81"/>
+        <x:v>Net finance and other non-operating expense/(income)</x:v>
+      </x:c>
+      <x:c r="D14" s="113" t="n">
+        <x:v>-2.2</x:v>
+      </x:c>
+      <x:c r="E14" s="113" t="n">
+        <x:v>-19.2</x:v>
+      </x:c>
+      <x:c r="F14" s="113" t="n">
+        <x:v>9.8</x:v>
+      </x:c>
+      <x:c r="G14" s="113" t="n">
+        <x:v>15.8</x:v>
+      </x:c>
+      <x:c r="H14" s="113" t="n">
+        <x:v>14.7</x:v>
+      </x:c>
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K14" s="1"/>
       <x:c r="L14" s="1"/>
@@ -9911,17 +10165,32 @@
     <x:row r="15">
       <x:c r="A15" s="1"/>
       <x:c r="B15" s="1"/>
-      <x:c r="C15" s="52" t="str">
+      <x:c r="C15" s="97" t="str">
         <x:v>Profit/(loss) before tax</x:v>
       </x:c>
-      <x:c r="D15" s="81"/>
-      <x:c r="E15" s="81"/>
-      <x:c r="F15" s="81"/>
-      <x:c r="G15" s="81"/>
-      <x:c r="H15" s="81"/>
+      <x:c r="D15" s="114" t="n">
+        <x:f>D12-D14</x:f>
+        <x:v>125.89999999999999</x:v>
+      </x:c>
+      <x:c r="E15" s="114" t="n">
+        <x:f>E12-E14</x:f>
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="F15" s="114" t="n">
+        <x:f>F12-F14</x:f>
+        <x:v>182.69999999999996</x:v>
+      </x:c>
+      <x:c r="G15" s="114" t="n">
+        <x:f>G12-G14</x:f>
+        <x:v>-106.3</x:v>
+      </x:c>
+      <x:c r="H15" s="114" t="n">
+        <x:f>H12-H14</x:f>
+        <x:v>155.1</x:v>
+      </x:c>
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K15" s="1"/>
       <x:c r="L15" s="1"/>
@@ -9944,16 +10213,26 @@
       <x:c r="A16" s="1"/>
       <x:c r="B16" s="1"/>
       <x:c r="C16" s="52" t="str">
-        <x:v>Tax expense</x:v>
-      </x:c>
-      <x:c r="D16" s="81"/>
-      <x:c r="E16" s="81"/>
-      <x:c r="F16" s="81"/>
-      <x:c r="G16" s="81"/>
-      <x:c r="H16" s="81"/>
+        <x:v>Tax expense/(income)</x:v>
+      </x:c>
+      <x:c r="D16" s="113" t="n">
+        <x:v>35.9</x:v>
+      </x:c>
+      <x:c r="E16" s="113" t="n">
+        <x:v>37.6</x:v>
+      </x:c>
+      <x:c r="F16" s="113" t="n">
+        <x:v>43.1</x:v>
+      </x:c>
+      <x:c r="G16" s="113" t="n">
+        <x:v>79.4</x:v>
+      </x:c>
+      <x:c r="H16" s="113" t="n">
+        <x:v>47.6</x:v>
+      </x:c>
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K16" s="1"/>
       <x:c r="L16" s="1"/>
@@ -9975,17 +10254,32 @@
     <x:row r="17">
       <x:c r="A17" s="1"/>
       <x:c r="B17" s="1"/>
-      <x:c r="C17" s="52" t="str">
-        <x:v>Net income</x:v>
-      </x:c>
-      <x:c r="D17" s="81"/>
-      <x:c r="E17" s="81"/>
-      <x:c r="F17" s="81"/>
-      <x:c r="G17" s="81"/>
-      <x:c r="H17" s="81"/>
+      <x:c r="C17" s="97" t="str">
+        <x:v>Profit/(loss) for the year</x:v>
+      </x:c>
+      <x:c r="D17" s="114" t="n">
+        <x:f>D15-D16</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E17" s="114" t="n">
+        <x:f>E15-E16</x:f>
+        <x:v>154.4</x:v>
+      </x:c>
+      <x:c r="F17" s="114" t="n">
+        <x:f>F15-F16</x:f>
+        <x:v>139.59999999999997</x:v>
+      </x:c>
+      <x:c r="G17" s="114" t="n">
+        <x:f>G15-G16</x:f>
+        <x:v>-185.7</x:v>
+      </x:c>
+      <x:c r="H17" s="114" t="n">
+        <x:f>H15-H16</x:f>
+        <x:v>107.5</x:v>
+      </x:c>
       <x:c r="I17" s="1"/>
       <x:c r="J17" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K17" s="1"/>
       <x:c r="L17" s="1"/>
@@ -10010,14 +10304,24 @@
       <x:c r="C18" s="52" t="str">
         <x:v>Statutory EPS (p)</x:v>
       </x:c>
-      <x:c r="D18" s="81"/>
-      <x:c r="E18" s="81"/>
-      <x:c r="F18" s="81"/>
-      <x:c r="G18" s="81"/>
-      <x:c r="H18" s="81"/>
+      <x:c r="D18" s="113" t="n">
+        <x:v>15.7</x:v>
+      </x:c>
+      <x:c r="E18" s="113" t="n">
+        <x:v>26.8</x:v>
+      </x:c>
+      <x:c r="F18" s="113" t="n">
+        <x:v>24.2</x:v>
+      </x:c>
+      <x:c r="G18" s="113" t="n">
+        <x:v>-33</x:v>
+      </x:c>
+      <x:c r="H18" s="113" t="n">
+        <x:v>20.1</x:v>
+      </x:c>
       <x:c r="I18" s="1"/>
       <x:c r="J18" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K18" s="1"/>
       <x:c r="L18" s="1"/>
@@ -10042,14 +10346,24 @@
       <x:c r="C19" s="52" t="str">
         <x:v>Underlying EPS (p)</x:v>
       </x:c>
-      <x:c r="D19" s="81"/>
-      <x:c r="E19" s="81"/>
-      <x:c r="F19" s="81"/>
-      <x:c r="G19" s="81"/>
-      <x:c r="H19" s="81"/>
+      <x:c r="D19" s="113" t="n">
+        <x:v>20.6</x:v>
+      </x:c>
+      <x:c r="E19" s="113" t="n">
+        <x:v>26.5</x:v>
+      </x:c>
+      <x:c r="F19" s="113" t="n">
+        <x:v>29.4</x:v>
+      </x:c>
+      <x:c r="G19" s="113" t="n">
+        <x:v>26.1</x:v>
+      </x:c>
+      <x:c r="H19" s="113" t="n">
+        <x:v>31.5</x:v>
+      </x:c>
       <x:c r="I19" s="1"/>
       <x:c r="J19" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p172; S007 p144; S006 p156</x:v>
       </x:c>
       <x:c r="K19" s="1"/>
       <x:c r="L19" s="1"/>
@@ -10072,11 +10386,11 @@
       <x:c r="A20" s="1"/>
       <x:c r="B20" s="1"/>
       <x:c r="C20" s="52"/>
-      <x:c r="D20" s="75"/>
-      <x:c r="E20" s="75"/>
-      <x:c r="F20" s="75"/>
-      <x:c r="G20" s="75"/>
-      <x:c r="H20" s="75"/>
+      <x:c r="D20" s="113"/>
+      <x:c r="E20" s="113"/>
+      <x:c r="F20" s="113"/>
+      <x:c r="G20" s="113"/>
+      <x:c r="H20" s="113"/>
       <x:c r="I20" s="1"/>
       <x:c r="J20" s="37"/>
       <x:c r="K20" s="1"/>
@@ -10102,11 +10416,11 @@
       <x:c r="C21" s="57" t="str">
         <x:v>Balance sheet</x:v>
       </x:c>
-      <x:c r="D21" s="82"/>
-      <x:c r="E21" s="82"/>
-      <x:c r="F21" s="82"/>
-      <x:c r="G21" s="82"/>
-      <x:c r="H21" s="82"/>
+      <x:c r="D21" s="115"/>
+      <x:c r="E21" s="115"/>
+      <x:c r="F21" s="115"/>
+      <x:c r="G21" s="115"/>
+      <x:c r="H21" s="115"/>
       <x:c r="I21" s="1"/>
       <x:c r="J21" s="37"/>
       <x:c r="K21" s="1"/>
@@ -10132,14 +10446,24 @@
       <x:c r="C22" s="52" t="str">
         <x:v>Cash and cash equivalents</x:v>
       </x:c>
-      <x:c r="D22" s="81"/>
-      <x:c r="E22" s="81"/>
-      <x:c r="F22" s="81"/>
-      <x:c r="G22" s="81"/>
-      <x:c r="H22" s="81"/>
+      <x:c r="D22" s="113" t="n">
+        <x:v>248.1</x:v>
+      </x:c>
+      <x:c r="E22" s="113" t="n">
+        <x:v>151.2</x:v>
+      </x:c>
+      <x:c r="F22" s="113" t="n">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="G22" s="113" t="n">
+        <x:v>290.6</x:v>
+      </x:c>
+      <x:c r="H22" s="113" t="n">
+        <x:v>259.2</x:v>
+      </x:c>
       <x:c r="I22" s="1"/>
       <x:c r="J22" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K22" s="1"/>
       <x:c r="L22" s="1"/>
@@ -10164,14 +10488,24 @@
       <x:c r="C23" s="52" t="str">
         <x:v>Trade and other receivables</x:v>
       </x:c>
-      <x:c r="D23" s="81"/>
-      <x:c r="E23" s="81"/>
-      <x:c r="F23" s="81"/>
-      <x:c r="G23" s="81"/>
-      <x:c r="H23" s="81"/>
+      <x:c r="D23" s="113" t="n">
+        <x:v>373.2</x:v>
+      </x:c>
+      <x:c r="E23" s="113" t="n">
+        <x:v>452.6</x:v>
+      </x:c>
+      <x:c r="F23" s="113" t="n">
+        <x:v>456.8</x:v>
+      </x:c>
+      <x:c r="G23" s="113" t="n">
+        <x:v>388.4</x:v>
+      </x:c>
+      <x:c r="H23" s="113" t="n">
+        <x:v>394.9</x:v>
+      </x:c>
       <x:c r="I23" s="1"/>
       <x:c r="J23" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p192; S007 p162; S006 p175</x:v>
       </x:c>
       <x:c r="K23" s="1"/>
       <x:c r="L23" s="1"/>
@@ -10194,16 +10528,26 @@
       <x:c r="A24" s="1"/>
       <x:c r="B24" s="1"/>
       <x:c r="C24" s="52" t="str">
-        <x:v>Contract assets</x:v>
-      </x:c>
-      <x:c r="D24" s="81"/>
-      <x:c r="E24" s="81"/>
-      <x:c r="F24" s="81"/>
-      <x:c r="G24" s="81"/>
-      <x:c r="H24" s="81"/>
+        <x:v>of which: contract assets</x:v>
+      </x:c>
+      <x:c r="D24" s="113" t="n">
+        <x:v>145.8</x:v>
+      </x:c>
+      <x:c r="E24" s="113" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="F24" s="113" t="n">
+        <x:v>171.6</x:v>
+      </x:c>
+      <x:c r="G24" s="113" t="n">
+        <x:v>154.5</x:v>
+      </x:c>
+      <x:c r="H24" s="113" t="n">
+        <x:v>178.2</x:v>
+      </x:c>
       <x:c r="I24" s="1"/>
       <x:c r="J24" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p192; S007 p162; S006 p175</x:v>
       </x:c>
       <x:c r="K24" s="1"/>
       <x:c r="L24" s="1"/>
@@ -10228,14 +10572,24 @@
       <x:c r="C25" s="52" t="str">
         <x:v>Inventory</x:v>
       </x:c>
-      <x:c r="D25" s="81"/>
-      <x:c r="E25" s="81"/>
-      <x:c r="F25" s="81"/>
-      <x:c r="G25" s="81"/>
-      <x:c r="H25" s="81"/>
+      <x:c r="D25" s="113" t="n">
+        <x:v>54.9</x:v>
+      </x:c>
+      <x:c r="E25" s="113" t="n">
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="F25" s="113" t="n">
+        <x:v>89.2</x:v>
+      </x:c>
+      <x:c r="G25" s="113" t="n">
+        <x:v>70.7</x:v>
+      </x:c>
+      <x:c r="H25" s="113" t="n">
+        <x:v>73.7</x:v>
+      </x:c>
       <x:c r="I25" s="1"/>
       <x:c r="J25" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K25" s="1"/>
       <x:c r="L25" s="1"/>
@@ -10260,14 +10614,24 @@
       <x:c r="C26" s="52" t="str">
         <x:v>Property, plant and equipment</x:v>
       </x:c>
-      <x:c r="D26" s="81"/>
-      <x:c r="E26" s="81"/>
-      <x:c r="F26" s="81"/>
-      <x:c r="G26" s="81"/>
-      <x:c r="H26" s="81"/>
+      <x:c r="D26" s="113" t="n">
+        <x:v>414.5</x:v>
+      </x:c>
+      <x:c r="E26" s="113" t="n">
+        <x:v>477.8</x:v>
+      </x:c>
+      <x:c r="F26" s="113" t="n">
+        <x:v>531.8</x:v>
+      </x:c>
+      <x:c r="G26" s="113" t="n">
+        <x:v>473.3</x:v>
+      </x:c>
+      <x:c r="H26" s="113" t="n">
+        <x:v>444.6</x:v>
+      </x:c>
       <x:c r="I26" s="1"/>
       <x:c r="J26" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K26" s="1"/>
       <x:c r="L26" s="1"/>
@@ -10292,14 +10656,24 @@
       <x:c r="C27" s="52" t="str">
         <x:v>Goodwill and intangible assets</x:v>
       </x:c>
-      <x:c r="D27" s="81"/>
-      <x:c r="E27" s="81"/>
-      <x:c r="F27" s="81"/>
-      <x:c r="G27" s="81"/>
-      <x:c r="H27" s="81"/>
+      <x:c r="D27" s="113" t="n">
+        <x:v>289.7</x:v>
+      </x:c>
+      <x:c r="E27" s="113" t="n">
+        <x:v>752</x:v>
+      </x:c>
+      <x:c r="F27" s="113" t="n">
+        <x:v>723.2</x:v>
+      </x:c>
+      <x:c r="G27" s="113" t="n">
+        <x:v>543.7</x:v>
+      </x:c>
+      <x:c r="H27" s="113" t="n">
+        <x:v>486.3</x:v>
+      </x:c>
       <x:c r="I27" s="1"/>
       <x:c r="J27" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K27" s="1"/>
       <x:c r="L27" s="1"/>
@@ -10321,17 +10695,27 @@
     <x:row r="28">
       <x:c r="A28" s="1"/>
       <x:c r="B28" s="1"/>
-      <x:c r="C28" s="52" t="str">
+      <x:c r="C28" s="97" t="str">
         <x:v>Total assets</x:v>
       </x:c>
-      <x:c r="D28" s="81"/>
-      <x:c r="E28" s="81"/>
-      <x:c r="F28" s="81"/>
-      <x:c r="G28" s="81"/>
-      <x:c r="H28" s="81"/>
+      <x:c r="D28" s="114" t="n">
+        <x:v>1768.7</x:v>
+      </x:c>
+      <x:c r="E28" s="114" t="n">
+        <x:v>2072.1</x:v>
+      </x:c>
+      <x:c r="F28" s="114" t="n">
+        <x:v>2106.2</x:v>
+      </x:c>
+      <x:c r="G28" s="114" t="n">
+        <x:v>1828.4</x:v>
+      </x:c>
+      <x:c r="H28" s="114" t="n">
+        <x:v>1738.4</x:v>
+      </x:c>
       <x:c r="I28" s="1"/>
       <x:c r="J28" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K28" s="1"/>
       <x:c r="L28" s="1"/>
@@ -10354,16 +10738,26 @@
       <x:c r="A29" s="1"/>
       <x:c r="B29" s="1"/>
       <x:c r="C29" s="52" t="str">
-        <x:v>Trade and other payables</x:v>
-      </x:c>
-      <x:c r="D29" s="81"/>
-      <x:c r="E29" s="81"/>
-      <x:c r="F29" s="81"/>
-      <x:c r="G29" s="81"/>
-      <x:c r="H29" s="81"/>
+        <x:v>Current trade and other payables</x:v>
+      </x:c>
+      <x:c r="D29" s="113" t="n">
+        <x:v>474.7</x:v>
+      </x:c>
+      <x:c r="E29" s="113" t="n">
+        <x:v>575.2</x:v>
+      </x:c>
+      <x:c r="F29" s="113" t="n">
+        <x:v>654.7</x:v>
+      </x:c>
+      <x:c r="G29" s="113" t="n">
+        <x:v>597.5</x:v>
+      </x:c>
+      <x:c r="H29" s="113" t="n">
+        <x:v>585.6</x:v>
+      </x:c>
       <x:c r="I29" s="1"/>
       <x:c r="J29" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K29" s="1"/>
       <x:c r="L29" s="1"/>
@@ -10386,16 +10780,26 @@
       <x:c r="A30" s="1"/>
       <x:c r="B30" s="1"/>
       <x:c r="C30" s="52" t="str">
-        <x:v>Contract liabilities</x:v>
-      </x:c>
-      <x:c r="D30" s="81"/>
-      <x:c r="E30" s="81"/>
-      <x:c r="F30" s="81"/>
-      <x:c r="G30" s="81"/>
-      <x:c r="H30" s="81"/>
+        <x:v>of which: current contract liabilities</x:v>
+      </x:c>
+      <x:c r="D30" s="113" t="n">
+        <x:v>182.5</x:v>
+      </x:c>
+      <x:c r="E30" s="113" t="n">
+        <x:v>216.9</x:v>
+      </x:c>
+      <x:c r="F30" s="113" t="n">
+        <x:v>212.6</x:v>
+      </x:c>
+      <x:c r="G30" s="113" t="n">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="H30" s="113" t="n">
+        <x:v>158.3</x:v>
+      </x:c>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p193; S007 p163; S006 p176</x:v>
       </x:c>
       <x:c r="K30" s="1"/>
       <x:c r="L30" s="1"/>
@@ -10418,16 +10822,26 @@
       <x:c r="A31" s="1"/>
       <x:c r="B31" s="1"/>
       <x:c r="C31" s="52" t="str">
-        <x:v>Provisions</x:v>
-      </x:c>
-      <x:c r="D31" s="81"/>
-      <x:c r="E31" s="81"/>
-      <x:c r="F31" s="81"/>
-      <x:c r="G31" s="81"/>
-      <x:c r="H31" s="81"/>
+        <x:v>Provisions (current and non-current)</x:v>
+      </x:c>
+      <x:c r="D31" s="113" t="n">
+        <x:v>27.1</x:v>
+      </x:c>
+      <x:c r="E31" s="113" t="n">
+        <x:v>26.8</x:v>
+      </x:c>
+      <x:c r="F31" s="113" t="n">
+        <x:v>19.5</x:v>
+      </x:c>
+      <x:c r="G31" s="113" t="n">
+        <x:v>59.7</x:v>
+      </x:c>
+      <x:c r="H31" s="113" t="n">
+        <x:v>50.7</x:v>
+      </x:c>
       <x:c r="I31" s="1"/>
       <x:c r="J31" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K31" s="1"/>
       <x:c r="L31" s="1"/>
@@ -10450,16 +10864,26 @@
       <x:c r="A32" s="1"/>
       <x:c r="B32" s="1"/>
       <x:c r="C32" s="52" t="str">
-        <x:v>Borrowings</x:v>
-      </x:c>
-      <x:c r="D32" s="81"/>
-      <x:c r="E32" s="81"/>
-      <x:c r="F32" s="81"/>
-      <x:c r="G32" s="81"/>
-      <x:c r="H32" s="81"/>
+        <x:v>Borrowings and other financial liabilities</x:v>
+      </x:c>
+      <x:c r="D32" s="113" t="n">
+        <x:v>24.1</x:v>
+      </x:c>
+      <x:c r="E32" s="113" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="F32" s="113" t="n">
+        <x:v>393.3</x:v>
+      </x:c>
+      <x:c r="G32" s="113" t="n">
+        <x:v>431.7</x:v>
+      </x:c>
+      <x:c r="H32" s="113" t="n">
+        <x:v>423.9</x:v>
+      </x:c>
       <x:c r="I32" s="1"/>
       <x:c r="J32" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K32" s="1"/>
       <x:c r="L32" s="1"/>
@@ -10481,17 +10905,27 @@
     <x:row r="33">
       <x:c r="A33" s="1"/>
       <x:c r="B33" s="1"/>
-      <x:c r="C33" s="52" t="str">
+      <x:c r="C33" s="97" t="str">
         <x:v>Total liabilities</x:v>
       </x:c>
-      <x:c r="D33" s="81"/>
-      <x:c r="E33" s="81"/>
-      <x:c r="F33" s="81"/>
-      <x:c r="G33" s="81"/>
-      <x:c r="H33" s="81"/>
+      <x:c r="D33" s="114" t="n">
+        <x:v>727.3</x:v>
+      </x:c>
+      <x:c r="E33" s="114" t="n">
+        <x:v>1103.8</x:v>
+      </x:c>
+      <x:c r="F33" s="114" t="n">
+        <x:v>1180.1</x:v>
+      </x:c>
+      <x:c r="G33" s="114" t="n">
+        <x:v>1201.9</x:v>
+      </x:c>
+      <x:c r="H33" s="114" t="n">
+        <x:v>1185.4</x:v>
+      </x:c>
       <x:c r="I33" s="1"/>
       <x:c r="J33" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K33" s="1"/>
       <x:c r="L33" s="1"/>
@@ -10513,17 +10947,27 @@
     <x:row r="34">
       <x:c r="A34" s="1"/>
       <x:c r="B34" s="1"/>
-      <x:c r="C34" s="52" t="str">
-        <x:v>Shareholders' equity</x:v>
-      </x:c>
-      <x:c r="D34" s="81"/>
-      <x:c r="E34" s="81"/>
-      <x:c r="F34" s="81"/>
-      <x:c r="G34" s="81"/>
-      <x:c r="H34" s="81"/>
+      <x:c r="C34" s="97" t="str">
+        <x:v>Total equity</x:v>
+      </x:c>
+      <x:c r="D34" s="114" t="n">
+        <x:v>1041.4</x:v>
+      </x:c>
+      <x:c r="E34" s="114" t="n">
+        <x:v>968.3</x:v>
+      </x:c>
+      <x:c r="F34" s="114" t="n">
+        <x:v>926.1</x:v>
+      </x:c>
+      <x:c r="G34" s="114" t="n">
+        <x:v>626.5</x:v>
+      </x:c>
+      <x:c r="H34" s="114" t="n">
+        <x:v>553</x:v>
+      </x:c>
       <x:c r="I34" s="1"/>
       <x:c r="J34" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p174; S007 p146; S006 p158</x:v>
       </x:c>
       <x:c r="K34" s="1"/>
       <x:c r="L34" s="1"/>
@@ -10545,27 +10989,32 @@
     <x:row r="35">
       <x:c r="A35" s="1"/>
       <x:c r="B35" s="1"/>
-      <x:c r="C35" s="79" t="str">
+      <x:c r="C35" s="100" t="str">
         <x:v>Balance-sheet check</x:v>
       </x:c>
-      <x:c r="D35" s="83" t="str">
-        <x:f>IF(COUNT(D28,D33,D34)=3,D28-D33-D34,"")</x:f>
-      </x:c>
-      <x:c r="E35" s="83" t="str">
-        <x:f>IF(COUNT(E28,E33,E34)=3,E28-E33-E34,"")</x:f>
-      </x:c>
-      <x:c r="F35" s="83" t="str">
-        <x:f>IF(COUNT(F28,F33,F34)=3,F28-F33-F34,"")</x:f>
-      </x:c>
-      <x:c r="G35" s="83" t="str">
-        <x:f>IF(COUNT(G28,G33,G34)=3,G28-G33-G34,"")</x:f>
-      </x:c>
-      <x:c r="H35" s="83" t="str">
-        <x:f>IF(COUNT(H28,H33,H34)=3,H28-H33-H34,"")</x:f>
+      <x:c r="D35" s="116" t="n">
+        <x:f>ROUND(D28-D33-D34,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="116" t="n">
+        <x:f>ROUND(E28-E33-E34,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="116" t="n">
+        <x:f>ROUND(F28-F33-F34,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G35" s="116" t="n">
+        <x:f>ROUND(G28-G33-G34,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H35" s="116" t="n">
+        <x:f>ROUND(H28-H33-H34,2)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I35" s="1"/>
       <x:c r="J35" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>Calculated: assets - liabilities - equity</x:v>
       </x:c>
       <x:c r="K35" s="1"/>
       <x:c r="L35" s="1"/>
@@ -10588,11 +11037,11 @@
       <x:c r="A36" s="1"/>
       <x:c r="B36" s="1"/>
       <x:c r="C36" s="52"/>
-      <x:c r="D36" s="75"/>
-      <x:c r="E36" s="75"/>
-      <x:c r="F36" s="75"/>
-      <x:c r="G36" s="75"/>
-      <x:c r="H36" s="75"/>
+      <x:c r="D36" s="113"/>
+      <x:c r="E36" s="113"/>
+      <x:c r="F36" s="113"/>
+      <x:c r="G36" s="113"/>
+      <x:c r="H36" s="113"/>
       <x:c r="I36" s="1"/>
       <x:c r="J36" s="37"/>
       <x:c r="K36" s="1"/>
@@ -10618,11 +11067,11 @@
       <x:c r="C37" s="57" t="str">
         <x:v>Cash-flow statement</x:v>
       </x:c>
-      <x:c r="D37" s="82"/>
-      <x:c r="E37" s="82"/>
-      <x:c r="F37" s="82"/>
-      <x:c r="G37" s="82"/>
-      <x:c r="H37" s="82"/>
+      <x:c r="D37" s="115"/>
+      <x:c r="E37" s="115"/>
+      <x:c r="F37" s="115"/>
+      <x:c r="G37" s="115"/>
+      <x:c r="H37" s="115"/>
       <x:c r="I37" s="1"/>
       <x:c r="J37" s="37"/>
       <x:c r="K37" s="1"/>
@@ -10646,16 +11095,31 @@
       <x:c r="A38" s="1"/>
       <x:c r="B38" s="1"/>
       <x:c r="C38" s="52" t="str">
-        <x:v>Net income</x:v>
-      </x:c>
-      <x:c r="D38" s="81"/>
-      <x:c r="E38" s="81"/>
-      <x:c r="F38" s="81"/>
-      <x:c r="G38" s="81"/>
-      <x:c r="H38" s="81"/>
+        <x:v>Profit/(loss) for the year</x:v>
+      </x:c>
+      <x:c r="D38" s="121" t="n">
+        <x:f>D17</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E38" s="121" t="n">
+        <x:f>E17</x:f>
+        <x:v>154.4</x:v>
+      </x:c>
+      <x:c r="F38" s="121" t="n">
+        <x:f>F17</x:f>
+        <x:v>139.59999999999997</x:v>
+      </x:c>
+      <x:c r="G38" s="121" t="n">
+        <x:f>G17</x:f>
+        <x:v>-185.7</x:v>
+      </x:c>
+      <x:c r="H38" s="121" t="n">
+        <x:f>H17</x:f>
+        <x:v>107.5</x:v>
+      </x:c>
       <x:c r="I38" s="1"/>
       <x:c r="J38" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p195; S007 p164; S006 pp176-177</x:v>
       </x:c>
       <x:c r="K38" s="1"/>
       <x:c r="L38" s="1"/>
@@ -10680,14 +11144,29 @@
       <x:c r="C39" s="52" t="str">
         <x:v>D&amp;A and impairments</x:v>
       </x:c>
-      <x:c r="D39" s="81"/>
-      <x:c r="E39" s="81"/>
-      <x:c r="F39" s="81"/>
-      <x:c r="G39" s="81"/>
-      <x:c r="H39" s="81"/>
+      <x:c r="D39" s="121" t="n">
+        <x:f>D11</x:f>
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="E39" s="121" t="n">
+        <x:f>E11</x:f>
+        <x:v>74.6</x:v>
+      </x:c>
+      <x:c r="F39" s="121" t="n">
+        <x:f>F11</x:f>
+        <x:v>91.4</x:v>
+      </x:c>
+      <x:c r="G39" s="121" t="n">
+        <x:f>G11</x:f>
+        <x:v>255.4</x:v>
+      </x:c>
+      <x:c r="H39" s="121" t="n">
+        <x:f>H11</x:f>
+        <x:v>120.1</x:v>
+      </x:c>
       <x:c r="I39" s="1"/>
       <x:c r="J39" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p195; S007 p164; S006 pp176-177</x:v>
       </x:c>
       <x:c r="K39" s="1"/>
       <x:c r="L39" s="1"/>
@@ -10712,14 +11191,24 @@
       <x:c r="C40" s="52" t="str">
         <x:v>Change in working capital</x:v>
       </x:c>
-      <x:c r="D40" s="81"/>
-      <x:c r="E40" s="81"/>
-      <x:c r="F40" s="81"/>
-      <x:c r="G40" s="81"/>
-      <x:c r="H40" s="81"/>
+      <x:c r="D40" s="113" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="E40" s="113" t="n">
+        <x:v>-7.7</x:v>
+      </x:c>
+      <x:c r="F40" s="113" t="n">
+        <x:v>9.8</x:v>
+      </x:c>
+      <x:c r="G40" s="113" t="n">
+        <x:v>49.8</x:v>
+      </x:c>
+      <x:c r="H40" s="113" t="n">
+        <x:v>-15.5</x:v>
+      </x:c>
       <x:c r="I40" s="1"/>
       <x:c r="J40" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p195; S007 p164; S006 pp176-177</x:v>
       </x:c>
       <x:c r="K40" s="1"/>
       <x:c r="L40" s="1"/>
@@ -10742,16 +11231,26 @@
       <x:c r="A41" s="1"/>
       <x:c r="B41" s="1"/>
       <x:c r="C41" s="52" t="str">
-        <x:v>Other operating adjustments</x:v>
-      </x:c>
-      <x:c r="D41" s="81"/>
-      <x:c r="E41" s="81"/>
-      <x:c r="F41" s="81"/>
-      <x:c r="G41" s="81"/>
-      <x:c r="H41" s="81"/>
+        <x:v>Other operating adjustments, cash tax and interest</x:v>
+      </x:c>
+      <x:c r="D41" s="113" t="n">
+        <x:v>12.7</x:v>
+      </x:c>
+      <x:c r="E41" s="113" t="n">
+        <x:v>-15.3</x:v>
+      </x:c>
+      <x:c r="F41" s="113" t="n">
+        <x:v>2.3</x:v>
+      </x:c>
+      <x:c r="G41" s="113" t="n">
+        <x:v>101.8</x:v>
+      </x:c>
+      <x:c r="H41" s="113" t="n">
+        <x:v>19.7</x:v>
+      </x:c>
       <x:c r="I41" s="1"/>
       <x:c r="J41" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p195; S007 p164; S006 pp176-177</x:v>
       </x:c>
       <x:c r="K41" s="1"/>
       <x:c r="L41" s="1"/>
@@ -10773,17 +11272,32 @@
     <x:row r="42">
       <x:c r="A42" s="1"/>
       <x:c r="B42" s="1"/>
-      <x:c r="C42" s="52" t="str">
-        <x:v>Operating cash flow</x:v>
-      </x:c>
-      <x:c r="D42" s="81"/>
-      <x:c r="E42" s="81"/>
-      <x:c r="F42" s="81"/>
-      <x:c r="G42" s="81"/>
-      <x:c r="H42" s="81"/>
+      <x:c r="C42" s="97" t="str">
+        <x:v>Net cash from operating activities</x:v>
+      </x:c>
+      <x:c r="D42" s="114" t="n">
+        <x:f>SUM(D38:D41)</x:f>
+        <x:v>188.7</x:v>
+      </x:c>
+      <x:c r="E42" s="114" t="n">
+        <x:f>SUM(E38:E41)</x:f>
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="F42" s="114" t="n">
+        <x:f>SUM(F38:F41)</x:f>
+        <x:v>243.1</x:v>
+      </x:c>
+      <x:c r="G42" s="114" t="n">
+        <x:f>SUM(G38:G41)</x:f>
+        <x:v>221.3</x:v>
+      </x:c>
+      <x:c r="H42" s="114" t="n">
+        <x:f>SUM(H38:H41)</x:f>
+        <x:v>231.79999999999998</x:v>
+      </x:c>
       <x:c r="I42" s="1"/>
       <x:c r="J42" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p195; S007 p164; S006 pp176-177</x:v>
       </x:c>
       <x:c r="K42" s="1"/>
       <x:c r="L42" s="1"/>
@@ -10808,14 +11322,24 @@
       <x:c r="C43" s="52" t="str">
         <x:v>Capital expenditure</x:v>
       </x:c>
-      <x:c r="D43" s="81"/>
-      <x:c r="E43" s="81"/>
-      <x:c r="F43" s="81"/>
-      <x:c r="G43" s="81"/>
-      <x:c r="H43" s="81"/>
+      <x:c r="D43" s="113" t="n">
+        <x:v>-84.3</x:v>
+      </x:c>
+      <x:c r="E43" s="113" t="n">
+        <x:v>-109</x:v>
+      </x:c>
+      <x:c r="F43" s="113" t="n">
+        <x:v>-96.3</x:v>
+      </x:c>
+      <x:c r="G43" s="113" t="n">
+        <x:v>-108.8</x:v>
+      </x:c>
+      <x:c r="H43" s="113" t="n">
+        <x:v>-72.5</x:v>
+      </x:c>
       <x:c r="I43" s="1"/>
       <x:c r="J43" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K43" s="1"/>
       <x:c r="L43" s="1"/>
@@ -10838,16 +11362,26 @@
       <x:c r="A44" s="1"/>
       <x:c r="B44" s="1"/>
       <x:c r="C44" s="52" t="str">
-        <x:v>Acquisitions and disposals</x:v>
-      </x:c>
-      <x:c r="D44" s="81"/>
-      <x:c r="E44" s="81"/>
-      <x:c r="F44" s="81"/>
-      <x:c r="G44" s="81"/>
-      <x:c r="H44" s="81"/>
+        <x:v>Other investing cash flow</x:v>
+      </x:c>
+      <x:c r="D44" s="113" t="n">
+        <x:v>2.7</x:v>
+      </x:c>
+      <x:c r="E44" s="113" t="n">
+        <x:v>-355.4</x:v>
+      </x:c>
+      <x:c r="F44" s="113" t="n">
+        <x:v>-2.8</x:v>
+      </x:c>
+      <x:c r="G44" s="113" t="n">
+        <x:v>109.2</x:v>
+      </x:c>
+      <x:c r="H44" s="113" t="n">
+        <x:v>17.9</x:v>
+      </x:c>
       <x:c r="I44" s="1"/>
       <x:c r="J44" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K44" s="1"/>
       <x:c r="L44" s="1"/>
@@ -10869,17 +11403,32 @@
     <x:row r="45">
       <x:c r="A45" s="1"/>
       <x:c r="B45" s="1"/>
-      <x:c r="C45" s="52" t="str">
-        <x:v>Investing cash flow</x:v>
-      </x:c>
-      <x:c r="D45" s="81"/>
-      <x:c r="E45" s="81"/>
-      <x:c r="F45" s="81"/>
-      <x:c r="G45" s="81"/>
-      <x:c r="H45" s="81"/>
+      <x:c r="C45" s="97" t="str">
+        <x:v>Net investing cash flow</x:v>
+      </x:c>
+      <x:c r="D45" s="114" t="n">
+        <x:f>SUM(D43:D44)</x:f>
+        <x:v>-81.6</x:v>
+      </x:c>
+      <x:c r="E45" s="114" t="n">
+        <x:f>SUM(E43:E44)</x:f>
+        <x:v>-464.4</x:v>
+      </x:c>
+      <x:c r="F45" s="114" t="n">
+        <x:f>SUM(F43:F44)</x:f>
+        <x:v>-99.1</x:v>
+      </x:c>
+      <x:c r="G45" s="114" t="n">
+        <x:f>SUM(G43:G44)</x:f>
+        <x:v>0.4000000000000057</x:v>
+      </x:c>
+      <x:c r="H45" s="114" t="n">
+        <x:f>SUM(H43:H44)</x:f>
+        <x:v>-54.6</x:v>
+      </x:c>
       <x:c r="I45" s="1"/>
       <x:c r="J45" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K45" s="1"/>
       <x:c r="L45" s="1"/>
@@ -10902,16 +11451,26 @@
       <x:c r="A46" s="1"/>
       <x:c r="B46" s="1"/>
       <x:c r="C46" s="52" t="str">
-        <x:v>Debt movement</x:v>
-      </x:c>
-      <x:c r="D46" s="81"/>
-      <x:c r="E46" s="81"/>
-      <x:c r="F46" s="81"/>
-      <x:c r="G46" s="81"/>
-      <x:c r="H46" s="81"/>
+        <x:v>Debt, leases, fees and hedges</x:v>
+      </x:c>
+      <x:c r="D46" s="113" t="n">
+        <x:v>-9.4</x:v>
+      </x:c>
+      <x:c r="E46" s="113" t="n">
+        <x:v>203.1</x:v>
+      </x:c>
+      <x:c r="F46" s="113" t="n">
+        <x:v>-0.5</x:v>
+      </x:c>
+      <x:c r="G46" s="113" t="n">
+        <x:v>-1.6</x:v>
+      </x:c>
+      <x:c r="H46" s="113" t="n">
+        <x:v>-12.6</x:v>
+      </x:c>
       <x:c r="I46" s="1"/>
       <x:c r="J46" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K46" s="1"/>
       <x:c r="L46" s="1"/>
@@ -10936,14 +11495,24 @@
       <x:c r="C47" s="52" t="str">
         <x:v>Dividends</x:v>
       </x:c>
-      <x:c r="D47" s="81"/>
-      <x:c r="E47" s="81"/>
-      <x:c r="F47" s="81"/>
-      <x:c r="G47" s="81"/>
-      <x:c r="H47" s="81"/>
+      <x:c r="D47" s="113" t="n">
+        <x:v>-40.2</x:v>
+      </x:c>
+      <x:c r="E47" s="113" t="n">
+        <x:v>-42.6</x:v>
+      </x:c>
+      <x:c r="F47" s="113" t="n">
+        <x:v>-45.6</x:v>
+      </x:c>
+      <x:c r="G47" s="113" t="n">
+        <x:v>-47.9</x:v>
+      </x:c>
+      <x:c r="H47" s="113" t="n">
+        <x:v>-48.7</x:v>
+      </x:c>
       <x:c r="I47" s="1"/>
       <x:c r="J47" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K47" s="1"/>
       <x:c r="L47" s="1"/>
@@ -10968,14 +11537,24 @@
       <x:c r="C48" s="52" t="str">
         <x:v>Share buybacks</x:v>
       </x:c>
-      <x:c r="D48" s="81"/>
-      <x:c r="E48" s="81"/>
-      <x:c r="F48" s="81"/>
-      <x:c r="G48" s="81"/>
-      <x:c r="H48" s="81"/>
+      <x:c r="D48" s="113" t="n">
+        <x:v>-0.8</x:v>
+      </x:c>
+      <x:c r="E48" s="113" t="n">
+        <x:v>-0.8</x:v>
+      </x:c>
+      <x:c r="F48" s="113" t="n">
+        <x:v>-17.1</x:v>
+      </x:c>
+      <x:c r="G48" s="113" t="n">
+        <x:v>-108.9</x:v>
+      </x:c>
+      <x:c r="H48" s="113" t="n">
+        <x:v>-146.9</x:v>
+      </x:c>
       <x:c r="I48" s="1"/>
       <x:c r="J48" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K48" s="1"/>
       <x:c r="L48" s="1"/>
@@ -10997,17 +11576,32 @@
     <x:row r="49">
       <x:c r="A49" s="1"/>
       <x:c r="B49" s="1"/>
-      <x:c r="C49" s="52" t="str">
-        <x:v>Financing cash flow</x:v>
-      </x:c>
-      <x:c r="D49" s="81"/>
-      <x:c r="E49" s="81"/>
-      <x:c r="F49" s="81"/>
-      <x:c r="G49" s="81"/>
-      <x:c r="H49" s="81"/>
+      <x:c r="C49" s="97" t="str">
+        <x:v>Net financing cash flow</x:v>
+      </x:c>
+      <x:c r="D49" s="114" t="n">
+        <x:f>SUM(D46:D48)</x:f>
+        <x:v>-50.4</x:v>
+      </x:c>
+      <x:c r="E49" s="114" t="n">
+        <x:f>SUM(E46:E48)</x:f>
+        <x:v>159.7</x:v>
+      </x:c>
+      <x:c r="F49" s="114" t="n">
+        <x:f>SUM(F46:F48)</x:f>
+        <x:v>-63.2</x:v>
+      </x:c>
+      <x:c r="G49" s="114" t="n">
+        <x:f>SUM(G46:G48)</x:f>
+        <x:v>-158.4</x:v>
+      </x:c>
+      <x:c r="H49" s="114" t="n">
+        <x:f>SUM(H46:H48)</x:f>
+        <x:v>-208.20000000000002</x:v>
+      </x:c>
       <x:c r="I49" s="1"/>
       <x:c r="J49" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K49" s="1"/>
       <x:c r="L49" s="1"/>
@@ -11030,16 +11624,26 @@
       <x:c r="A50" s="1"/>
       <x:c r="B50" s="1"/>
       <x:c r="C50" s="52" t="str">
-        <x:v>FX and other</x:v>
-      </x:c>
-      <x:c r="D50" s="81"/>
-      <x:c r="E50" s="81"/>
-      <x:c r="F50" s="81"/>
-      <x:c r="G50" s="81"/>
-      <x:c r="H50" s="81"/>
+        <x:v>FX impact on cash</x:v>
+      </x:c>
+      <x:c r="D50" s="113" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="E50" s="113" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="F50" s="113" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="G50" s="113" t="n">
+        <x:v>-3.7</x:v>
+      </x:c>
+      <x:c r="H50" s="113" t="n">
+        <x:v>-0.4</x:v>
+      </x:c>
       <x:c r="I50" s="1"/>
       <x:c r="J50" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K50" s="1"/>
       <x:c r="L50" s="1"/>
@@ -11061,17 +11665,32 @@
     <x:row r="51">
       <x:c r="A51" s="1"/>
       <x:c r="B51" s="1"/>
-      <x:c r="C51" s="52" t="str">
-        <x:v>Net change in cash</x:v>
-      </x:c>
-      <x:c r="D51" s="81"/>
-      <x:c r="E51" s="81"/>
-      <x:c r="F51" s="81"/>
-      <x:c r="G51" s="81"/>
-      <x:c r="H51" s="81"/>
+      <x:c r="C51" s="97" t="str">
+        <x:v>Net change in cash after FX</x:v>
+      </x:c>
+      <x:c r="D51" s="114" t="n">
+        <x:f>SUM(D42,D45,D49,D50)</x:f>
+        <x:v>57.99999999999999</x:v>
+      </x:c>
+      <x:c r="E51" s="114" t="n">
+        <x:f>SUM(E42,E45,E49,E50)</x:f>
+        <x:v>-96.89999999999999</x:v>
+      </x:c>
+      <x:c r="F51" s="114" t="n">
+        <x:f>SUM(F42,F45,F49,F50)</x:f>
+        <x:v>79.8</x:v>
+      </x:c>
+      <x:c r="G51" s="114" t="n">
+        <x:f>SUM(G42,G45,G49,G50)</x:f>
+        <x:v>59.60000000000001</x:v>
+      </x:c>
+      <x:c r="H51" s="114" t="n">
+        <x:f>SUM(H42,H45,H49,H50)</x:f>
+        <x:v>-31.400000000000027</x:v>
+      </x:c>
       <x:c r="I51" s="1"/>
       <x:c r="J51" s="37" t="str">
-        <x:v>Annual report / page</x:v>
+        <x:v>S008 p175; S007 p147; S006 p159</x:v>
       </x:c>
       <x:c r="K51" s="1"/>
       <x:c r="L51" s="1"/>
@@ -11093,14 +11712,30 @@
     <x:row r="52">
       <x:c r="A52" s="1"/>
       <x:c r="B52" s="1"/>
-      <x:c r="C52" s="52"/>
-      <x:c r="D52" s="67"/>
-      <x:c r="E52" s="67"/>
-      <x:c r="F52" s="67"/>
-      <x:c r="G52" s="67"/>
-      <x:c r="H52" s="67"/>
+      <x:c r="C52" s="100" t="str">
+        <x:v>Cash-flow check</x:v>
+      </x:c>
+      <x:c r="D52" s="116"/>
+      <x:c r="E52" s="116" t="n">
+        <x:f>ROUND(E22-D22-E51,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F52" s="116" t="n">
+        <x:f>ROUND(F22-E22-F51,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G52" s="116" t="n">
+        <x:f>ROUND(G22-F22-G51,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H52" s="116" t="n">
+        <x:f>ROUND(H22-G22-H51,2)</x:f>
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I52" s="1"/>
-      <x:c r="J52" s="1"/>
+      <x:c r="J52" s="37" t="str">
+        <x:v>Calculated: cash movement vs balance sheet</x:v>
+      </x:c>
       <x:c r="K52" s="1"/>
       <x:c r="L52" s="1"/>
       <x:c r="M52" s="1"/>
@@ -12909,12 +13544,24 @@
     <x:row r="13">
       <x:c r="A13" s="1"/>
       <x:c r="B13" s="1"/>
-      <x:c r="C13" s="1"/>
-      <x:c r="D13" s="1"/>
-      <x:c r="E13" s="1"/>
-      <x:c r="F13" s="1"/>
-      <x:c r="G13" s="1"/>
-      <x:c r="H13" s="1"/>
+      <x:c r="C13" s="123" t="str">
+        <x:v>S007</x:v>
+      </x:c>
+      <x:c r="D13" s="124" t="str">
+        <x:v>Annual Report and Accounts 2025</x:v>
+      </x:c>
+      <x:c r="E13" s="125" t="n">
+        <x:v>45799</x:v>
+      </x:c>
+      <x:c r="F13" s="124" t="str">
+        <x:v>FY24-FY25 audited statements and cash-flow reconciliation</x:v>
+      </x:c>
+      <x:c r="G13" s="124" t="str">
+        <x:v>pp.144, 146-147 and 162-164</x:v>
+      </x:c>
+      <x:c r="H13" s="124" t="str">
+        <x:v>https://www.qinetiq.com/-/media/7bd40d12009a456282f3aa28fff305ab.ashx</x:v>
+      </x:c>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
       <x:c r="K13" s="1"/>
@@ -12937,12 +13584,24 @@
     <x:row r="14">
       <x:c r="A14" s="1"/>
       <x:c r="B14" s="1"/>
-      <x:c r="C14" s="1"/>
-      <x:c r="D14" s="1"/>
-      <x:c r="E14" s="1"/>
-      <x:c r="F14" s="1"/>
-      <x:c r="G14" s="1"/>
-      <x:c r="H14" s="1"/>
+      <x:c r="C14" s="123" t="str">
+        <x:v>S008</x:v>
+      </x:c>
+      <x:c r="D14" s="124" t="str">
+        <x:v>Annual Report and Accounts 2023</x:v>
+      </x:c>
+      <x:c r="E14" s="125" t="n">
+        <x:v>45071</x:v>
+      </x:c>
+      <x:c r="F14" s="124" t="str">
+        <x:v>FY22-FY23 restated audited statements and cash-flow reconciliation</x:v>
+      </x:c>
+      <x:c r="G14" s="124" t="str">
+        <x:v>pp.172, 174-175 and 192-195</x:v>
+      </x:c>
+      <x:c r="H14" s="124" t="str">
+        <x:v>https://www.annualreports.com/HostedData/AnnualReportArchive/q/LSE_QQ.L_2023.pdf</x:v>
+      </x:c>
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
       <x:c r="K14" s="1"/>

</xml_diff>

<commit_message>
Add WACC and terminal growth sensitivity
</commit_message>
<xml_diff>
--- a/model/QinetiQ_Valuation_Model.xlsx
+++ b/model/QinetiQ_Valuation_Model.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R81adbe68bf784308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Rbbfffacc940941e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="R32241b7020fc44f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R6d003ecb74154f32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R2e24e8ebc67b47bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="R81a1ab245e38478b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R7494672db3024f04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="R89e43fa6a5c64464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="Rfec0ec7286654b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R50afd8d467e344b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R693f2a8fe056411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="R9b59678c392d4fc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1069,7 +1069,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1146,8 +1146,33 @@
         <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="21">
+  <x:borders count="22">
     <x:border diagonalUp="0" diagonalDown="0"/>
     <x:border diagonalUp="0" diagonalDown="0">
       <x:bottom style="medium">
@@ -1300,6 +1325,20 @@
         <x:color rgb="FFD9E1F2"/>
       </x:bottom>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1F2"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="21">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1330,7 +1369,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="294">
+  <x:cellXfs count="323">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2212,6 +2251,93 @@
     </x:xf>
     <x:xf numFmtId="205" fontId="27" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="26" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="26" fillId="18" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="19" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="8" fillId="17" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="26" fillId="18" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="19" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="7">
@@ -2739,7 +2865,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="1" t="str">
-        <x:v>0.4</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
@@ -2803,7 +2929,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D12" s="1" t="str">
-        <x:v>Base-case DCF valuation complete</x:v>
+        <x:v>Base-case DCF sensitivity complete</x:v>
       </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
@@ -19558,6 +19684,189 @@
       <x:c r="E108" s="208"/>
       <x:c r="F108" s="208"/>
     </x:row>
+    <x:row r="111" ht="22" customHeight="1">
+      <x:c r="A111" s="316" t="str">
+        <x:v>WACC / terminal-growth sensitivity</x:v>
+      </x:c>
+      <x:c r="B111" s="316"/>
+      <x:c r="C111" s="316"/>
+      <x:c r="D111" s="316"/>
+      <x:c r="E111" s="316"/>
+      <x:c r="F111" s="316"/>
+    </x:row>
+    <x:row r="112" ht="20" customHeight="1">
+      <x:c r="A112" s="317" t="str">
+        <x:v>Implied value per share (£)</x:v>
+      </x:c>
+      <x:c r="B112" s="318" t="n">
+        <x:f>B88-1.0%</x:f>
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C112" s="318" t="n">
+        <x:f>B88-0.5%</x:f>
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="D112" s="318" t="n">
+        <x:f>B88</x:f>
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="E112" s="318" t="n">
+        <x:f>B88+0.5%</x:f>
+        <x:v>0.025</x:v>
+      </x:c>
+      <x:c r="F112" s="318" t="n">
+        <x:f>B88+1.0%</x:f>
+        <x:v>0.03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="318" t="n">
+        <x:f>B83-1.0%</x:f>
+        <x:v>0.0758995535342735</x:v>
+      </x:c>
+      <x:c r="B113" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A113)^$B$96,$C$95/(1+$A113)^$C$96,$D$95/(1+$A113)^$D$96,$E$95/(1+$A113)^$E$96,$F$95/(1+$A113)^$F$96)+$F$95*(1+B$112)/($A113-B$112)/(1+$A113)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.682422829730986</x:v>
+      </x:c>
+      <x:c r="C113" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A113)^$B$96,$C$95/(1+$A113)^$C$96,$D$95/(1+$A113)^$D$96,$E$95/(1+$A113)^$E$96,$F$95/(1+$A113)^$F$96)+$F$95*(1+C$112)/($A113-C$112)/(1+$A113)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>6.07107253100267</x:v>
+      </x:c>
+      <x:c r="D113" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A113)^$B$96,$C$95/(1+$A113)^$C$96,$D$95/(1+$A113)^$D$96,$E$95/(1+$A113)^$E$96,$F$95/(1+$A113)^$F$96)+$F$95*(1+D$112)/($A113-D$112)/(1+$A113)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>6.52924867330995</x:v>
+      </x:c>
+      <x:c r="E113" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A113)^$B$96,$C$95/(1+$A113)^$C$96,$D$95/(1+$A113)^$D$96,$E$95/(1+$A113)^$E$96,$F$95/(1+$A113)^$F$96)+$F$95*(1+E$112)/($A113-E$112)/(1+$A113)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>7.0774405643798906</x:v>
+      </x:c>
+      <x:c r="F113" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A113)^$B$96,$C$95/(1+$A113)^$C$96,$D$95/(1+$A113)^$D$96,$E$95/(1+$A113)^$E$96,$F$95/(1+$A113)^$F$96)+$F$95*(1+F$112)/($A113-F$112)/(1+$A113)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>7.745065401711631</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="318" t="n">
+        <x:f>B83-0.5%</x:f>
+        <x:v>0.08089955353427349</x:v>
+      </x:c>
+      <x:c r="B114" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A114)^$B$96,$C$95/(1+$A114)^$C$96,$D$95/(1+$A114)^$D$96,$E$95/(1+$A114)^$E$96,$F$95/(1+$A114)^$F$96)+$F$95*(1+B$112)/($A114-B$112)/(1+$A114)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.266357287108647</x:v>
+      </x:c>
+      <x:c r="C114" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A114)^$B$96,$C$95/(1+$A114)^$C$96,$D$95/(1+$A114)^$D$96,$E$95/(1+$A114)^$E$96,$F$95/(1+$A114)^$F$96)+$F$95*(1+C$112)/($A114-C$112)/(1+$A114)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.594816396556393</x:v>
+      </x:c>
+      <x:c r="D114" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A114)^$B$96,$C$95/(1+$A114)^$C$96,$D$95/(1+$A114)^$D$96,$E$95/(1+$A114)^$E$96,$F$95/(1+$A114)^$F$96)+$F$95*(1+D$112)/($A114-D$112)/(1+$A114)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.977210073728497</x:v>
+      </x:c>
+      <x:c r="E114" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A114)^$B$96,$C$95/(1+$A114)^$C$96,$D$95/(1+$A114)^$D$96,$E$95/(1+$A114)^$E$96,$F$95/(1+$A114)^$F$96)+$F$95*(1+E$112)/($A114-E$112)/(1+$A114)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>6.428011037362675</x:v>
+      </x:c>
+      <x:c r="F114" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A114)^$B$96,$C$95/(1+$A114)^$C$96,$D$95/(1+$A114)^$D$96,$E$95/(1+$A114)^$E$96,$F$95/(1+$A114)^$F$96)+$F$95*(1+F$112)/($A114-F$112)/(1+$A114)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>6.9673787824973274</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="318" t="n">
+        <x:f>B83</x:f>
+        <x:v>0.08589955353427349</x:v>
+      </x:c>
+      <x:c r="B115" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A115)^$B$96,$C$95/(1+$A115)^$C$96,$D$95/(1+$A115)^$D$96,$E$95/(1+$A115)^$E$96,$F$95/(1+$A115)^$F$96)+$F$95*(1+B$112)/($A115-B$112)/(1+$A115)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>4.905157975801304</x:v>
+      </x:c>
+      <x:c r="C115" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A115)^$B$96,$C$95/(1+$A115)^$C$96,$D$95/(1+$A115)^$D$96,$E$95/(1+$A115)^$E$96,$F$95/(1+$A115)^$F$96)+$F$95*(1+C$112)/($A115-C$112)/(1+$A115)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.185772051885234</x:v>
+      </x:c>
+      <x:c r="D115" s="320" t="n">
+        <x:f>(SUM($B$95/(1+$A115)^$B$96,$C$95/(1+$A115)^$C$96,$D$95/(1+$A115)^$D$96,$E$95/(1+$A115)^$E$96,$F$95/(1+$A115)^$F$96)+$F$95*(1+D$112)/($A115-D$112)/(1+$A115)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.5089682185956175</x:v>
+      </x:c>
+      <x:c r="E115" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A115)^$B$96,$C$95/(1+$A115)^$C$96,$D$95/(1+$A115)^$D$96,$E$95/(1+$A115)^$E$96,$F$95/(1+$A115)^$F$96)+$F$95*(1+E$112)/($A115-E$112)/(1+$A115)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.885234752485046</x:v>
+      </x:c>
+      <x:c r="F115" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A115)^$B$96,$C$95/(1+$A115)^$C$96,$D$95/(1+$A115)^$D$96,$E$95/(1+$A115)^$E$96,$F$95/(1+$A115)^$F$96)+$F$95*(1+F$112)/($A115-F$112)/(1+$A115)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>6.328812474049477</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="318" t="n">
+        <x:f>B83+0.5%</x:f>
+        <x:v>0.0908995535342735</x:v>
+      </x:c>
+      <x:c r="B116" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A116)^$B$96,$C$95/(1+$A116)^$C$96,$D$95/(1+$A116)^$D$96,$E$95/(1+$A116)^$E$96,$F$95/(1+$A116)^$F$96)+$F$95*(1+B$112)/($A116-B$112)/(1+$A116)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>4.58865060237105</x:v>
+      </x:c>
+      <x:c r="C116" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A116)^$B$96,$C$95/(1+$A116)^$C$96,$D$95/(1+$A116)^$D$96,$E$95/(1+$A116)^$E$96,$F$95/(1+$A116)^$F$96)+$F$95*(1+C$112)/($A116-C$112)/(1+$A116)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>4.830655382679221</x:v>
+      </x:c>
+      <x:c r="D116" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A116)^$B$96,$C$95/(1+$A116)^$C$96,$D$95/(1+$A116)^$D$96,$E$95/(1+$A116)^$E$96,$F$95/(1+$A116)^$F$96)+$F$95*(1+D$112)/($A116-D$112)/(1+$A116)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.106793633262518</x:v>
+      </x:c>
+      <x:c r="E116" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A116)^$B$96,$C$95/(1+$A116)^$C$96,$D$95/(1+$A116)^$D$96,$E$95/(1+$A116)^$E$96,$F$95/(1+$A116)^$F$96)+$F$95*(1+E$112)/($A116-E$112)/(1+$A116)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.424834785424607</x:v>
+      </x:c>
+      <x:c r="F116" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A116)^$B$96,$C$95/(1+$A116)^$C$96,$D$95/(1+$A116)^$D$96,$E$95/(1+$A116)^$E$96,$F$95/(1+$A116)^$F$96)+$F$95*(1+F$112)/($A116-F$112)/(1+$A116)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.795099826548884</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="318" t="n">
+        <x:f>B83+1.0%</x:f>
+        <x:v>0.09589955353427349</x:v>
+      </x:c>
+      <x:c r="B117" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A117)^$B$96,$C$95/(1+$A117)^$C$96,$D$95/(1+$A117)^$D$96,$E$95/(1+$A117)^$E$96,$F$95/(1+$A117)^$F$96)+$F$95*(1+B$112)/($A117-B$112)/(1+$A117)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>4.309029788169878</x:v>
+      </x:c>
+      <x:c r="C117" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A117)^$B$96,$C$95/(1+$A117)^$C$96,$D$95/(1+$A117)^$D$96,$E$95/(1+$A117)^$E$96,$F$95/(1+$A117)^$F$96)+$F$95*(1+C$112)/($A117-C$112)/(1+$A117)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>4.519466403690085</x:v>
+      </x:c>
+      <x:c r="D117" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A117)^$B$96,$C$95/(1+$A117)^$C$96,$D$95/(1+$A117)^$D$96,$E$95/(1+$A117)^$E$96,$F$95/(1+$A117)^$F$96)+$F$95*(1+D$112)/($A117-D$112)/(1+$A117)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>4.757628691591909</x:v>
+      </x:c>
+      <x:c r="E117" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A117)^$B$96,$C$95/(1+$A117)^$C$96,$D$95/(1+$A117)^$D$96,$E$95/(1+$A117)^$E$96,$F$95/(1+$A117)^$F$96)+$F$95*(1+E$112)/($A117-E$112)/(1+$A117)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.029382486919331</x:v>
+      </x:c>
+      <x:c r="F117" s="319" t="n">
+        <x:f>(SUM($B$95/(1+$A117)^$B$96,$C$95/(1+$A117)^$C$96,$D$95/(1+$A117)^$D$96,$E$95/(1+$A117)^$E$96,$F$95/(1+$A117)^$F$96)+$F$95*(1+F$112)/($A117-F$112)/(1+$A117)^$F$96-$B$104)/$B$106</x:f>
+        <x:v>5.342373859855848</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="321"/>
+      <x:c r="B118" s="321"/>
+      <x:c r="C118" s="321"/>
+      <x:c r="D118" s="321"/>
+      <x:c r="E118" s="321"/>
+      <x:c r="F118" s="321"/>
+    </x:row>
+    <x:row r="119" ht="32" customHeight="1">
+      <x:c r="A119" s="322" t="str">
+        <x:v>Lower WACC and higher terminal growth increase value. The centre cell matches the £5.51 base case; the full matrix recalculates both explicit-period and terminal-value discounting.</x:v>
+      </x:c>
+      <x:c r="B119" s="322"/>
+      <x:c r="C119" s="322"/>
+      <x:c r="D119" s="322"/>
+      <x:c r="E119" s="322"/>
+      <x:c r="F119" s="322"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -19594,8 +19903,10 @@
     <x:mergeCell ref="C89:F89"/>
     <x:mergeCell ref="C90:F90"/>
     <x:mergeCell ref="A93:F93"/>
+    <x:mergeCell ref="A111:F111"/>
+    <x:mergeCell ref="A119:F119"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf83e2b9dd3044b63"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R451118abf94f4c8e"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add restructuring-case DCF valuation
</commit_message>
<xml_diff>
--- a/model/QinetiQ_Valuation_Model.xlsx
+++ b/model/QinetiQ_Valuation_Model.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R7494672db3024f04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="R89e43fa6a5c64464"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="Rfec0ec7286654b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R50afd8d467e344b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R693f2a8fe056411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="R9b59678c392d4fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rdc87691d38d4448a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Re5c7837cf80348b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="Ra89a542787154db7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="Rea7517387a7a4a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R66d0ca86384145c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="R6f7e9b285aed4bae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -876,7 +876,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="16">
+  <x:numFmts count="20">
     <x:numFmt numFmtId="164" formatCode="General"/>
     <x:numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <x:numFmt numFmtId="166" formatCode="#,##0.0;\(#,##0.0\);\-"/>
@@ -893,8 +893,12 @@
     <x:numFmt numFmtId="203" formatCode="0.0x"/>
     <x:numFmt numFmtId="204" formatCode="£0.00"/>
     <x:numFmt numFmtId="205" formatCode="0.00"/>
+    <x:numFmt numFmtId="206" formatCode="0.0;[Red](0.0);-"/>
+    <x:numFmt numFmtId="207" formatCode="#,##0.0;[Red](#,##0.0);-"/>
+    <x:numFmt numFmtId="208" formatCode="0.000"/>
+    <x:numFmt numFmtId="209" formatCode="0.00;[Red](0.00);-"/>
   </x:numFmts>
-  <x:fonts count="31">
+  <x:fonts count="32">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -1068,8 +1072,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="36">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1164,6 +1173,81 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -1369,7 +1453,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="323">
+  <x:cellXfs count="418">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2337,6 +2421,291 @@
       <x:alignment horizontal="general" vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="164" fontId="12" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="22" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="22" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="24" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="22" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="22" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="24" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="23" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="27" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="27" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="29" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="28" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="32" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="32" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2865,7 +3234,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="1" t="str">
-        <x:v>0.5</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
@@ -2929,7 +3298,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D12" s="1" t="str">
-        <x:v>Base-case DCF sensitivity complete</x:v>
+        <x:v>Restructuring-case DCF complete</x:v>
       </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
@@ -15749,12 +16118,24 @@
     <x:row r="22" ht="15" hidden="0">
       <x:c r="A22" s="1"/>
       <x:c r="B22" s="1"/>
-      <x:c r="C22" s="1"/>
-      <x:c r="D22" s="1"/>
-      <x:c r="E22" s="1"/>
-      <x:c r="F22" s="1"/>
-      <x:c r="G22" s="1"/>
-      <x:c r="H22" s="1"/>
+      <x:c r="C22" s="1" t="str">
+        <x:v>S016</x:v>
+      </x:c>
+      <x:c r="D22" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E22" s="1" t="str">
+        <x:v>2025-03-17</x:v>
+      </x:c>
+      <x:c r="F22" s="1" t="str">
+        <x:v>QinetiQ Group plc</x:v>
+      </x:c>
+      <x:c r="G22" s="1" t="str">
+        <x:v>FY25 Fourth Quarter Trading Update</x:v>
+      </x:c>
+      <x:c r="H22" s="1" t="str">
+        <x:v>https://www.qinetiq.com/en/news/qinetiq-group-plc-fy25-fourth-quarter-trading-update</x:v>
+      </x:c>
       <x:c r="I22" s="1"/>
       <x:c r="J22" s="1"/>
       <x:c r="K22" s="1"/>
@@ -19866,6 +20247,1276 @@
       <x:c r="D119" s="322"/>
       <x:c r="E119" s="322"/>
       <x:c r="F119" s="322"/>
+    </x:row>
+    <x:row r="122" ht="22" customHeight="1">
+      <x:c r="A122" s="407" t="str">
+        <x:v>Restructuring-case assumptions</x:v>
+      </x:c>
+      <x:c r="B122" s="407"/>
+      <x:c r="C122" s="407"/>
+      <x:c r="D122" s="407"/>
+      <x:c r="E122" s="407"/>
+      <x:c r="F122" s="407"/>
+      <x:c r="G122" s="321"/>
+    </x:row>
+    <x:row r="123" ht="20" customHeight="1">
+      <x:c r="A123" s="408" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="B123" s="409" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="C123" s="409" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="D123" s="409" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="E123" s="409" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="F123" s="409" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+      <x:c r="G123" s="321"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="366" t="str">
+        <x:v>Global Solutions revenue growth</x:v>
+      </x:c>
+      <x:c r="B124" s="367" t="n">
+        <x:v>-0.04</x:v>
+      </x:c>
+      <x:c r="C124" s="367" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D124" s="367" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="E124" s="367" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="F124" s="367" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="G124" s="321"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="366" t="str">
+        <x:v>Global Solutions operating margin</x:v>
+      </x:c>
+      <x:c r="B125" s="367" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="C125" s="367" t="n">
+        <x:v>0.09</x:v>
+      </x:c>
+      <x:c r="D125" s="367" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="E125" s="367" t="n">
+        <x:v>0.105</x:v>
+      </x:c>
+      <x:c r="F125" s="367" t="n">
+        <x:v>0.11</x:v>
+      </x:c>
+      <x:c r="G125" s="321"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="366" t="str">
+        <x:v>Gross restructuring cash costs (£m)</x:v>
+      </x:c>
+      <x:c r="B126" s="368" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C126" s="368" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D126" s="368" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E126" s="368" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F126" s="368" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G126" s="321"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="366" t="str">
+        <x:v>After-tax restructuring cash costs (£m)</x:v>
+      </x:c>
+      <x:c r="B127" s="369" t="n">
+        <x:f>B126*(1-B45)</x:f>
+        <x:v>11.025</x:v>
+      </x:c>
+      <x:c r="C127" s="369" t="n">
+        <x:f>C126*(1-C45)</x:f>
+        <x:v>7.35</x:v>
+      </x:c>
+      <x:c r="D127" s="369" t="n">
+        <x:f>D126*(1-D45)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E127" s="369" t="n">
+        <x:f>E126*(1-E45)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F127" s="369" t="n">
+        <x:f>F126*(1-F45)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G127" s="321"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="370" t="str">
+        <x:v>Implementation status</x:v>
+      </x:c>
+      <x:c r="B128" s="371" t="str">
+        <x:v>Main actions</x:v>
+      </x:c>
+      <x:c r="C128" s="371" t="str">
+        <x:v>Completion</x:v>
+      </x:c>
+      <x:c r="D128" s="371" t="str">
+        <x:v>Benefits building</x:v>
+      </x:c>
+      <x:c r="E128" s="371" t="str">
+        <x:v>Fully implemented</x:v>
+      </x:c>
+      <x:c r="F128" s="371" t="str">
+        <x:v>Steady state</x:v>
+      </x:c>
+      <x:c r="G128" s="321"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="321"/>
+      <x:c r="B129" s="321"/>
+      <x:c r="C129" s="321"/>
+      <x:c r="D129" s="321"/>
+      <x:c r="E129" s="321"/>
+      <x:c r="F129" s="321"/>
+      <x:c r="G129" s="321"/>
+    </x:row>
+    <x:row r="130" ht="34" customHeight="1">
+      <x:c r="A130" s="417" t="str">
+        <x:v>Hypothetical incremental restructuring case. Assumptions and evidence are documented in research/restructuring_case_assumptions.md; costs are estimates, not management guidance.</x:v>
+      </x:c>
+      <x:c r="B130" s="417"/>
+      <x:c r="C130" s="417"/>
+      <x:c r="D130" s="417"/>
+      <x:c r="E130" s="417"/>
+      <x:c r="F130" s="417"/>
+      <x:c r="G130" s="321"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="321"/>
+      <x:c r="B131" s="321"/>
+      <x:c r="C131" s="321"/>
+      <x:c r="D131" s="321"/>
+      <x:c r="E131" s="321"/>
+      <x:c r="F131" s="321"/>
+      <x:c r="G131" s="321"/>
+    </x:row>
+    <x:row r="132" ht="22" customHeight="1">
+      <x:c r="A132" s="407" t="str">
+        <x:v>Restructuring-case segment forecast</x:v>
+      </x:c>
+      <x:c r="B132" s="407"/>
+      <x:c r="C132" s="407"/>
+      <x:c r="D132" s="407"/>
+      <x:c r="E132" s="407"/>
+      <x:c r="F132" s="407"/>
+      <x:c r="G132" s="407"/>
+    </x:row>
+    <x:row r="133" ht="20" customHeight="1">
+      <x:c r="A133" s="408" t="str">
+        <x:v>£m except percentages</x:v>
+      </x:c>
+      <x:c r="B133" s="409" t="str">
+        <x:v>FY26A</x:v>
+      </x:c>
+      <x:c r="C133" s="409" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="D133" s="409" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="E133" s="409" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="F133" s="409" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="G133" s="409" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="321" t="str">
+        <x:v>EMEA Services revenue</x:v>
+      </x:c>
+      <x:c r="B134" s="373" t="n">
+        <x:f>B15</x:f>
+        <x:v>1529.2</x:v>
+      </x:c>
+      <x:c r="C134" s="373" t="n">
+        <x:f>C15</x:f>
+        <x:v>1605.66</x:v>
+      </x:c>
+      <x:c r="D134" s="373" t="n">
+        <x:f>D15</x:f>
+        <x:v>1685.9430000000002</x:v>
+      </x:c>
+      <x:c r="E134" s="373" t="n">
+        <x:f>E15</x:f>
+        <x:v>1761.810435</x:v>
+      </x:c>
+      <x:c r="F134" s="373" t="n">
+        <x:f>F15</x:f>
+        <x:v>1832.2828524000001</x:v>
+      </x:c>
+      <x:c r="G134" s="373" t="n">
+        <x:f>G15</x:f>
+        <x:v>1896.412752234</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="321" t="str">
+        <x:v>Global Solutions revenue</x:v>
+      </x:c>
+      <x:c r="B135" s="373" t="n">
+        <x:f>B16</x:f>
+        <x:v>393.4</x:v>
+      </x:c>
+      <x:c r="C135" s="373" t="n">
+        <x:f>B135*(1+B124)</x:f>
+        <x:v>377.664</x:v>
+      </x:c>
+      <x:c r="D135" s="373" t="n">
+        <x:f>C135*(1+C124)</x:f>
+        <x:v>377.664</x:v>
+      </x:c>
+      <x:c r="E135" s="373" t="n">
+        <x:f>D135*(1+D124)</x:f>
+        <x:v>392.77056</x:v>
+      </x:c>
+      <x:c r="F135" s="373" t="n">
+        <x:f>E135*(1+E124)</x:f>
+        <x:v>412.409088</x:v>
+      </x:c>
+      <x:c r="G135" s="373" t="n">
+        <x:f>F135*(1+F124)</x:f>
+        <x:v>428.90545152</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="321" t="str">
+        <x:v>Group revenue</x:v>
+      </x:c>
+      <x:c r="B136" s="373" t="n">
+        <x:f>B134+B135</x:f>
+        <x:v>1922.6</x:v>
+      </x:c>
+      <x:c r="C136" s="373" t="n">
+        <x:f>C134+C135</x:f>
+        <x:v>1983.324</x:v>
+      </x:c>
+      <x:c r="D136" s="373" t="n">
+        <x:f>D134+D135</x:f>
+        <x:v>2063.607</x:v>
+      </x:c>
+      <x:c r="E136" s="373" t="n">
+        <x:f>E134+E135</x:f>
+        <x:v>2154.5809950000003</x:v>
+      </x:c>
+      <x:c r="F136" s="373" t="n">
+        <x:f>F134+F135</x:f>
+        <x:v>2244.6919404</x:v>
+      </x:c>
+      <x:c r="G136" s="373" t="n">
+        <x:f>G134+G135</x:f>
+        <x:v>2325.318203754</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="321" t="str">
+        <x:v>Group revenue growth</x:v>
+      </x:c>
+      <x:c r="B137" s="374" t="n">
+        <x:f>B18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C137" s="374" t="n">
+        <x:f>C136/B136-1</x:f>
+        <x:v>0.03158431290960162</x:v>
+      </x:c>
+      <x:c r="D137" s="374" t="n">
+        <x:f>D136/C136-1</x:f>
+        <x:v>0.040479014018889536</x:v>
+      </x:c>
+      <x:c r="E137" s="374" t="n">
+        <x:f>E136/D136-1</x:f>
+        <x:v>0.044084942045651276</x:v>
+      </x:c>
+      <x:c r="F137" s="374" t="n">
+        <x:f>F136/E136-1</x:f>
+        <x:v>0.04182295565082694</x:v>
+      </x:c>
+      <x:c r="G137" s="374" t="n">
+        <x:f>G136/F136-1</x:f>
+        <x:v>0.035918631818864455</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="321" t="str"/>
+      <x:c r="B138" s="375"/>
+      <x:c r="C138" s="375"/>
+      <x:c r="D138" s="375"/>
+      <x:c r="E138" s="375"/>
+      <x:c r="F138" s="375"/>
+      <x:c r="G138" s="375"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="321" t="str">
+        <x:v>EMEA Services operating profit</x:v>
+      </x:c>
+      <x:c r="B139" s="376" t="n">
+        <x:f>Segments!H16</x:f>
+        <x:v>182.3</x:v>
+      </x:c>
+      <x:c r="C139" s="373" t="n">
+        <x:f>C20</x:f>
+        <x:v>191.07354</x:v>
+      </x:c>
+      <x:c r="D139" s="373" t="n">
+        <x:f>D20</x:f>
+        <x:v>202.31316</x:v>
+      </x:c>
+      <x:c r="E139" s="373" t="n">
+        <x:f>E20</x:f>
+        <x:v>213.179062635</x:v>
+      </x:c>
+      <x:c r="F139" s="373" t="n">
+        <x:f>F20</x:f>
+        <x:v>221.70622514040002</x:v>
+      </x:c>
+      <x:c r="G139" s="373" t="n">
+        <x:f>G20</x:f>
+        <x:v>227.56953026808</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="321" t="str">
+        <x:v>Global Solutions operating profit</x:v>
+      </x:c>
+      <x:c r="B140" s="376" t="n">
+        <x:f>Segments!H17</x:f>
+        <x:v>35.6</x:v>
+      </x:c>
+      <x:c r="C140" s="373" t="n">
+        <x:f>C135*B125</x:f>
+        <x:v>28.3248</x:v>
+      </x:c>
+      <x:c r="D140" s="373" t="n">
+        <x:f>D135*C125</x:f>
+        <x:v>33.98976</x:v>
+      </x:c>
+      <x:c r="E140" s="373" t="n">
+        <x:f>E135*D125</x:f>
+        <x:v>39.277056</x:v>
+      </x:c>
+      <x:c r="F140" s="373" t="n">
+        <x:f>F135*E125</x:f>
+        <x:v>43.30295424</x:v>
+      </x:c>
+      <x:c r="G140" s="373" t="n">
+        <x:f>G135*F125</x:f>
+        <x:v>47.1795996672</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="321" t="str">
+        <x:v>Group operating profit</x:v>
+      </x:c>
+      <x:c r="B141" s="373" t="n">
+        <x:f>B139+B140</x:f>
+        <x:v>217.9</x:v>
+      </x:c>
+      <x:c r="C141" s="373" t="n">
+        <x:f>C139+C140</x:f>
+        <x:v>219.39834000000002</x:v>
+      </x:c>
+      <x:c r="D141" s="373" t="n">
+        <x:f>D139+D140</x:f>
+        <x:v>236.30292</x:v>
+      </x:c>
+      <x:c r="E141" s="373" t="n">
+        <x:f>E139+E140</x:f>
+        <x:v>252.456118635</x:v>
+      </x:c>
+      <x:c r="F141" s="373" t="n">
+        <x:f>F139+F140</x:f>
+        <x:v>265.00917938040004</x:v>
+      </x:c>
+      <x:c r="G141" s="373" t="n">
+        <x:f>G139+G140</x:f>
+        <x:v>274.74912993528</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="321" t="str">
+        <x:v>Group operating margin</x:v>
+      </x:c>
+      <x:c r="B142" s="374" t="n">
+        <x:f>B141/B136</x:f>
+        <x:v>0.11333610735462396</x:v>
+      </x:c>
+      <x:c r="C142" s="374" t="n">
+        <x:f>C141/C136</x:f>
+        <x:v>0.11062153233662277</x:v>
+      </x:c>
+      <x:c r="D142" s="374" t="n">
+        <x:f>D141/D136</x:f>
+        <x:v>0.1145096522739068</x:v>
+      </x:c>
+      <x:c r="E142" s="374" t="n">
+        <x:f>E141/E136</x:f>
+        <x:v>0.11717179313326301</x:v>
+      </x:c>
+      <x:c r="F142" s="374" t="n">
+        <x:f>F141/F136</x:f>
+        <x:v>0.11806037817963382</x:v>
+      </x:c>
+      <x:c r="G142" s="374" t="n">
+        <x:f>G141/G136</x:f>
+        <x:v>0.11815549781175078</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="321"/>
+      <x:c r="B143" s="321"/>
+      <x:c r="C143" s="321"/>
+      <x:c r="D143" s="321"/>
+      <x:c r="E143" s="321"/>
+      <x:c r="F143" s="321"/>
+      <x:c r="G143" s="321"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="321"/>
+      <x:c r="B144" s="321"/>
+      <x:c r="C144" s="321"/>
+      <x:c r="D144" s="321"/>
+      <x:c r="E144" s="321"/>
+      <x:c r="F144" s="321"/>
+      <x:c r="G144" s="321"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="321"/>
+      <x:c r="B145" s="321"/>
+      <x:c r="C145" s="321"/>
+      <x:c r="D145" s="321"/>
+      <x:c r="E145" s="321"/>
+      <x:c r="F145" s="321"/>
+      <x:c r="G145" s="321"/>
+    </x:row>
+    <x:row r="146" ht="22" customHeight="1">
+      <x:c r="A146" s="407" t="str">
+        <x:v>Restructuring-case unlevered free cash flow</x:v>
+      </x:c>
+      <x:c r="B146" s="407"/>
+      <x:c r="C146" s="407"/>
+      <x:c r="D146" s="407"/>
+      <x:c r="E146" s="407"/>
+      <x:c r="F146" s="407"/>
+      <x:c r="G146" s="321"/>
+    </x:row>
+    <x:row r="147" ht="20" customHeight="1">
+      <x:c r="A147" s="408" t="str">
+        <x:v>£m except percentages</x:v>
+      </x:c>
+      <x:c r="B147" s="409" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="C147" s="409" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="D147" s="409" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="E147" s="409" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="F147" s="409" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+      <x:c r="G147" s="321"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="321" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="B148" s="377" t="n">
+        <x:f>C136</x:f>
+        <x:v>1983.324</x:v>
+      </x:c>
+      <x:c r="C148" s="377" t="n">
+        <x:f>D136</x:f>
+        <x:v>2063.607</x:v>
+      </x:c>
+      <x:c r="D148" s="377" t="n">
+        <x:f>E136</x:f>
+        <x:v>2154.5809950000003</x:v>
+      </x:c>
+      <x:c r="E148" s="377" t="n">
+        <x:f>F136</x:f>
+        <x:v>2244.6919404</x:v>
+      </x:c>
+      <x:c r="F148" s="377" t="n">
+        <x:f>G136</x:f>
+        <x:v>2325.318203754</x:v>
+      </x:c>
+      <x:c r="G148" s="321"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="321" t="str">
+        <x:v>EBIT</x:v>
+      </x:c>
+      <x:c r="B149" s="377" t="n">
+        <x:f>C141</x:f>
+        <x:v>219.39834000000002</x:v>
+      </x:c>
+      <x:c r="C149" s="377" t="n">
+        <x:f>D141</x:f>
+        <x:v>236.30292</x:v>
+      </x:c>
+      <x:c r="D149" s="377" t="n">
+        <x:f>E141</x:f>
+        <x:v>252.456118635</x:v>
+      </x:c>
+      <x:c r="E149" s="377" t="n">
+        <x:f>F141</x:f>
+        <x:v>265.00917938040004</x:v>
+      </x:c>
+      <x:c r="F149" s="377" t="n">
+        <x:f>G141</x:f>
+        <x:v>274.74912993528</x:v>
+      </x:c>
+      <x:c r="G149" s="321"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="321" t="str">
+        <x:v>Cash tax rate</x:v>
+      </x:c>
+      <x:c r="B150" s="378" t="n">
+        <x:f>B45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="C150" s="378" t="n">
+        <x:f>C45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="D150" s="378" t="n">
+        <x:f>D45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="E150" s="378" t="n">
+        <x:f>E45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="F150" s="378" t="n">
+        <x:f>F45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="G150" s="321"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="321" t="str">
+        <x:v>NOPAT</x:v>
+      </x:c>
+      <x:c r="B151" s="377" t="n">
+        <x:f>B149*(1-B150)</x:f>
+        <x:v>161.2577799</x:v>
+      </x:c>
+      <x:c r="C151" s="377" t="n">
+        <x:f>C149*(1-C150)</x:f>
+        <x:v>173.6826462</x:v>
+      </x:c>
+      <x:c r="D151" s="377" t="n">
+        <x:f>D149*(1-D150)</x:f>
+        <x:v>185.555247196725</x:v>
+      </x:c>
+      <x:c r="E151" s="377" t="n">
+        <x:f>E149*(1-E150)</x:f>
+        <x:v>194.78174684459404</x:v>
+      </x:c>
+      <x:c r="F151" s="377" t="n">
+        <x:f>F149*(1-F150)</x:f>
+        <x:v>201.9406105024308</x:v>
+      </x:c>
+      <x:c r="G151" s="321"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="321" t="str">
+        <x:v>D&amp;A</x:v>
+      </x:c>
+      <x:c r="B152" s="377" t="n">
+        <x:f>B148*B46</x:f>
+        <x:v>99.1662</x:v>
+      </x:c>
+      <x:c r="C152" s="377" t="n">
+        <x:f>C148*C46</x:f>
+        <x:v>103.18035</x:v>
+      </x:c>
+      <x:c r="D152" s="377" t="n">
+        <x:f>D148*D46</x:f>
+        <x:v>107.72904975000002</x:v>
+      </x:c>
+      <x:c r="E152" s="377" t="n">
+        <x:f>E148*E46</x:f>
+        <x:v>112.23459702000001</x:v>
+      </x:c>
+      <x:c r="F152" s="377" t="n">
+        <x:f>F148*F46</x:f>
+        <x:v>116.2659101877</x:v>
+      </x:c>
+      <x:c r="G152" s="321"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="321" t="str">
+        <x:v>CapEx</x:v>
+      </x:c>
+      <x:c r="B153" s="377" t="n">
+        <x:f>-B148*B47</x:f>
+        <x:v>-89.24958</x:v>
+      </x:c>
+      <x:c r="C153" s="377" t="n">
+        <x:f>-C148*C47</x:f>
+        <x:v>-92.862315</x:v>
+      </x:c>
+      <x:c r="D153" s="377" t="n">
+        <x:f>-D148*D47</x:f>
+        <x:v>-96.95614477500001</x:v>
+      </x:c>
+      <x:c r="E153" s="377" t="n">
+        <x:f>-E148*E47</x:f>
+        <x:v>-101.011137318</x:v>
+      </x:c>
+      <x:c r="F153" s="377" t="n">
+        <x:f>-F148*F47</x:f>
+        <x:v>-104.63931916893</x:v>
+      </x:c>
+      <x:c r="G153" s="321"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="321" t="str">
+        <x:v>Change in NWC</x:v>
+      </x:c>
+      <x:c r="B154" s="377" t="n">
+        <x:f>-(B148-$B$136)*B48</x:f>
+        <x:v>-0.6072400000000017</x:v>
+      </x:c>
+      <x:c r="C154" s="377" t="n">
+        <x:f>-(C148-B148)*C48</x:f>
+        <x:v>-0.802829999999999</x:v>
+      </x:c>
+      <x:c r="D154" s="377" t="n">
+        <x:f>-(D148-C148)*D48</x:f>
+        <x:v>-0.9097399500000029</x:v>
+      </x:c>
+      <x:c r="E154" s="377" t="n">
+        <x:f>-(E148-D148)*E48</x:f>
+        <x:v>-0.9011094539999976</x:v>
+      </x:c>
+      <x:c r="F154" s="377" t="n">
+        <x:f>-(F148-E148)*F48</x:f>
+        <x:v>-0.80626263354</x:v>
+      </x:c>
+      <x:c r="G154" s="321"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="321" t="str">
+        <x:v>UFCF before restructuring</x:v>
+      </x:c>
+      <x:c r="B155" s="377" t="n">
+        <x:f>SUM(B151:B154)</x:f>
+        <x:v>170.56715990000004</x:v>
+      </x:c>
+      <x:c r="C155" s="377" t="n">
+        <x:f>SUM(C151:C154)</x:f>
+        <x:v>183.1978512</x:v>
+      </x:c>
+      <x:c r="D155" s="377" t="n">
+        <x:f>SUM(D151:D154)</x:f>
+        <x:v>195.418412221725</x:v>
+      </x:c>
+      <x:c r="E155" s="377" t="n">
+        <x:f>SUM(E151:E154)</x:f>
+        <x:v>205.10409709259403</x:v>
+      </x:c>
+      <x:c r="F155" s="377" t="n">
+        <x:f>SUM(F151:F154)</x:f>
+        <x:v>212.76093888766079</x:v>
+      </x:c>
+      <x:c r="G155" s="321"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="321" t="str">
+        <x:v>After-tax restructuring cash costs</x:v>
+      </x:c>
+      <x:c r="B156" s="377" t="n">
+        <x:f>-B127</x:f>
+        <x:v>-11.025</x:v>
+      </x:c>
+      <x:c r="C156" s="377" t="n">
+        <x:f>-C127</x:f>
+        <x:v>-7.35</x:v>
+      </x:c>
+      <x:c r="D156" s="377" t="n">
+        <x:f>-D127</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E156" s="377" t="n">
+        <x:f>-E127</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F156" s="377" t="n">
+        <x:f>-F127</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G156" s="321"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="410" t="str">
+        <x:v>UFCF after restructuring</x:v>
+      </x:c>
+      <x:c r="B157" s="411" t="n">
+        <x:f>SUM(B155:B156)</x:f>
+        <x:v>159.54215990000003</x:v>
+      </x:c>
+      <x:c r="C157" s="411" t="n">
+        <x:f>SUM(C155:C156)</x:f>
+        <x:v>175.8478512</x:v>
+      </x:c>
+      <x:c r="D157" s="411" t="n">
+        <x:f>SUM(D155:D156)</x:f>
+        <x:v>195.418412221725</x:v>
+      </x:c>
+      <x:c r="E157" s="411" t="n">
+        <x:f>SUM(E155:E156)</x:f>
+        <x:v>205.10409709259403</x:v>
+      </x:c>
+      <x:c r="F157" s="411" t="n">
+        <x:f>SUM(F155:F156)</x:f>
+        <x:v>212.76093888766079</x:v>
+      </x:c>
+      <x:c r="G157" s="321"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="321"/>
+      <x:c r="B158" s="321"/>
+      <x:c r="C158" s="321"/>
+      <x:c r="D158" s="321"/>
+      <x:c r="E158" s="321"/>
+      <x:c r="F158" s="321"/>
+      <x:c r="G158" s="321"/>
+    </x:row>
+    <x:row r="159" ht="22" customHeight="1">
+      <x:c r="A159" s="407" t="str">
+        <x:v>Restructuring-case DCF valuation</x:v>
+      </x:c>
+      <x:c r="B159" s="407"/>
+      <x:c r="C159" s="407"/>
+      <x:c r="D159" s="407"/>
+      <x:c r="E159" s="407"/>
+      <x:c r="F159" s="407"/>
+      <x:c r="G159" s="321"/>
+    </x:row>
+    <x:row r="160" ht="20" customHeight="1">
+      <x:c r="A160" s="408" t="str">
+        <x:v>£m except per-share data</x:v>
+      </x:c>
+      <x:c r="B160" s="409" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="C160" s="409" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="D160" s="409" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="E160" s="409" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="F160" s="409" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+      <x:c r="G160" s="321"/>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="321" t="str">
+        <x:v>UFCF</x:v>
+      </x:c>
+      <x:c r="B161" s="377" t="n">
+        <x:f>B157</x:f>
+        <x:v>159.54215990000003</x:v>
+      </x:c>
+      <x:c r="C161" s="377" t="n">
+        <x:f>C157</x:f>
+        <x:v>175.8478512</x:v>
+      </x:c>
+      <x:c r="D161" s="377" t="n">
+        <x:f>D157</x:f>
+        <x:v>195.418412221725</x:v>
+      </x:c>
+      <x:c r="E161" s="377" t="n">
+        <x:f>E157</x:f>
+        <x:v>205.10409709259403</x:v>
+      </x:c>
+      <x:c r="F161" s="377" t="n">
+        <x:f>F157</x:f>
+        <x:v>212.76093888766079</x:v>
+      </x:c>
+      <x:c r="G161" s="321"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="321" t="str">
+        <x:v>Discount period</x:v>
+      </x:c>
+      <x:c r="B162" s="381" t="n">
+        <x:f>B96</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C162" s="381" t="n">
+        <x:f>C96</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="D162" s="381" t="n">
+        <x:f>D96</x:f>
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="E162" s="381" t="n">
+        <x:f>E96</x:f>
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="F162" s="381" t="n">
+        <x:f>F96</x:f>
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="G162" s="321"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="321" t="str">
+        <x:v>Discount factor</x:v>
+      </x:c>
+      <x:c r="B163" s="381" t="n">
+        <x:f>1/(1+$B$83)^B162</x:f>
+        <x:v>0.9596329968646349</x:v>
+      </x:c>
+      <x:c r="C163" s="381" t="n">
+        <x:f>1/(1+$B$83)^C162</x:f>
+        <x:v>0.883721697592858</x:v>
+      </x:c>
+      <x:c r="D163" s="381" t="n">
+        <x:f>1/(1+$B$83)^D162</x:f>
+        <x:v>0.8138153245542943</x:v>
+      </x:c>
+      <x:c r="E163" s="381" t="n">
+        <x:f>1/(1+$B$83)^E162</x:f>
+        <x:v>0.7494388609937009</x:v>
+      </x:c>
+      <x:c r="F163" s="381" t="n">
+        <x:f>1/(1+$B$83)^F162</x:f>
+        <x:v>0.6901548661241318</x:v>
+      </x:c>
+      <x:c r="G163" s="321"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="321" t="str">
+        <x:v>Present value of UFCF</x:v>
+      </x:c>
+      <x:c r="B164" s="377" t="n">
+        <x:f>B161*B163</x:f>
+        <x:v>153.1019210310938</x:v>
+      </x:c>
+      <x:c r="C164" s="377" t="n">
+        <x:f>C161*C163</x:f>
+        <x:v>155.4005615805203</x:v>
+      </x:c>
+      <x:c r="D164" s="377" t="n">
+        <x:f>D161*D163</x:f>
+        <x:v>159.034498566108</x:v>
+      </x:c>
+      <x:c r="E164" s="377" t="n">
+        <x:f>E161*E163</x:f>
+        <x:v>153.71298091021512</x:v>
+      </x:c>
+      <x:c r="F164" s="377" t="n">
+        <x:f>F161*F163</x:f>
+        <x:v>146.83799729445812</x:v>
+      </x:c>
+      <x:c r="G164" s="321"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="321" t="str"/>
+      <x:c r="B165" s="321"/>
+      <x:c r="C165" s="321"/>
+      <x:c r="D165" s="321"/>
+      <x:c r="E165" s="321"/>
+      <x:c r="F165" s="321"/>
+      <x:c r="G165" s="321"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="321" t="str">
+        <x:v>PV of explicit-period UFCF</x:v>
+      </x:c>
+      <x:c r="B166" s="377" t="n">
+        <x:f>SUM(B164:F164)</x:f>
+        <x:v>768.0879593823954</x:v>
+      </x:c>
+      <x:c r="C166" s="321"/>
+      <x:c r="D166" s="321"/>
+      <x:c r="E166" s="321"/>
+      <x:c r="F166" s="321"/>
+      <x:c r="G166" s="321"/>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="321" t="str">
+        <x:v>Terminal value</x:v>
+      </x:c>
+      <x:c r="B167" s="377" t="n">
+        <x:f>F161*(1+$B$88)/($B$83-$B$88)</x:f>
+        <x:v>3293.135477049124</x:v>
+      </x:c>
+      <x:c r="C167" s="321"/>
+      <x:c r="D167" s="321"/>
+      <x:c r="E167" s="321"/>
+      <x:c r="F167" s="321"/>
+      <x:c r="G167" s="321"/>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="321" t="str">
+        <x:v>PV of terminal value</x:v>
+      </x:c>
+      <x:c r="B168" s="377" t="n">
+        <x:f>B167*F163</x:f>
+        <x:v>2272.773474291467</x:v>
+      </x:c>
+      <x:c r="C168" s="321"/>
+      <x:c r="D168" s="321"/>
+      <x:c r="E168" s="321"/>
+      <x:c r="F168" s="321"/>
+      <x:c r="G168" s="321"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="410" t="str">
+        <x:v>Enterprise value</x:v>
+      </x:c>
+      <x:c r="B169" s="411" t="n">
+        <x:f>B166+B168</x:f>
+        <x:v>3040.861433673863</x:v>
+      </x:c>
+      <x:c r="C169" s="321"/>
+      <x:c r="D169" s="321"/>
+      <x:c r="E169" s="321"/>
+      <x:c r="F169" s="321"/>
+      <x:c r="G169" s="321"/>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="321" t="str">
+        <x:v>Less: net debt</x:v>
+      </x:c>
+      <x:c r="B170" s="377" t="n">
+        <x:f>$B$104</x:f>
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="C170" s="321"/>
+      <x:c r="D170" s="321"/>
+      <x:c r="E170" s="321"/>
+      <x:c r="F170" s="321"/>
+      <x:c r="G170" s="321"/>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="410" t="str">
+        <x:v>Equity value</x:v>
+      </x:c>
+      <x:c r="B171" s="411" t="n">
+        <x:f>B169-B170</x:f>
+        <x:v>2881.761433673863</x:v>
+      </x:c>
+      <x:c r="C171" s="321"/>
+      <x:c r="D171" s="321"/>
+      <x:c r="E171" s="321"/>
+      <x:c r="F171" s="321"/>
+      <x:c r="G171" s="321"/>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="321" t="str">
+        <x:v>Diluted shares (m)</x:v>
+      </x:c>
+      <x:c r="B172" s="377" t="n">
+        <x:f>$B$106</x:f>
+        <x:v>522.1</x:v>
+      </x:c>
+      <x:c r="C172" s="321"/>
+      <x:c r="D172" s="321"/>
+      <x:c r="E172" s="321"/>
+      <x:c r="F172" s="321"/>
+      <x:c r="G172" s="321"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="410" t="str">
+        <x:v>Implied value per share (£)</x:v>
+      </x:c>
+      <x:c r="B173" s="412" t="n">
+        <x:f>B171/B172</x:f>
+        <x:v>5.519558386657466</x:v>
+      </x:c>
+      <x:c r="C173" s="321"/>
+      <x:c r="D173" s="321"/>
+      <x:c r="E173" s="321"/>
+      <x:c r="F173" s="321"/>
+      <x:c r="G173" s="321"/>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="321" t="str">
+        <x:v>Difference vs base (£/share)</x:v>
+      </x:c>
+      <x:c r="B174" s="383" t="n">
+        <x:f>B173-$B$107</x:f>
+        <x:v>0.010590168061848537</x:v>
+      </x:c>
+      <x:c r="C174" s="321"/>
+      <x:c r="D174" s="321"/>
+      <x:c r="E174" s="321"/>
+      <x:c r="F174" s="321"/>
+      <x:c r="G174" s="321"/>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="321" t="str">
+        <x:v>Change vs base</x:v>
+      </x:c>
+      <x:c r="B175" s="378" t="n">
+        <x:f>B173/$B$107-1</x:f>
+        <x:v>0.0019223505458065837</x:v>
+      </x:c>
+      <x:c r="C175" s="321"/>
+      <x:c r="D175" s="321"/>
+      <x:c r="E175" s="321"/>
+      <x:c r="F175" s="321"/>
+      <x:c r="G175" s="321"/>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="321" t="str">
+        <x:v>Terminal value / enterprise value</x:v>
+      </x:c>
+      <x:c r="B176" s="378" t="n">
+        <x:f>B168/B169</x:f>
+        <x:v>0.7474110622481017</x:v>
+      </x:c>
+      <x:c r="C176" s="321"/>
+      <x:c r="D176" s="321"/>
+      <x:c r="E176" s="321"/>
+      <x:c r="F176" s="321"/>
+      <x:c r="G176" s="321"/>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="321"/>
+      <x:c r="B177" s="321"/>
+      <x:c r="C177" s="321"/>
+      <x:c r="D177" s="321"/>
+      <x:c r="E177" s="321"/>
+      <x:c r="F177" s="321"/>
+      <x:c r="G177" s="321"/>
+    </x:row>
+    <x:row r="178" ht="22" customHeight="1">
+      <x:c r="A178" s="407" t="str">
+        <x:v>Base case vs restructuring case</x:v>
+      </x:c>
+      <x:c r="B178" s="407"/>
+      <x:c r="C178" s="407"/>
+      <x:c r="D178" s="407"/>
+      <x:c r="E178" s="321"/>
+      <x:c r="F178" s="321"/>
+      <x:c r="G178" s="321"/>
+    </x:row>
+    <x:row r="179" ht="20" customHeight="1">
+      <x:c r="A179" s="408" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B179" s="409" t="str">
+        <x:v>Base case</x:v>
+      </x:c>
+      <x:c r="C179" s="409" t="str">
+        <x:v>Restructuring</x:v>
+      </x:c>
+      <x:c r="D179" s="409" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+      <x:c r="E179" s="321"/>
+      <x:c r="F179" s="321"/>
+      <x:c r="G179" s="321"/>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="366" t="str">
+        <x:v>FY27 UFCF (£m)</x:v>
+      </x:c>
+      <x:c r="B180" s="413" t="n">
+        <x:f>B61</x:f>
+        <x:v>174.2474169</x:v>
+      </x:c>
+      <x:c r="C180" s="415" t="n">
+        <x:f>B157</x:f>
+        <x:v>159.54215990000003</x:v>
+      </x:c>
+      <x:c r="D180" s="386" t="n">
+        <x:f>C180-B180</x:f>
+        <x:v>-14.70525699999996</x:v>
+      </x:c>
+      <x:c r="E180" s="321"/>
+      <x:c r="F180" s="321"/>
+      <x:c r="G180" s="321"/>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" s="366" t="str">
+        <x:v>FY31 UFCF (£m)</x:v>
+      </x:c>
+      <x:c r="B181" s="413" t="n">
+        <x:f>F61</x:f>
+        <x:v>210.3970536036348</x:v>
+      </x:c>
+      <x:c r="C181" s="415" t="n">
+        <x:f>F157</x:f>
+        <x:v>212.76093888766079</x:v>
+      </x:c>
+      <x:c r="D181" s="386" t="n">
+        <x:f>C181-B181</x:f>
+        <x:v>2.363885284025997</x:v>
+      </x:c>
+      <x:c r="E181" s="321"/>
+      <x:c r="F181" s="321"/>
+      <x:c r="G181" s="321"/>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="366" t="str">
+        <x:v>PV of explicit UFCF (£m)</x:v>
+      </x:c>
+      <x:c r="B182" s="413" t="n">
+        <x:f>B100</x:f>
+        <x:v>787.8105343730214</x:v>
+      </x:c>
+      <x:c r="C182" s="415" t="n">
+        <x:f>B166</x:f>
+        <x:v>768.0879593823954</x:v>
+      </x:c>
+      <x:c r="D182" s="386" t="n">
+        <x:f>C182-B182</x:f>
+        <x:v>-19.722574990625958</x:v>
+      </x:c>
+      <x:c r="E182" s="321"/>
+      <x:c r="F182" s="321"/>
+      <x:c r="G182" s="321"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="366" t="str">
+        <x:v>PV of terminal value (£m)</x:v>
+      </x:c>
+      <x:c r="B183" s="413" t="n">
+        <x:f>B102</x:f>
+        <x:v>2247.5217725557504</x:v>
+      </x:c>
+      <x:c r="C183" s="415" t="n">
+        <x:f>B168</x:f>
+        <x:v>2272.773474291467</x:v>
+      </x:c>
+      <x:c r="D183" s="386" t="n">
+        <x:f>C183-B183</x:f>
+        <x:v>25.25170173571678</x:v>
+      </x:c>
+      <x:c r="E183" s="321"/>
+      <x:c r="F183" s="321"/>
+      <x:c r="G183" s="321"/>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" s="366" t="str">
+        <x:v>Enterprise value (£m)</x:v>
+      </x:c>
+      <x:c r="B184" s="413" t="n">
+        <x:f>B103</x:f>
+        <x:v>3035.3323069287717</x:v>
+      </x:c>
+      <x:c r="C184" s="415" t="n">
+        <x:f>B169</x:f>
+        <x:v>3040.861433673863</x:v>
+      </x:c>
+      <x:c r="D184" s="386" t="n">
+        <x:f>C184-B184</x:f>
+        <x:v>5.529126745091162</x:v>
+      </x:c>
+      <x:c r="E184" s="321"/>
+      <x:c r="F184" s="321"/>
+      <x:c r="G184" s="321"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" s="366" t="str">
+        <x:v>Equity value (£m)</x:v>
+      </x:c>
+      <x:c r="B185" s="413" t="n">
+        <x:f>B105</x:f>
+        <x:v>2876.232306928772</x:v>
+      </x:c>
+      <x:c r="C185" s="415" t="n">
+        <x:f>B171</x:f>
+        <x:v>2881.761433673863</x:v>
+      </x:c>
+      <x:c r="D185" s="386" t="n">
+        <x:f>C185-B185</x:f>
+        <x:v>5.529126745091162</x:v>
+      </x:c>
+      <x:c r="E185" s="321"/>
+      <x:c r="F185" s="321"/>
+      <x:c r="G185" s="321"/>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" s="370" t="str">
+        <x:v>Implied value per share (£)</x:v>
+      </x:c>
+      <x:c r="B186" s="414" t="n">
+        <x:f>B107</x:f>
+        <x:v>5.5089682185956175</x:v>
+      </x:c>
+      <x:c r="C186" s="416" t="n">
+        <x:f>B173</x:f>
+        <x:v>5.519558386657466</x:v>
+      </x:c>
+      <x:c r="D186" s="389" t="n">
+        <x:f>C186-B186</x:f>
+        <x:v>0.010590168061848537</x:v>
+      </x:c>
+      <x:c r="E186" s="321"/>
+      <x:c r="F186" s="321"/>
+      <x:c r="G186" s="321"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" s="321"/>
+      <x:c r="B187" s="321"/>
+      <x:c r="C187" s="321"/>
+      <x:c r="D187" s="321"/>
+      <x:c r="E187" s="321"/>
+      <x:c r="F187" s="321"/>
+      <x:c r="G187" s="321"/>
+    </x:row>
+    <x:row r="188" ht="34" customHeight="1">
+      <x:c r="A188" s="417" t="str">
+        <x:v>Conclusion: restructuring is approximately value-neutral in this case. Higher long-run cash flow is largely offset by upfront costs and near-term disruption, so the assumptions do not force a preferred strategic answer.</x:v>
+      </x:c>
+      <x:c r="B188" s="417"/>
+      <x:c r="C188" s="417"/>
+      <x:c r="D188" s="417"/>
+      <x:c r="E188" s="417"/>
+      <x:c r="F188" s="417"/>
+      <x:c r="G188" s="321"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -19905,8 +21556,15 @@
     <x:mergeCell ref="A93:F93"/>
     <x:mergeCell ref="A111:F111"/>
     <x:mergeCell ref="A119:F119"/>
+    <x:mergeCell ref="A122:F122"/>
+    <x:mergeCell ref="A130:F130"/>
+    <x:mergeCell ref="A132:G132"/>
+    <x:mergeCell ref="A146:F146"/>
+    <x:mergeCell ref="A159:F159"/>
+    <x:mergeCell ref="A178:D178"/>
+    <x:mergeCell ref="A188:F188"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R451118abf94f4c8e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fbaa9f14b6a47c7"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add US disposal-case valuation
</commit_message>
<xml_diff>
--- a/model/QinetiQ_Valuation_Model.xlsx
+++ b/model/QinetiQ_Valuation_Model.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rdc87691d38d4448a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Re5c7837cf80348b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="Ra89a542787154db7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="Rea7517387a7a4a92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R66d0ca86384145c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="R6f7e9b285aed4bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R7962d4b259f148c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Reabf71765248468e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="R794de2ba3ec94caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R72ed22169d0b4b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rfaafeabe54994597"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="R629b11454a6142df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -876,7 +876,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="20">
+  <x:numFmts count="21">
     <x:numFmt numFmtId="164" formatCode="General"/>
     <x:numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <x:numFmt numFmtId="166" formatCode="#,##0.0;\(#,##0.0\);\-"/>
@@ -897,6 +897,7 @@
     <x:numFmt numFmtId="207" formatCode="#,##0.0;[Red](#,##0.0);-"/>
     <x:numFmt numFmtId="208" formatCode="0.000"/>
     <x:numFmt numFmtId="209" formatCode="0.00;[Red](0.00);-"/>
+    <x:numFmt numFmtId="210" formatCode="0.000x"/>
   </x:numFmts>
   <x:fonts count="32">
     <x:font>
@@ -1078,7 +1079,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="36">
+  <x:fills count="46">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1173,6 +1174,56 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -1453,7 +1504,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="418">
+  <x:cellXfs count="522">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2706,6 +2757,318 @@
       <x:alignment horizontal="general" vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="164" fontId="12" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="10" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="39" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="40" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="37" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="10" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="39" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="40" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="42" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="42" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="43" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="0" fillId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="10" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="44" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="43" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="45" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3234,7 +3597,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="1" t="str">
-        <x:v>0.6</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
@@ -3298,7 +3661,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D12" s="1" t="str">
-        <x:v>Restructuring-case DCF complete</x:v>
+        <x:v>US disposal-case DCF complete</x:v>
       </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
@@ -16158,12 +16521,24 @@
     <x:row r="23" ht="15" hidden="0">
       <x:c r="A23" s="1"/>
       <x:c r="B23" s="1"/>
-      <x:c r="C23" s="1"/>
-      <x:c r="D23" s="1"/>
-      <x:c r="E23" s="1"/>
-      <x:c r="F23" s="1"/>
-      <x:c r="G23" s="1"/>
-      <x:c r="H23" s="1"/>
+      <x:c r="C23" s="1" t="str">
+        <x:v>S017</x:v>
+      </x:c>
+      <x:c r="D23" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E23" s="1" t="str">
+        <x:v>2026-05-21</x:v>
+      </x:c>
+      <x:c r="F23" s="1" t="str">
+        <x:v>QinetiQ Group plc</x:v>
+      </x:c>
+      <x:c r="G23" s="1" t="str">
+        <x:v>FY26 Group Performance</x:v>
+      </x:c>
+      <x:c r="H23" s="1" t="str">
+        <x:v>https://www.qinetiq.com/en/news/fy26-group-performance</x:v>
+      </x:c>
       <x:c r="I23" s="1"/>
       <x:c r="J23" s="1"/>
       <x:c r="K23" s="1"/>
@@ -16186,12 +16561,24 @@
     <x:row r="24" ht="15" hidden="0">
       <x:c r="A24" s="1"/>
       <x:c r="B24" s="1"/>
-      <x:c r="C24" s="1"/>
-      <x:c r="D24" s="1"/>
-      <x:c r="E24" s="1"/>
-      <x:c r="F24" s="1"/>
-      <x:c r="G24" s="1"/>
-      <x:c r="H24" s="1"/>
+      <x:c r="C24" s="1" t="str">
+        <x:v>S018</x:v>
+      </x:c>
+      <x:c r="D24" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E24" s="1" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="F24" s="1" t="str">
+        <x:v>QinetiQ Group plc</x:v>
+      </x:c>
+      <x:c r="G24" s="1" t="str">
+        <x:v>FY27 Q1 Trading Update</x:v>
+      </x:c>
+      <x:c r="H24" s="1" t="str">
+        <x:v>https://www.qinetiq.com/en/news/q1-trading-update</x:v>
+      </x:c>
       <x:c r="I24" s="1"/>
       <x:c r="J24" s="1"/>
       <x:c r="K24" s="1"/>
@@ -16214,12 +16601,24 @@
     <x:row r="25" ht="15" hidden="0">
       <x:c r="A25" s="1"/>
       <x:c r="B25" s="1"/>
-      <x:c r="C25" s="1"/>
-      <x:c r="D25" s="1"/>
-      <x:c r="E25" s="1"/>
-      <x:c r="F25" s="1"/>
-      <x:c r="G25" s="1"/>
-      <x:c r="H25" s="1"/>
+      <x:c r="C25" s="1" t="str">
+        <x:v>S019</x:v>
+      </x:c>
+      <x:c r="D25" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E25" s="1" t="str">
+        <x:v>2022-08-05</x:v>
+      </x:c>
+      <x:c r="F25" s="1" t="str">
+        <x:v>QinetiQ Group plc</x:v>
+      </x:c>
+      <x:c r="G25" s="1" t="str">
+        <x:v>Proposed Acquisition of Avantus Federal LLC</x:v>
+      </x:c>
+      <x:c r="H25" s="1" t="str">
+        <x:v>https://www.qinetiq.com/en/news/proposed-acquisition-of-avantus-federal-llc</x:v>
+      </x:c>
       <x:c r="I25" s="1"/>
       <x:c r="J25" s="1"/>
       <x:c r="K25" s="1"/>
@@ -21517,6 +21916,1634 @@
       <x:c r="E188" s="417"/>
       <x:c r="F188" s="417"/>
       <x:c r="G188" s="321"/>
+    </x:row>
+    <x:row r="191" ht="22" customHeight="1">
+      <x:c r="A191" s="496" t="str">
+        <x:v>US disposal-case transaction assumptions</x:v>
+      </x:c>
+      <x:c r="B191" s="496"/>
+      <x:c r="C191" s="496"/>
+      <x:c r="D191" s="496"/>
+      <x:c r="E191" s="496"/>
+      <x:c r="F191" s="496"/>
+      <x:c r="G191" s="321"/>
+    </x:row>
+    <x:row r="192" ht="20" customHeight="1">
+      <x:c r="A192" s="497" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="B192" s="498" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C192" s="321"/>
+      <x:c r="D192" s="321"/>
+      <x:c r="E192" s="321"/>
+      <x:c r="F192" s="321"/>
+      <x:c r="G192" s="321"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" s="366" t="str">
+        <x:v>US revenue sold (£m)</x:v>
+      </x:c>
+      <x:c r="B193" s="469" t="n">
+        <x:v>290.7</x:v>
+      </x:c>
+      <x:c r="C193" s="321"/>
+      <x:c r="D193" s="321"/>
+      <x:c r="E193" s="321"/>
+      <x:c r="F193" s="321"/>
+      <x:c r="G193" s="321"/>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" s="366" t="str">
+        <x:v>Assumed FY26 US operating margin</x:v>
+      </x:c>
+      <x:c r="B194" s="367" t="n">
+        <x:v>0.075</x:v>
+      </x:c>
+      <x:c r="C194" s="321"/>
+      <x:c r="D194" s="321"/>
+      <x:c r="E194" s="321"/>
+      <x:c r="F194" s="321"/>
+      <x:c r="G194" s="321"/>
+    </x:row>
+    <x:row r="195">
+      <x:c r="A195" s="366" t="str">
+        <x:v>Implied US operating profit (£m)</x:v>
+      </x:c>
+      <x:c r="B195" s="470" t="n">
+        <x:f>B193*B194</x:f>
+        <x:v>21.8025</x:v>
+      </x:c>
+      <x:c r="C195" s="321"/>
+      <x:c r="D195" s="321"/>
+      <x:c r="E195" s="321"/>
+      <x:c r="F195" s="321"/>
+      <x:c r="G195" s="321"/>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" s="366" t="str">
+        <x:v>Other Products revenue retained (£m)</x:v>
+      </x:c>
+      <x:c r="B196" s="470" t="n">
+        <x:f>B16-B193</x:f>
+        <x:v>102.69999999999999</x:v>
+      </x:c>
+      <x:c r="C196" s="321"/>
+      <x:c r="D196" s="321"/>
+      <x:c r="E196" s="321"/>
+      <x:c r="F196" s="321"/>
+      <x:c r="G196" s="321"/>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="366" t="str">
+        <x:v>Implied Other Products operating profit (£m)</x:v>
+      </x:c>
+      <x:c r="B197" s="471" t="n">
+        <x:f>Segments!H17-B195</x:f>
+        <x:v>13.797500000000003</x:v>
+      </x:c>
+      <x:c r="C197" s="321"/>
+      <x:c r="D197" s="321"/>
+      <x:c r="E197" s="321"/>
+      <x:c r="F197" s="321"/>
+      <x:c r="G197" s="321"/>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" s="366" t="str">
+        <x:v>Implied Other Products operating margin</x:v>
+      </x:c>
+      <x:c r="B198" s="472" t="n">
+        <x:f>B197/B196</x:f>
+        <x:v>0.1343476144109056</x:v>
+      </x:c>
+      <x:c r="C198" s="321"/>
+      <x:c r="D198" s="321"/>
+      <x:c r="E198" s="321"/>
+      <x:c r="F198" s="321"/>
+      <x:c r="G198" s="321"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="366" t="str">
+        <x:v>Sale EV / revenue</x:v>
+      </x:c>
+      <x:c r="B199" s="473" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C199" s="321"/>
+      <x:c r="D199" s="321"/>
+      <x:c r="E199" s="321"/>
+      <x:c r="F199" s="321"/>
+      <x:c r="G199" s="321"/>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" s="366" t="str">
+        <x:v>Gross sale proceeds (£m)</x:v>
+      </x:c>
+      <x:c r="B200" s="470" t="n">
+        <x:f>B193*B199</x:f>
+        <x:v>290.7</x:v>
+      </x:c>
+      <x:c r="C200" s="321"/>
+      <x:c r="D200" s="321"/>
+      <x:c r="E200" s="321"/>
+      <x:c r="F200" s="321"/>
+      <x:c r="G200" s="321"/>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" s="366" t="str">
+        <x:v>Proceeds leakage</x:v>
+      </x:c>
+      <x:c r="B201" s="367" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C201" s="321"/>
+      <x:c r="D201" s="321"/>
+      <x:c r="E201" s="321"/>
+      <x:c r="F201" s="321"/>
+      <x:c r="G201" s="321"/>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="366" t="str">
+        <x:v>Net sale proceeds (£m)</x:v>
+      </x:c>
+      <x:c r="B202" s="470" t="n">
+        <x:f>B200*(1-B201)</x:f>
+        <x:v>261.63</x:v>
+      </x:c>
+      <x:c r="C202" s="321"/>
+      <x:c r="D202" s="321"/>
+      <x:c r="E202" s="321"/>
+      <x:c r="F202" s="321"/>
+      <x:c r="G202" s="321"/>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="366" t="str">
+        <x:v>Break-even sale EV / revenue</x:v>
+      </x:c>
+      <x:c r="B203" s="474" t="n">
+        <x:f>($B$105-$B$249+$B$104)/($B$193*(1-$B$201))</x:f>
+        <x:v>1.1322097486901377</x:v>
+      </x:c>
+      <x:c r="C203" s="321"/>
+      <x:c r="D203" s="321"/>
+      <x:c r="E203" s="321"/>
+      <x:c r="F203" s="321"/>
+      <x:c r="G203" s="321"/>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" s="370" t="str">
+        <x:v>Transaction timing</x:v>
+      </x:c>
+      <x:c r="B204" s="475" t="str">
+        <x:v>Immediate at valuation date</x:v>
+      </x:c>
+      <x:c r="C204" s="321"/>
+      <x:c r="D204" s="321"/>
+      <x:c r="E204" s="321"/>
+      <x:c r="F204" s="321"/>
+      <x:c r="G204" s="321"/>
+    </x:row>
+    <x:row r="205" ht="34" customHeight="1">
+      <x:c r="A205" s="521" t="str">
+        <x:v>The case sells only the £290.7m US operation and retains Other Products. The 10% proceeds allowance covers fees, separation, tax and working-capital adjustments.</x:v>
+      </x:c>
+      <x:c r="B205" s="521"/>
+      <x:c r="C205" s="521"/>
+      <x:c r="D205" s="521"/>
+      <x:c r="E205" s="521"/>
+      <x:c r="F205" s="521"/>
+      <x:c r="G205" s="321"/>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" s="321"/>
+      <x:c r="B206" s="321"/>
+      <x:c r="C206" s="321"/>
+      <x:c r="D206" s="321"/>
+      <x:c r="E206" s="321"/>
+      <x:c r="F206" s="321"/>
+      <x:c r="G206" s="321"/>
+    </x:row>
+    <x:row r="207" ht="22" customHeight="1">
+      <x:c r="A207" s="496" t="str">
+        <x:v>Retained-business forecast assumptions</x:v>
+      </x:c>
+      <x:c r="B207" s="496"/>
+      <x:c r="C207" s="496"/>
+      <x:c r="D207" s="496"/>
+      <x:c r="E207" s="496"/>
+      <x:c r="F207" s="496"/>
+      <x:c r="G207" s="321"/>
+    </x:row>
+    <x:row r="208" ht="20" customHeight="1">
+      <x:c r="A208" s="497" t="str">
+        <x:v>Assumption</x:v>
+      </x:c>
+      <x:c r="B208" s="498" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="C208" s="498" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="D208" s="498" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="E208" s="498" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="F208" s="498" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+      <x:c r="G208" s="321"/>
+    </x:row>
+    <x:row r="209">
+      <x:c r="A209" s="321" t="str">
+        <x:v>Other Products revenue growth</x:v>
+      </x:c>
+      <x:c r="B209" s="477" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C209" s="477" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="D209" s="477" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="E209" s="477" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="F209" s="477" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="G209" s="321"/>
+    </x:row>
+    <x:row r="210">
+      <x:c r="A210" s="321" t="str">
+        <x:v>Other Products operating margin</x:v>
+      </x:c>
+      <x:c r="B210" s="477" t="n">
+        <x:v>0.135</x:v>
+      </x:c>
+      <x:c r="C210" s="477" t="n">
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="D210" s="477" t="n">
+        <x:v>0.145</x:v>
+      </x:c>
+      <x:c r="E210" s="477" t="n">
+        <x:v>0.145</x:v>
+      </x:c>
+      <x:c r="F210" s="477" t="n">
+        <x:v>0.145</x:v>
+      </x:c>
+      <x:c r="G210" s="321"/>
+    </x:row>
+    <x:row r="211">
+      <x:c r="A211" s="321" t="str">
+        <x:v>Stranded overhead cost (£m)</x:v>
+      </x:c>
+      <x:c r="B211" s="478" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C211" s="478" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D211" s="478" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E211" s="478" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F211" s="478" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G211" s="321"/>
+    </x:row>
+    <x:row r="212" ht="34" customHeight="1">
+      <x:c r="A212" s="521" t="str">
+        <x:v>EMEA assumptions are unchanged. Other Products growth tapers from 5% to 3%; stranded overhead is removed over three years rather than assumed to disappear immediately.</x:v>
+      </x:c>
+      <x:c r="B212" s="521"/>
+      <x:c r="C212" s="521"/>
+      <x:c r="D212" s="521"/>
+      <x:c r="E212" s="521"/>
+      <x:c r="F212" s="521"/>
+      <x:c r="G212" s="321"/>
+    </x:row>
+    <x:row r="213">
+      <x:c r="A213" s="321"/>
+      <x:c r="B213" s="321"/>
+      <x:c r="C213" s="321"/>
+      <x:c r="D213" s="321"/>
+      <x:c r="E213" s="321"/>
+      <x:c r="F213" s="321"/>
+      <x:c r="G213" s="321"/>
+    </x:row>
+    <x:row r="214" ht="22" customHeight="1">
+      <x:c r="A214" s="496" t="str">
+        <x:v>US disposal-case retained-business forecast</x:v>
+      </x:c>
+      <x:c r="B214" s="496"/>
+      <x:c r="C214" s="496"/>
+      <x:c r="D214" s="496"/>
+      <x:c r="E214" s="496"/>
+      <x:c r="F214" s="496"/>
+      <x:c r="G214" s="496"/>
+    </x:row>
+    <x:row r="215" ht="20" customHeight="1">
+      <x:c r="A215" s="497" t="str">
+        <x:v>£m except percentages</x:v>
+      </x:c>
+      <x:c r="B215" s="498" t="str">
+        <x:v>FY26A</x:v>
+      </x:c>
+      <x:c r="C215" s="498" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="D215" s="498" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="E215" s="498" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="F215" s="498" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="G215" s="498" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216">
+      <x:c r="A216" s="321" t="str">
+        <x:v>EMEA Services revenue</x:v>
+      </x:c>
+      <x:c r="B216" s="377" t="n">
+        <x:f>B15</x:f>
+        <x:v>1529.2</x:v>
+      </x:c>
+      <x:c r="C216" s="377" t="n">
+        <x:f>C15</x:f>
+        <x:v>1605.66</x:v>
+      </x:c>
+      <x:c r="D216" s="377" t="n">
+        <x:f>D15</x:f>
+        <x:v>1685.9430000000002</x:v>
+      </x:c>
+      <x:c r="E216" s="377" t="n">
+        <x:f>E15</x:f>
+        <x:v>1761.810435</x:v>
+      </x:c>
+      <x:c r="F216" s="377" t="n">
+        <x:f>F15</x:f>
+        <x:v>1832.2828524000001</x:v>
+      </x:c>
+      <x:c r="G216" s="377" t="n">
+        <x:f>G15</x:f>
+        <x:v>1896.412752234</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217">
+      <x:c r="A217" s="321" t="str">
+        <x:v>Other Products revenue</x:v>
+      </x:c>
+      <x:c r="B217" s="377" t="n">
+        <x:f>$B$196</x:f>
+        <x:v>102.69999999999999</x:v>
+      </x:c>
+      <x:c r="C217" s="377" t="n">
+        <x:f>B217*(1+B209)</x:f>
+        <x:v>107.835</x:v>
+      </x:c>
+      <x:c r="D217" s="377" t="n">
+        <x:f>C217*(1+C209)</x:f>
+        <x:v>113.22675</x:v>
+      </x:c>
+      <x:c r="E217" s="377" t="n">
+        <x:f>D217*(1+D209)</x:f>
+        <x:v>117.75582</x:v>
+      </x:c>
+      <x:c r="F217" s="377" t="n">
+        <x:f>E217*(1+E209)</x:f>
+        <x:v>122.4660528</x:v>
+      </x:c>
+      <x:c r="G217" s="377" t="n">
+        <x:f>F217*(1+F209)</x:f>
+        <x:v>126.140034384</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218">
+      <x:c r="A218" s="321" t="str">
+        <x:v>Retained-business revenue</x:v>
+      </x:c>
+      <x:c r="B218" s="377" t="n">
+        <x:f>B216+B217</x:f>
+        <x:v>1631.9</x:v>
+      </x:c>
+      <x:c r="C218" s="377" t="n">
+        <x:f>C216+C217</x:f>
+        <x:v>1713.4950000000001</x:v>
+      </x:c>
+      <x:c r="D218" s="377" t="n">
+        <x:f>D216+D217</x:f>
+        <x:v>1799.1697500000002</x:v>
+      </x:c>
+      <x:c r="E218" s="377" t="n">
+        <x:f>E216+E217</x:f>
+        <x:v>1879.5662550000002</x:v>
+      </x:c>
+      <x:c r="F218" s="377" t="n">
+        <x:f>F216+F217</x:f>
+        <x:v>1954.7489052</x:v>
+      </x:c>
+      <x:c r="G218" s="377" t="n">
+        <x:f>G216+G217</x:f>
+        <x:v>2022.552786618</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219">
+      <x:c r="A219" s="321" t="str">
+        <x:v>Retained-business revenue growth</x:v>
+      </x:c>
+      <x:c r="B219" s="321"/>
+      <x:c r="C219" s="378" t="n">
+        <x:f>C218/B218-1</x:f>
+        <x:v>0.050000000000000044</x:v>
+      </x:c>
+      <x:c r="D219" s="378" t="n">
+        <x:f>D218/C218-1</x:f>
+        <x:v>0.050000000000000044</x:v>
+      </x:c>
+      <x:c r="E219" s="378" t="n">
+        <x:f>E218/D218-1</x:f>
+        <x:v>0.04468533611128134</x:v>
+      </x:c>
+      <x:c r="F219" s="378" t="n">
+        <x:f>F218/E218-1</x:f>
+        <x:v>0.040000000000000036</x:v>
+      </x:c>
+      <x:c r="G219" s="378" t="n">
+        <x:f>G218/F218-1</x:f>
+        <x:v>0.034686747355442415</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220">
+      <x:c r="A220" s="321" t="str"/>
+      <x:c r="B220" s="321"/>
+      <x:c r="C220" s="321"/>
+      <x:c r="D220" s="321"/>
+      <x:c r="E220" s="321"/>
+      <x:c r="F220" s="321"/>
+      <x:c r="G220" s="321"/>
+    </x:row>
+    <x:row r="221">
+      <x:c r="A221" s="321" t="str">
+        <x:v>EMEA Services operating profit</x:v>
+      </x:c>
+      <x:c r="B221" s="376" t="n">
+        <x:f>Segments!H16</x:f>
+        <x:v>182.3</x:v>
+      </x:c>
+      <x:c r="C221" s="377" t="n">
+        <x:f>C20</x:f>
+        <x:v>191.07354</x:v>
+      </x:c>
+      <x:c r="D221" s="377" t="n">
+        <x:f>D20</x:f>
+        <x:v>202.31316</x:v>
+      </x:c>
+      <x:c r="E221" s="377" t="n">
+        <x:f>E20</x:f>
+        <x:v>213.179062635</x:v>
+      </x:c>
+      <x:c r="F221" s="377" t="n">
+        <x:f>F20</x:f>
+        <x:v>221.70622514040002</x:v>
+      </x:c>
+      <x:c r="G221" s="377" t="n">
+        <x:f>G20</x:f>
+        <x:v>227.56953026808</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222">
+      <x:c r="A222" s="321" t="str">
+        <x:v>Other Products operating profit</x:v>
+      </x:c>
+      <x:c r="B222" s="377" t="n">
+        <x:f>$B$197</x:f>
+        <x:v>13.797500000000003</x:v>
+      </x:c>
+      <x:c r="C222" s="377" t="n">
+        <x:f>C217*B210</x:f>
+        <x:v>14.557725</x:v>
+      </x:c>
+      <x:c r="D222" s="377" t="n">
+        <x:f>D217*C210</x:f>
+        <x:v>15.851745000000001</x:v>
+      </x:c>
+      <x:c r="E222" s="377" t="n">
+        <x:f>E217*D210</x:f>
+        <x:v>17.0745939</x:v>
+      </x:c>
+      <x:c r="F222" s="377" t="n">
+        <x:f>F217*E210</x:f>
+        <x:v>17.757577656</x:v>
+      </x:c>
+      <x:c r="G222" s="377" t="n">
+        <x:f>G217*F210</x:f>
+        <x:v>18.29030498568</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223">
+      <x:c r="A223" s="321" t="str">
+        <x:v>Less: stranded overhead</x:v>
+      </x:c>
+      <x:c r="B223" s="377" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C223" s="377" t="n">
+        <x:f>-B211</x:f>
+        <x:v>-6</x:v>
+      </x:c>
+      <x:c r="D223" s="377" t="n">
+        <x:f>-C211</x:f>
+        <x:v>-4</x:v>
+      </x:c>
+      <x:c r="E223" s="377" t="n">
+        <x:f>-D211</x:f>
+        <x:v>-2</x:v>
+      </x:c>
+      <x:c r="F223" s="377" t="n">
+        <x:f>-E211</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G223" s="377" t="n">
+        <x:f>-F211</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224">
+      <x:c r="A224" s="321" t="str">
+        <x:v>Retained-business EBIT</x:v>
+      </x:c>
+      <x:c r="B224" s="377" t="n">
+        <x:f>SUM(B221:B223)</x:f>
+        <x:v>196.09750000000003</x:v>
+      </x:c>
+      <x:c r="C224" s="377" t="n">
+        <x:f>SUM(C221:C223)</x:f>
+        <x:v>199.631265</x:v>
+      </x:c>
+      <x:c r="D224" s="377" t="n">
+        <x:f>SUM(D221:D223)</x:f>
+        <x:v>214.164905</x:v>
+      </x:c>
+      <x:c r="E224" s="377" t="n">
+        <x:f>SUM(E221:E223)</x:f>
+        <x:v>228.253656535</x:v>
+      </x:c>
+      <x:c r="F224" s="377" t="n">
+        <x:f>SUM(F221:F223)</x:f>
+        <x:v>239.46380279640002</x:v>
+      </x:c>
+      <x:c r="G224" s="377" t="n">
+        <x:f>SUM(G221:G223)</x:f>
+        <x:v>245.85983525376</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" s="321" t="str">
+        <x:v>Retained-business operating margin</x:v>
+      </x:c>
+      <x:c r="B225" s="378" t="n">
+        <x:f>B224/B218</x:f>
+        <x:v>0.12016514492309578</x:v>
+      </x:c>
+      <x:c r="C225" s="378" t="n">
+        <x:f>C224/C218</x:f>
+        <x:v>0.11650530932392567</x:v>
+      </x:c>
+      <x:c r="D225" s="378" t="n">
+        <x:f>D224/D218</x:f>
+        <x:v>0.11903540785965303</x:v>
+      </x:c>
+      <x:c r="E225" s="378" t="n">
+        <x:f>E224/E218</x:f>
+        <x:v>0.12143953740806013</x:v>
+      </x:c>
+      <x:c r="F225" s="378" t="n">
+        <x:f>F224/F218</x:f>
+        <x:v>0.12250361269387655</x:v>
+      </x:c>
+      <x:c r="G225" s="378" t="n">
+        <x:f>G224/G218</x:f>
+        <x:v>0.12155916863108088</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226">
+      <x:c r="A226" s="321"/>
+      <x:c r="B226" s="321"/>
+      <x:c r="C226" s="321"/>
+      <x:c r="D226" s="321"/>
+      <x:c r="E226" s="321"/>
+      <x:c r="F226" s="321"/>
+      <x:c r="G226" s="321"/>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" s="321"/>
+      <x:c r="B227" s="321"/>
+      <x:c r="C227" s="321"/>
+      <x:c r="D227" s="321"/>
+      <x:c r="E227" s="321"/>
+      <x:c r="F227" s="321"/>
+      <x:c r="G227" s="321"/>
+    </x:row>
+    <x:row r="228" ht="22" customHeight="1">
+      <x:c r="A228" s="496" t="str">
+        <x:v>US disposal-case unlevered free cash flow</x:v>
+      </x:c>
+      <x:c r="B228" s="496"/>
+      <x:c r="C228" s="496"/>
+      <x:c r="D228" s="496"/>
+      <x:c r="E228" s="496"/>
+      <x:c r="F228" s="496"/>
+      <x:c r="G228" s="321"/>
+    </x:row>
+    <x:row r="229" ht="20" customHeight="1">
+      <x:c r="A229" s="497" t="str">
+        <x:v>£m except percentages</x:v>
+      </x:c>
+      <x:c r="B229" s="498" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="C229" s="498" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="D229" s="498" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="E229" s="498" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="F229" s="498" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+      <x:c r="G229" s="321"/>
+    </x:row>
+    <x:row r="230">
+      <x:c r="A230" s="321" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="B230" s="377" t="n">
+        <x:f>C218</x:f>
+        <x:v>1713.4950000000001</x:v>
+      </x:c>
+      <x:c r="C230" s="377" t="n">
+        <x:f>D218</x:f>
+        <x:v>1799.1697500000002</x:v>
+      </x:c>
+      <x:c r="D230" s="377" t="n">
+        <x:f>E218</x:f>
+        <x:v>1879.5662550000002</x:v>
+      </x:c>
+      <x:c r="E230" s="377" t="n">
+        <x:f>F218</x:f>
+        <x:v>1954.7489052</x:v>
+      </x:c>
+      <x:c r="F230" s="377" t="n">
+        <x:f>G218</x:f>
+        <x:v>2022.552786618</x:v>
+      </x:c>
+      <x:c r="G230" s="321"/>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" s="321" t="str">
+        <x:v>EBIT</x:v>
+      </x:c>
+      <x:c r="B231" s="377" t="n">
+        <x:f>C224</x:f>
+        <x:v>199.631265</x:v>
+      </x:c>
+      <x:c r="C231" s="377" t="n">
+        <x:f>D224</x:f>
+        <x:v>214.164905</x:v>
+      </x:c>
+      <x:c r="D231" s="377" t="n">
+        <x:f>E224</x:f>
+        <x:v>228.253656535</x:v>
+      </x:c>
+      <x:c r="E231" s="377" t="n">
+        <x:f>F224</x:f>
+        <x:v>239.46380279640002</x:v>
+      </x:c>
+      <x:c r="F231" s="377" t="n">
+        <x:f>G224</x:f>
+        <x:v>245.85983525376</x:v>
+      </x:c>
+      <x:c r="G231" s="321"/>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" s="321" t="str">
+        <x:v>Cash tax rate</x:v>
+      </x:c>
+      <x:c r="B232" s="378" t="n">
+        <x:f>B45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="C232" s="378" t="n">
+        <x:f>C45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="D232" s="378" t="n">
+        <x:f>D45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="E232" s="378" t="n">
+        <x:f>E45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="F232" s="378" t="n">
+        <x:f>F45</x:f>
+        <x:v>0.265</x:v>
+      </x:c>
+      <x:c r="G232" s="321"/>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" s="321" t="str">
+        <x:v>NOPAT</x:v>
+      </x:c>
+      <x:c r="B233" s="377" t="n">
+        <x:f>B231*(1-B232)</x:f>
+        <x:v>146.728979775</x:v>
+      </x:c>
+      <x:c r="C233" s="377" t="n">
+        <x:f>C231*(1-C232)</x:f>
+        <x:v>157.411205175</x:v>
+      </x:c>
+      <x:c r="D233" s="377" t="n">
+        <x:f>D231*(1-D232)</x:f>
+        <x:v>167.766437553225</x:v>
+      </x:c>
+      <x:c r="E233" s="377" t="n">
+        <x:f>E231*(1-E232)</x:f>
+        <x:v>176.00589505535402</x:v>
+      </x:c>
+      <x:c r="F233" s="377" t="n">
+        <x:f>F231*(1-F232)</x:f>
+        <x:v>180.7069789115136</x:v>
+      </x:c>
+      <x:c r="G233" s="321"/>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" s="321" t="str">
+        <x:v>D&amp;A</x:v>
+      </x:c>
+      <x:c r="B234" s="377" t="n">
+        <x:f>B230*B46</x:f>
+        <x:v>85.67475000000002</x:v>
+      </x:c>
+      <x:c r="C234" s="377" t="n">
+        <x:f>C230*C46</x:f>
+        <x:v>89.95848750000002</x:v>
+      </x:c>
+      <x:c r="D234" s="377" t="n">
+        <x:f>D230*D46</x:f>
+        <x:v>93.97831275000001</x:v>
+      </x:c>
+      <x:c r="E234" s="377" t="n">
+        <x:f>E230*E46</x:f>
+        <x:v>97.73744526000002</x:v>
+      </x:c>
+      <x:c r="F234" s="377" t="n">
+        <x:f>F230*F46</x:f>
+        <x:v>101.12763933090001</x:v>
+      </x:c>
+      <x:c r="G234" s="321"/>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" s="321" t="str">
+        <x:v>CapEx</x:v>
+      </x:c>
+      <x:c r="B235" s="377" t="n">
+        <x:f>-B230*B47</x:f>
+        <x:v>-77.107275</x:v>
+      </x:c>
+      <x:c r="C235" s="377" t="n">
+        <x:f>-C230*C47</x:f>
+        <x:v>-80.96263875000001</x:v>
+      </x:c>
+      <x:c r="D235" s="377" t="n">
+        <x:f>-D230*D47</x:f>
+        <x:v>-84.580481475</x:v>
+      </x:c>
+      <x:c r="E235" s="377" t="n">
+        <x:f>-E230*E47</x:f>
+        <x:v>-87.963700734</x:v>
+      </x:c>
+      <x:c r="F235" s="377" t="n">
+        <x:f>-F230*F47</x:f>
+        <x:v>-91.01487539781</x:v>
+      </x:c>
+      <x:c r="G235" s="321"/>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" s="321" t="str">
+        <x:v>Change in NWC</x:v>
+      </x:c>
+      <x:c r="B236" s="377" t="n">
+        <x:f>-(B230-$B$218)*B48</x:f>
+        <x:v>-0.8159500000000003</x:v>
+      </x:c>
+      <x:c r="C236" s="377" t="n">
+        <x:f>-(C230-B230)*C48</x:f>
+        <x:v>-0.8567475000000013</x:v>
+      </x:c>
+      <x:c r="D236" s="377" t="n">
+        <x:f>-(D230-C230)*D48</x:f>
+        <x:v>-0.8039650499999994</x:v>
+      </x:c>
+      <x:c r="E236" s="377" t="n">
+        <x:f>-(E230-D230)*E48</x:f>
+        <x:v>-0.751826501999999</x:v>
+      </x:c>
+      <x:c r="F236" s="377" t="n">
+        <x:f>-(F230-E230)*F48</x:f>
+        <x:v>-0.6780388141799994</x:v>
+      </x:c>
+      <x:c r="G236" s="321"/>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" s="500" t="str">
+        <x:v>UFCF</x:v>
+      </x:c>
+      <x:c r="B237" s="501" t="n">
+        <x:f>SUM(B233:B236)</x:f>
+        <x:v>154.48050477500004</x:v>
+      </x:c>
+      <x:c r="C237" s="501" t="n">
+        <x:f>SUM(C233:C236)</x:f>
+        <x:v>165.550306425</x:v>
+      </x:c>
+      <x:c r="D237" s="501" t="n">
+        <x:f>SUM(D233:D236)</x:f>
+        <x:v>176.36030377822505</x:v>
+      </x:c>
+      <x:c r="E237" s="501" t="n">
+        <x:f>SUM(E233:E236)</x:f>
+        <x:v>185.02781307935405</x:v>
+      </x:c>
+      <x:c r="F237" s="501" t="n">
+        <x:f>SUM(F233:F236)</x:f>
+        <x:v>190.14170403042363</x:v>
+      </x:c>
+      <x:c r="G237" s="321"/>
+    </x:row>
+    <x:row r="238">
+      <x:c r="A238" s="321"/>
+      <x:c r="B238" s="321"/>
+      <x:c r="C238" s="321"/>
+      <x:c r="D238" s="321"/>
+      <x:c r="E238" s="321"/>
+      <x:c r="F238" s="321"/>
+      <x:c r="G238" s="321"/>
+    </x:row>
+    <x:row r="239" ht="22" customHeight="1">
+      <x:c r="A239" s="496" t="str">
+        <x:v>US disposal-case DCF valuation</x:v>
+      </x:c>
+      <x:c r="B239" s="496"/>
+      <x:c r="C239" s="496"/>
+      <x:c r="D239" s="496"/>
+      <x:c r="E239" s="496"/>
+      <x:c r="F239" s="496"/>
+      <x:c r="G239" s="321"/>
+    </x:row>
+    <x:row r="240" ht="20" customHeight="1">
+      <x:c r="A240" s="497" t="str">
+        <x:v>£m except per-share data</x:v>
+      </x:c>
+      <x:c r="B240" s="498" t="str">
+        <x:v>FY27E</x:v>
+      </x:c>
+      <x:c r="C240" s="498" t="str">
+        <x:v>FY28E</x:v>
+      </x:c>
+      <x:c r="D240" s="498" t="str">
+        <x:v>FY29E</x:v>
+      </x:c>
+      <x:c r="E240" s="498" t="str">
+        <x:v>FY30E</x:v>
+      </x:c>
+      <x:c r="F240" s="498" t="str">
+        <x:v>FY31E</x:v>
+      </x:c>
+      <x:c r="G240" s="321"/>
+    </x:row>
+    <x:row r="241">
+      <x:c r="A241" s="321" t="str">
+        <x:v>UFCF</x:v>
+      </x:c>
+      <x:c r="B241" s="377" t="n">
+        <x:f>B237</x:f>
+        <x:v>154.48050477500004</x:v>
+      </x:c>
+      <x:c r="C241" s="377" t="n">
+        <x:f>C237</x:f>
+        <x:v>165.550306425</x:v>
+      </x:c>
+      <x:c r="D241" s="377" t="n">
+        <x:f>D237</x:f>
+        <x:v>176.36030377822505</x:v>
+      </x:c>
+      <x:c r="E241" s="377" t="n">
+        <x:f>E237</x:f>
+        <x:v>185.02781307935405</x:v>
+      </x:c>
+      <x:c r="F241" s="377" t="n">
+        <x:f>F237</x:f>
+        <x:v>190.14170403042363</x:v>
+      </x:c>
+      <x:c r="G241" s="321"/>
+    </x:row>
+    <x:row r="242">
+      <x:c r="A242" s="321" t="str">
+        <x:v>Discount period</x:v>
+      </x:c>
+      <x:c r="B242" s="381" t="n">
+        <x:f>B96</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C242" s="381" t="n">
+        <x:f>C96</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="D242" s="381" t="n">
+        <x:f>D96</x:f>
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="E242" s="381" t="n">
+        <x:f>E96</x:f>
+        <x:v>3.5</x:v>
+      </x:c>
+      <x:c r="F242" s="381" t="n">
+        <x:f>F96</x:f>
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="G242" s="321"/>
+    </x:row>
+    <x:row r="243">
+      <x:c r="A243" s="321" t="str">
+        <x:v>Discount factor</x:v>
+      </x:c>
+      <x:c r="B243" s="381" t="n">
+        <x:f>1/(1+$B$83)^B242</x:f>
+        <x:v>0.9596329968646349</x:v>
+      </x:c>
+      <x:c r="C243" s="381" t="n">
+        <x:f>1/(1+$B$83)^C242</x:f>
+        <x:v>0.883721697592858</x:v>
+      </x:c>
+      <x:c r="D243" s="381" t="n">
+        <x:f>1/(1+$B$83)^D242</x:f>
+        <x:v>0.8138153245542943</x:v>
+      </x:c>
+      <x:c r="E243" s="381" t="n">
+        <x:f>1/(1+$B$83)^E242</x:f>
+        <x:v>0.7494388609937009</x:v>
+      </x:c>
+      <x:c r="F243" s="381" t="n">
+        <x:f>1/(1+$B$83)^F242</x:f>
+        <x:v>0.6901548661241318</x:v>
+      </x:c>
+      <x:c r="G243" s="321"/>
+    </x:row>
+    <x:row r="244">
+      <x:c r="A244" s="321" t="str">
+        <x:v>Present value of UFCF</x:v>
+      </x:c>
+      <x:c r="B244" s="377" t="n">
+        <x:f>B241*B243</x:f>
+        <x:v>148.24458975439484</x:v>
+      </x:c>
+      <x:c r="C244" s="377" t="n">
+        <x:f>C241*C243</x:f>
+        <x:v>146.30039783091883</x:v>
+      </x:c>
+      <x:c r="D244" s="377" t="n">
+        <x:f>D241*D243</x:f>
+        <x:v>143.52471785777016</x:v>
+      </x:c>
+      <x:c r="E244" s="377" t="n">
+        <x:f>E241*E243</x:f>
+        <x:v>138.6670334863465</x:v>
+      </x:c>
+      <x:c r="F244" s="377" t="n">
+        <x:f>F241*F243</x:f>
+        <x:v>131.22722228973132</x:v>
+      </x:c>
+      <x:c r="G244" s="321"/>
+    </x:row>
+    <x:row r="245">
+      <x:c r="A245" s="321" t="str"/>
+      <x:c r="B245" s="321"/>
+      <x:c r="C245" s="321"/>
+      <x:c r="D245" s="321"/>
+      <x:c r="E245" s="321"/>
+      <x:c r="F245" s="321"/>
+      <x:c r="G245" s="321"/>
+    </x:row>
+    <x:row r="246">
+      <x:c r="A246" s="321" t="str">
+        <x:v>PV of explicit-period UFCF</x:v>
+      </x:c>
+      <x:c r="B246" s="377" t="n">
+        <x:f>SUM(B244:F244)</x:f>
+        <x:v>707.9639612191617</x:v>
+      </x:c>
+      <x:c r="C246" s="321"/>
+      <x:c r="D246" s="321"/>
+      <x:c r="E246" s="321"/>
+      <x:c r="F246" s="321"/>
+      <x:c r="G246" s="321"/>
+    </x:row>
+    <x:row r="247">
+      <x:c r="A247" s="321" t="str">
+        <x:v>Terminal value</x:v>
+      </x:c>
+      <x:c r="B247" s="377" t="n">
+        <x:f>F241*(1+$B$88)/($B$83-$B$88)</x:f>
+        <x:v>2943.032656665331</x:v>
+      </x:c>
+      <x:c r="C247" s="321"/>
+      <x:c r="D247" s="321"/>
+      <x:c r="E247" s="321"/>
+      <x:c r="F247" s="321"/>
+      <x:c r="G247" s="321"/>
+    </x:row>
+    <x:row r="248">
+      <x:c r="A248" s="321" t="str">
+        <x:v>PV of terminal value</x:v>
+      </x:c>
+      <x:c r="B248" s="377" t="n">
+        <x:f>B247*F243</x:f>
+        <x:v>2031.1483091598095</x:v>
+      </x:c>
+      <x:c r="C248" s="321"/>
+      <x:c r="D248" s="321"/>
+      <x:c r="E248" s="321"/>
+      <x:c r="F248" s="321"/>
+      <x:c r="G248" s="321"/>
+    </x:row>
+    <x:row r="249">
+      <x:c r="A249" s="500" t="str">
+        <x:v>Retained-business enterprise value</x:v>
+      </x:c>
+      <x:c r="B249" s="501" t="n">
+        <x:f>B246+B248</x:f>
+        <x:v>2739.112270378971</x:v>
+      </x:c>
+      <x:c r="C249" s="321"/>
+      <x:c r="D249" s="321"/>
+      <x:c r="E249" s="321"/>
+      <x:c r="F249" s="321"/>
+      <x:c r="G249" s="321"/>
+    </x:row>
+    <x:row r="250">
+      <x:c r="A250" s="321" t="str">
+        <x:v>Add: net sale proceeds</x:v>
+      </x:c>
+      <x:c r="B250" s="377" t="n">
+        <x:f>$B$202</x:f>
+        <x:v>261.63</x:v>
+      </x:c>
+      <x:c r="C250" s="321"/>
+      <x:c r="D250" s="321"/>
+      <x:c r="E250" s="321"/>
+      <x:c r="F250" s="321"/>
+      <x:c r="G250" s="321"/>
+    </x:row>
+    <x:row r="251">
+      <x:c r="A251" s="321" t="str">
+        <x:v>Value before net debt</x:v>
+      </x:c>
+      <x:c r="B251" s="377" t="n">
+        <x:f>B249+B250</x:f>
+        <x:v>3000.742270378971</x:v>
+      </x:c>
+      <x:c r="C251" s="321"/>
+      <x:c r="D251" s="321"/>
+      <x:c r="E251" s="321"/>
+      <x:c r="F251" s="321"/>
+      <x:c r="G251" s="321"/>
+    </x:row>
+    <x:row r="252">
+      <x:c r="A252" s="321" t="str">
+        <x:v>Less: group net debt</x:v>
+      </x:c>
+      <x:c r="B252" s="377" t="n">
+        <x:f>$B$104</x:f>
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="C252" s="321"/>
+      <x:c r="D252" s="321"/>
+      <x:c r="E252" s="321"/>
+      <x:c r="F252" s="321"/>
+      <x:c r="G252" s="321"/>
+    </x:row>
+    <x:row r="253">
+      <x:c r="A253" s="500" t="str">
+        <x:v>Equity value</x:v>
+      </x:c>
+      <x:c r="B253" s="501" t="n">
+        <x:f>B251-B252</x:f>
+        <x:v>2841.6422703789713</x:v>
+      </x:c>
+      <x:c r="C253" s="321"/>
+      <x:c r="D253" s="321"/>
+      <x:c r="E253" s="321"/>
+      <x:c r="F253" s="321"/>
+      <x:c r="G253" s="321"/>
+    </x:row>
+    <x:row r="254">
+      <x:c r="A254" s="321" t="str">
+        <x:v>Diluted shares (m)</x:v>
+      </x:c>
+      <x:c r="B254" s="377" t="n">
+        <x:f>$B$106</x:f>
+        <x:v>522.1</x:v>
+      </x:c>
+      <x:c r="C254" s="321"/>
+      <x:c r="D254" s="321"/>
+      <x:c r="E254" s="321"/>
+      <x:c r="F254" s="321"/>
+      <x:c r="G254" s="321"/>
+    </x:row>
+    <x:row r="255">
+      <x:c r="A255" s="500" t="str">
+        <x:v>Implied value per share (£)</x:v>
+      </x:c>
+      <x:c r="B255" s="502" t="n">
+        <x:f>B253/B254</x:f>
+        <x:v>5.442716472666101</x:v>
+      </x:c>
+      <x:c r="C255" s="321"/>
+      <x:c r="D255" s="321"/>
+      <x:c r="E255" s="321"/>
+      <x:c r="F255" s="321"/>
+      <x:c r="G255" s="321"/>
+    </x:row>
+    <x:row r="256">
+      <x:c r="A256" s="321" t="str">
+        <x:v>Difference vs base (£/share)</x:v>
+      </x:c>
+      <x:c r="B256" s="383" t="n">
+        <x:f>B255-$B$107</x:f>
+        <x:v>-0.06625174592951666</x:v>
+      </x:c>
+      <x:c r="C256" s="321"/>
+      <x:c r="D256" s="321"/>
+      <x:c r="E256" s="321"/>
+      <x:c r="F256" s="321"/>
+      <x:c r="G256" s="321"/>
+    </x:row>
+    <x:row r="257">
+      <x:c r="A257" s="321" t="str">
+        <x:v>Change vs base</x:v>
+      </x:c>
+      <x:c r="B257" s="378" t="n">
+        <x:f>B255/$B$107-1</x:f>
+        <x:v>-0.012026162304927257</x:v>
+      </x:c>
+      <x:c r="C257" s="321"/>
+      <x:c r="D257" s="321"/>
+      <x:c r="E257" s="321"/>
+      <x:c r="F257" s="321"/>
+      <x:c r="G257" s="321"/>
+    </x:row>
+    <x:row r="258">
+      <x:c r="A258" s="321" t="str">
+        <x:v>Terminal value / retained-business EV</x:v>
+      </x:c>
+      <x:c r="B258" s="378" t="n">
+        <x:f>B248/B249</x:f>
+        <x:v>0.7415352525432589</x:v>
+      </x:c>
+      <x:c r="C258" s="321"/>
+      <x:c r="D258" s="321"/>
+      <x:c r="E258" s="321"/>
+      <x:c r="F258" s="321"/>
+      <x:c r="G258" s="321"/>
+    </x:row>
+    <x:row r="259">
+      <x:c r="A259" s="321"/>
+      <x:c r="B259" s="321"/>
+      <x:c r="C259" s="321"/>
+      <x:c r="D259" s="321"/>
+      <x:c r="E259" s="321"/>
+      <x:c r="F259" s="321"/>
+      <x:c r="G259" s="321"/>
+    </x:row>
+    <x:row r="260" ht="22" customHeight="1">
+      <x:c r="A260" s="496" t="str">
+        <x:v>US sale-multiple sensitivity</x:v>
+      </x:c>
+      <x:c r="B260" s="496"/>
+      <x:c r="C260" s="496"/>
+      <x:c r="D260" s="496"/>
+      <x:c r="E260" s="496"/>
+      <x:c r="F260" s="321"/>
+      <x:c r="G260" s="321"/>
+    </x:row>
+    <x:row r="261" ht="20" customHeight="1">
+      <x:c r="A261" s="497" t="str">
+        <x:v>Sale multiple</x:v>
+      </x:c>
+      <x:c r="B261" s="498" t="str">
+        <x:v>Gross proceeds</x:v>
+      </x:c>
+      <x:c r="C261" s="498" t="str">
+        <x:v>Net proceeds</x:v>
+      </x:c>
+      <x:c r="D261" s="498" t="str">
+        <x:v>Value / share</x:v>
+      </x:c>
+      <x:c r="E261" s="498" t="str">
+        <x:v>Vs base</x:v>
+      </x:c>
+      <x:c r="F261" s="321"/>
+      <x:c r="G261" s="321"/>
+    </x:row>
+    <x:row r="262">
+      <x:c r="A262" s="482" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="B262" s="386" t="n">
+        <x:f>$B$193*A262</x:f>
+        <x:v>218.02499999999998</x:v>
+      </x:c>
+      <x:c r="C262" s="386" t="n">
+        <x:f>B262*(1-$B$201)</x:f>
+        <x:v>196.2225</x:v>
+      </x:c>
+      <x:c r="D262" s="483" t="n">
+        <x:f>($B$249+C262-$B$104)/$B$106</x:f>
+        <x:v>5.317438748092264</x:v>
+      </x:c>
+      <x:c r="E262" s="483" t="n">
+        <x:f>D262-$B$107</x:f>
+        <x:v>-0.19152947050335367</x:v>
+      </x:c>
+      <x:c r="F262" s="321"/>
+      <x:c r="G262" s="321"/>
+    </x:row>
+    <x:row r="263">
+      <x:c r="A263" s="482" t="n">
+        <x:v>0.875</x:v>
+      </x:c>
+      <x:c r="B263" s="386" t="n">
+        <x:f>$B$193*A263</x:f>
+        <x:v>254.36249999999998</x:v>
+      </x:c>
+      <x:c r="C263" s="386" t="n">
+        <x:f>B263*(1-$B$201)</x:f>
+        <x:v>228.92624999999998</x:v>
+      </x:c>
+      <x:c r="D263" s="483" t="n">
+        <x:f>($B$249+C263-$B$104)/$B$106</x:f>
+        <x:v>5.380077610379182</x:v>
+      </x:c>
+      <x:c r="E263" s="483" t="n">
+        <x:f>D263-$B$107</x:f>
+        <x:v>-0.1288906082164356</x:v>
+      </x:c>
+      <x:c r="F263" s="321"/>
+      <x:c r="G263" s="321"/>
+    </x:row>
+    <x:row r="264">
+      <x:c r="A264" s="505" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B264" s="506" t="n">
+        <x:f>$B$193*A264</x:f>
+        <x:v>290.7</x:v>
+      </x:c>
+      <x:c r="C264" s="506" t="n">
+        <x:f>B264*(1-$B$201)</x:f>
+        <x:v>261.63</x:v>
+      </x:c>
+      <x:c r="D264" s="507" t="n">
+        <x:f>($B$249+C264-$B$104)/$B$106</x:f>
+        <x:v>5.442716472666101</x:v>
+      </x:c>
+      <x:c r="E264" s="507" t="n">
+        <x:f>D264-$B$107</x:f>
+        <x:v>-0.06625174592951666</x:v>
+      </x:c>
+      <x:c r="F264" s="321"/>
+      <x:c r="G264" s="321"/>
+    </x:row>
+    <x:row r="265">
+      <x:c r="A265" s="482" t="n">
+        <x:v>1.125</x:v>
+      </x:c>
+      <x:c r="B265" s="386" t="n">
+        <x:f>$B$193*A265</x:f>
+        <x:v>327.03749999999997</x:v>
+      </x:c>
+      <x:c r="C265" s="386" t="n">
+        <x:f>B265*(1-$B$201)</x:f>
+        <x:v>294.33374999999995</x:v>
+      </x:c>
+      <x:c r="D265" s="483" t="n">
+        <x:f>($B$249+C265-$B$104)/$B$106</x:f>
+        <x:v>5.505355334953018</x:v>
+      </x:c>
+      <x:c r="E265" s="483" t="n">
+        <x:f>D265-$B$107</x:f>
+        <x:v>-0.003612883642599485</x:v>
+      </x:c>
+      <x:c r="F265" s="321"/>
+      <x:c r="G265" s="321"/>
+    </x:row>
+    <x:row r="266">
+      <x:c r="A266" s="487" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="B266" s="488" t="n">
+        <x:f>$B$193*A266</x:f>
+        <x:v>363.375</x:v>
+      </x:c>
+      <x:c r="C266" s="488" t="n">
+        <x:f>B266*(1-$B$201)</x:f>
+        <x:v>327.0375</x:v>
+      </x:c>
+      <x:c r="D266" s="389" t="n">
+        <x:f>($B$249+C266-$B$104)/$B$106</x:f>
+        <x:v>5.567994197239937</x:v>
+      </x:c>
+      <x:c r="E266" s="389" t="n">
+        <x:f>D266-$B$107</x:f>
+        <x:v>0.059025978644319466</x:v>
+      </x:c>
+      <x:c r="F266" s="321"/>
+      <x:c r="G266" s="321"/>
+    </x:row>
+    <x:row r="267">
+      <x:c r="A267" s="321"/>
+      <x:c r="B267" s="321"/>
+      <x:c r="C267" s="321"/>
+      <x:c r="D267" s="321"/>
+      <x:c r="E267" s="321"/>
+      <x:c r="F267" s="321"/>
+      <x:c r="G267" s="321"/>
+    </x:row>
+    <x:row r="268" ht="34" customHeight="1">
+      <x:c r="A268" s="521" t="str">
+        <x:v>Break-even: approximately 1.13x FY26 US revenue after the 10% proceeds allowance. Below this multiple, disposal is worth less than the base case.</x:v>
+      </x:c>
+      <x:c r="B268" s="521"/>
+      <x:c r="C268" s="521"/>
+      <x:c r="D268" s="521"/>
+      <x:c r="E268" s="521"/>
+      <x:c r="F268" s="521"/>
+      <x:c r="G268" s="321"/>
+    </x:row>
+    <x:row r="269">
+      <x:c r="A269" s="321"/>
+      <x:c r="B269" s="321"/>
+      <x:c r="C269" s="321"/>
+      <x:c r="D269" s="321"/>
+      <x:c r="E269" s="321"/>
+      <x:c r="F269" s="321"/>
+      <x:c r="G269" s="321"/>
+    </x:row>
+    <x:row r="270" ht="22" customHeight="1">
+      <x:c r="A270" s="496" t="str">
+        <x:v>Strategic alternatives comparison</x:v>
+      </x:c>
+      <x:c r="B270" s="496"/>
+      <x:c r="C270" s="496"/>
+      <x:c r="D270" s="496"/>
+      <x:c r="E270" s="321"/>
+      <x:c r="F270" s="321"/>
+      <x:c r="G270" s="321"/>
+    </x:row>
+    <x:row r="271" ht="20" customHeight="1">
+      <x:c r="A271" s="497" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B271" s="498" t="str">
+        <x:v>Base case</x:v>
+      </x:c>
+      <x:c r="C271" s="498" t="str">
+        <x:v>Restructuring</x:v>
+      </x:c>
+      <x:c r="D271" s="498" t="str">
+        <x:v>US disposal</x:v>
+      </x:c>
+      <x:c r="E271" s="321"/>
+      <x:c r="F271" s="321"/>
+      <x:c r="G271" s="321"/>
+    </x:row>
+    <x:row r="272">
+      <x:c r="A272" s="366" t="str">
+        <x:v>FY27 UFCF (£m)</x:v>
+      </x:c>
+      <x:c r="B272" s="514" t="n">
+        <x:f>B61</x:f>
+        <x:v>174.2474169</x:v>
+      </x:c>
+      <x:c r="C272" s="506" t="n">
+        <x:f>B157</x:f>
+        <x:v>159.54215990000003</x:v>
+      </x:c>
+      <x:c r="D272" s="518" t="n">
+        <x:f>B237</x:f>
+        <x:v>154.48050477500004</x:v>
+      </x:c>
+      <x:c r="E272" s="321"/>
+      <x:c r="F272" s="321"/>
+      <x:c r="G272" s="321"/>
+    </x:row>
+    <x:row r="273">
+      <x:c r="A273" s="366" t="str">
+        <x:v>FY31 UFCF (£m)</x:v>
+      </x:c>
+      <x:c r="B273" s="514" t="n">
+        <x:f>F61</x:f>
+        <x:v>210.3970536036348</x:v>
+      </x:c>
+      <x:c r="C273" s="506" t="n">
+        <x:f>F157</x:f>
+        <x:v>212.76093888766079</x:v>
+      </x:c>
+      <x:c r="D273" s="518" t="n">
+        <x:f>F237</x:f>
+        <x:v>190.14170403042363</x:v>
+      </x:c>
+      <x:c r="E273" s="321"/>
+      <x:c r="F273" s="321"/>
+      <x:c r="G273" s="321"/>
+    </x:row>
+    <x:row r="274">
+      <x:c r="A274" s="366" t="str">
+        <x:v>PV of explicit UFCF (£m)</x:v>
+      </x:c>
+      <x:c r="B274" s="514" t="n">
+        <x:f>B100</x:f>
+        <x:v>787.8105343730214</x:v>
+      </x:c>
+      <x:c r="C274" s="506" t="n">
+        <x:f>B166</x:f>
+        <x:v>768.0879593823954</x:v>
+      </x:c>
+      <x:c r="D274" s="518" t="n">
+        <x:f>B246</x:f>
+        <x:v>707.9639612191617</x:v>
+      </x:c>
+      <x:c r="E274" s="321"/>
+      <x:c r="F274" s="321"/>
+      <x:c r="G274" s="321"/>
+    </x:row>
+    <x:row r="275">
+      <x:c r="A275" s="366" t="str">
+        <x:v>PV of terminal value (£m)</x:v>
+      </x:c>
+      <x:c r="B275" s="514" t="n">
+        <x:f>B102</x:f>
+        <x:v>2247.5217725557504</x:v>
+      </x:c>
+      <x:c r="C275" s="506" t="n">
+        <x:f>B168</x:f>
+        <x:v>2272.773474291467</x:v>
+      </x:c>
+      <x:c r="D275" s="518" t="n">
+        <x:f>B248</x:f>
+        <x:v>2031.1483091598095</x:v>
+      </x:c>
+      <x:c r="E275" s="321"/>
+      <x:c r="F275" s="321"/>
+      <x:c r="G275" s="321"/>
+    </x:row>
+    <x:row r="276">
+      <x:c r="A276" s="366" t="str">
+        <x:v>Operating-business EV (£m)</x:v>
+      </x:c>
+      <x:c r="B276" s="514" t="n">
+        <x:f>B103</x:f>
+        <x:v>3035.3323069287717</x:v>
+      </x:c>
+      <x:c r="C276" s="506" t="n">
+        <x:f>B169</x:f>
+        <x:v>3040.861433673863</x:v>
+      </x:c>
+      <x:c r="D276" s="518" t="n">
+        <x:f>B249</x:f>
+        <x:v>2739.112270378971</x:v>
+      </x:c>
+      <x:c r="E276" s="321"/>
+      <x:c r="F276" s="321"/>
+      <x:c r="G276" s="321"/>
+    </x:row>
+    <x:row r="277">
+      <x:c r="A277" s="366" t="str">
+        <x:v>Net sale proceeds (£m)</x:v>
+      </x:c>
+      <x:c r="B277" s="514" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C277" s="506" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D277" s="518" t="n">
+        <x:f>B250</x:f>
+        <x:v>261.63</x:v>
+      </x:c>
+      <x:c r="E277" s="321"/>
+      <x:c r="F277" s="321"/>
+      <x:c r="G277" s="321"/>
+    </x:row>
+    <x:row r="278">
+      <x:c r="A278" s="366" t="str">
+        <x:v>Equity value (£m)</x:v>
+      </x:c>
+      <x:c r="B278" s="514" t="n">
+        <x:f>B105</x:f>
+        <x:v>2876.232306928772</x:v>
+      </x:c>
+      <x:c r="C278" s="506" t="n">
+        <x:f>B171</x:f>
+        <x:v>2881.761433673863</x:v>
+      </x:c>
+      <x:c r="D278" s="518" t="n">
+        <x:f>B253</x:f>
+        <x:v>2841.6422703789713</x:v>
+      </x:c>
+      <x:c r="E278" s="321"/>
+      <x:c r="F278" s="321"/>
+      <x:c r="G278" s="321"/>
+    </x:row>
+    <x:row r="279">
+      <x:c r="A279" s="366" t="str">
+        <x:v>Implied value per share (£)</x:v>
+      </x:c>
+      <x:c r="B279" s="515" t="n">
+        <x:f>B107</x:f>
+        <x:v>5.5089682185956175</x:v>
+      </x:c>
+      <x:c r="C279" s="507" t="n">
+        <x:f>B173</x:f>
+        <x:v>5.519558386657466</x:v>
+      </x:c>
+      <x:c r="D279" s="519" t="n">
+        <x:f>B255</x:f>
+        <x:v>5.442716472666101</x:v>
+      </x:c>
+      <x:c r="E279" s="321"/>
+      <x:c r="F279" s="321"/>
+      <x:c r="G279" s="321"/>
+    </x:row>
+    <x:row r="280">
+      <x:c r="A280" s="370" t="str">
+        <x:v>Change vs base</x:v>
+      </x:c>
+      <x:c r="B280" s="516" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C280" s="517" t="n">
+        <x:f>B175</x:f>
+        <x:v>0.0019223505458065837</x:v>
+      </x:c>
+      <x:c r="D280" s="520" t="n">
+        <x:f>B257</x:f>
+        <x:v>-0.012026162304927257</x:v>
+      </x:c>
+      <x:c r="E280" s="321"/>
+      <x:c r="F280" s="321"/>
+      <x:c r="G280" s="321"/>
+    </x:row>
+    <x:row r="281">
+      <x:c r="A281" s="321"/>
+      <x:c r="B281" s="321"/>
+      <x:c r="C281" s="321"/>
+      <x:c r="D281" s="321"/>
+      <x:c r="E281" s="321"/>
+      <x:c r="F281" s="321"/>
+      <x:c r="G281" s="321"/>
+    </x:row>
+    <x:row r="282" ht="34" customHeight="1">
+      <x:c r="A282" s="521" t="str">
+        <x:v>Conclusion: at a 1.00x revenue sale multiple, disposal is worth £5.44 per share, below both retain cases. Disposal breaks even with the base case at approximately 1.13x revenue.</x:v>
+      </x:c>
+      <x:c r="B282" s="521"/>
+      <x:c r="C282" s="521"/>
+      <x:c r="D282" s="521"/>
+      <x:c r="E282" s="521"/>
+      <x:c r="F282" s="521"/>
+      <x:c r="G282" s="321"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -21563,8 +23590,19 @@
     <x:mergeCell ref="A159:F159"/>
     <x:mergeCell ref="A178:D178"/>
     <x:mergeCell ref="A188:F188"/>
+    <x:mergeCell ref="A191:F191"/>
+    <x:mergeCell ref="A205:F205"/>
+    <x:mergeCell ref="A207:F207"/>
+    <x:mergeCell ref="A212:F212"/>
+    <x:mergeCell ref="A214:G214"/>
+    <x:mergeCell ref="A228:F228"/>
+    <x:mergeCell ref="A239:F239"/>
+    <x:mergeCell ref="A260:E260"/>
+    <x:mergeCell ref="A268:F268"/>
+    <x:mergeCell ref="A270:D270"/>
+    <x:mergeCell ref="A282:F282"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fbaa9f14b6a47c7"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R937bd0bfe7244709"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add trading comps and precedent transactions
</commit_message>
<xml_diff>
--- a/model/QinetiQ_Valuation_Model.xlsx
+++ b/model/QinetiQ_Valuation_Model.xlsx
@@ -2,12 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R7962d4b259f148c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Reabf71765248468e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="R794de2ba3ec94caf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R72ed22169d0b4b59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rfaafeabe54994597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="R629b11454a6142df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R864877b2e1ea4973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Ra785ac3e09a547bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="R12e7e3ba42c24885"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R6dddc7574af34fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R35651bbadb6f4be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="Rdc47e0d8d3ab4457"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="7" r:id="R83a5855761034028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedents" sheetId="8" r:id="Ra09e5cb618034833"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -876,7 +878,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="21">
+  <x:numFmts count="22">
     <x:numFmt numFmtId="164" formatCode="General"/>
     <x:numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
     <x:numFmt numFmtId="166" formatCode="#,##0.0;\(#,##0.0\);\-"/>
@@ -898,8 +900,9 @@
     <x:numFmt numFmtId="208" formatCode="0.000"/>
     <x:numFmt numFmtId="209" formatCode="0.00;[Red](0.00);-"/>
     <x:numFmt numFmtId="210" formatCode="0.000x"/>
+    <x:numFmt numFmtId="211" formatCode="£0.00;[Red](£0.00);-"/>
   </x:numFmts>
-  <x:fonts count="32">
+  <x:fonts count="34">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -1078,8 +1081,20 @@
       <x:color rgb="FF0000FF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="46">
+  <x:fills count="51">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1306,6 +1321,31 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="22">
     <x:border diagonalUp="0" diagonalDown="0"/>
@@ -1504,7 +1544,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="522">
+  <x:cellXfs count="617">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -3070,6 +3110,291 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="12" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="47" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="48" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="48" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="33" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="16" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="16" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="33" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="16" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="16" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="33" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="16" fillId="49" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="16" fillId="49" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="27" fillId="49" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="27" fillId="49" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="27" fillId="49" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="27" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="49" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="50" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="27" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="49" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="27" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="0" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="0" fillId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="27" fillId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="49" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="50" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="33" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="7">
@@ -3597,7 +3922,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="1" t="str">
-        <x:v>0.7</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
@@ -3661,7 +3986,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D12" s="1" t="str">
-        <x:v>US disposal-case DCF complete</x:v>
+        <x:v>Trading comparables and precedent transactions complete</x:v>
       </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
@@ -16641,12 +16966,24 @@
     <x:row r="26" ht="15" hidden="0">
       <x:c r="A26" s="1"/>
       <x:c r="B26" s="1"/>
-      <x:c r="C26" s="1"/>
-      <x:c r="D26" s="1"/>
-      <x:c r="E26" s="1"/>
-      <x:c r="F26" s="1"/>
-      <x:c r="G26" s="1"/>
-      <x:c r="H26" s="1"/>
+      <x:c r="C26" s="1" t="str">
+        <x:v>S020</x:v>
+      </x:c>
+      <x:c r="D26" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E26" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="F26" s="1" t="str">
+        <x:v>London Stock Exchange</x:v>
+      </x:c>
+      <x:c r="G26" s="1" t="str">
+        <x:v>Babcock International Group company page</x:v>
+      </x:c>
+      <x:c r="H26" s="1" t="str">
+        <x:v>https://www.londonstockexchange.com/stock/BAB/babcock-international-group-plc/company-page</x:v>
+      </x:c>
       <x:c r="I26" s="1"/>
       <x:c r="J26" s="1"/>
       <x:c r="K26" s="1"/>
@@ -16669,12 +17006,24 @@
     <x:row r="27" ht="15" hidden="0">
       <x:c r="A27" s="1"/>
       <x:c r="B27" s="1"/>
-      <x:c r="C27" s="1"/>
-      <x:c r="D27" s="1"/>
-      <x:c r="E27" s="1"/>
-      <x:c r="F27" s="1"/>
-      <x:c r="G27" s="1"/>
-      <x:c r="H27" s="1"/>
+      <x:c r="C27" s="1" t="str">
+        <x:v>S021</x:v>
+      </x:c>
+      <x:c r="D27" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E27" s="1" t="str">
+        <x:v>2026-06-22</x:v>
+      </x:c>
+      <x:c r="F27" s="1" t="str">
+        <x:v>Babcock International Group plc</x:v>
+      </x:c>
+      <x:c r="G27" s="1" t="str">
+        <x:v>Annual Report and Financial Statements 2026</x:v>
+      </x:c>
+      <x:c r="H27" s="1" t="str">
+        <x:v>https://www.babcockinternational.com/investors/annual-report-financial-statements-2026/</x:v>
+      </x:c>
       <x:c r="I27" s="1"/>
       <x:c r="J27" s="1"/>
       <x:c r="K27" s="1"/>
@@ -16697,12 +17046,24 @@
     <x:row r="28" ht="15" hidden="0">
       <x:c r="A28" s="1"/>
       <x:c r="B28" s="1"/>
-      <x:c r="C28" s="1"/>
-      <x:c r="D28" s="1"/>
-      <x:c r="E28" s="1"/>
-      <x:c r="F28" s="1"/>
-      <x:c r="G28" s="1"/>
-      <x:c r="H28" s="1"/>
+      <x:c r="C28" s="1" t="str">
+        <x:v>S022</x:v>
+      </x:c>
+      <x:c r="D28" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E28" s="1" t="str">
+        <x:v>2025-12-09</x:v>
+      </x:c>
+      <x:c r="F28" s="1" t="str">
+        <x:v>Chemring Group plc</x:v>
+      </x:c>
+      <x:c r="G28" s="1" t="str">
+        <x:v>FY25 Full Year Results</x:v>
+      </x:c>
+      <x:c r="H28" s="1" t="str">
+        <x:v>https://www.chemring.com/media/press-releases/2025/09-12-2025</x:v>
+      </x:c>
       <x:c r="I28" s="1"/>
       <x:c r="J28" s="1"/>
       <x:c r="K28" s="1"/>
@@ -16725,12 +17086,24 @@
     <x:row r="29" ht="15" hidden="0">
       <x:c r="A29" s="1"/>
       <x:c r="B29" s="1"/>
-      <x:c r="C29" s="1"/>
-      <x:c r="D29" s="1"/>
-      <x:c r="E29" s="1"/>
-      <x:c r="F29" s="1"/>
-      <x:c r="G29" s="1"/>
-      <x:c r="H29" s="1"/>
+      <x:c r="C29" s="1" t="str">
+        <x:v>S023</x:v>
+      </x:c>
+      <x:c r="D29" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E29" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="F29" s="1" t="str">
+        <x:v>London Stock Exchange</x:v>
+      </x:c>
+      <x:c r="G29" s="1" t="str">
+        <x:v>Chemring Group company page</x:v>
+      </x:c>
+      <x:c r="H29" s="1" t="str">
+        <x:v>https://www.londonstockexchange.com/stock/CHG/chemring-group-plc/company-page</x:v>
+      </x:c>
       <x:c r="I29" s="1"/>
       <x:c r="J29" s="1"/>
       <x:c r="K29" s="1"/>
@@ -16753,12 +17126,24 @@
     <x:row r="30" ht="15" hidden="0">
       <x:c r="A30" s="1"/>
       <x:c r="B30" s="1"/>
-      <x:c r="C30" s="1"/>
-      <x:c r="D30" s="1"/>
-      <x:c r="E30" s="1"/>
-      <x:c r="F30" s="1"/>
-      <x:c r="G30" s="1"/>
-      <x:c r="H30" s="1"/>
+      <x:c r="C30" s="1" t="str">
+        <x:v>S024</x:v>
+      </x:c>
+      <x:c r="D30" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E30" s="1" t="str">
+        <x:v>2026-07-23</x:v>
+      </x:c>
+      <x:c r="F30" s="1" t="str">
+        <x:v>Cohort plc</x:v>
+      </x:c>
+      <x:c r="G30" s="1" t="str">
+        <x:v>Annual Report Summary 2026</x:v>
+      </x:c>
+      <x:c r="H30" s="1" t="str">
+        <x:v>https://www.cohortplc.com/investors/annual-report-summary</x:v>
+      </x:c>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="1"/>
       <x:c r="K30" s="1"/>
@@ -16781,12 +17166,24 @@
     <x:row r="31" ht="15" hidden="0">
       <x:c r="A31" s="1"/>
       <x:c r="B31" s="1"/>
-      <x:c r="C31" s="1"/>
-      <x:c r="D31" s="1"/>
-      <x:c r="E31" s="1"/>
-      <x:c r="F31" s="1"/>
-      <x:c r="G31" s="1"/>
-      <x:c r="H31" s="1"/>
+      <x:c r="C31" s="1" t="str">
+        <x:v>S025</x:v>
+      </x:c>
+      <x:c r="D31" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E31" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="F31" s="1" t="str">
+        <x:v>London Stock Exchange</x:v>
+      </x:c>
+      <x:c r="G31" s="1" t="str">
+        <x:v>Cohort plc company page</x:v>
+      </x:c>
+      <x:c r="H31" s="1" t="str">
+        <x:v>https://www.londonstockexchange.com/stock/CHRT/cohort-plc/company-page</x:v>
+      </x:c>
       <x:c r="I31" s="1"/>
       <x:c r="J31" s="1"/>
       <x:c r="K31" s="1"/>
@@ -16809,12 +17206,24 @@
     <x:row r="32" ht="15" hidden="0">
       <x:c r="A32" s="1"/>
       <x:c r="B32" s="1"/>
-      <x:c r="C32" s="1"/>
-      <x:c r="D32" s="1"/>
-      <x:c r="E32" s="1"/>
-      <x:c r="F32" s="1"/>
-      <x:c r="G32" s="1"/>
-      <x:c r="H32" s="1"/>
+      <x:c r="C32" s="1" t="str">
+        <x:v>S026</x:v>
+      </x:c>
+      <x:c r="D32" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E32" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="F32" s="1" t="str">
+        <x:v>Serco Group plc</x:v>
+      </x:c>
+      <x:c r="G32" s="1" t="str">
+        <x:v>Analysts' consensus</x:v>
+      </x:c>
+      <x:c r="H32" s="1" t="str">
+        <x:v>https://www.serco.com/investors/analysts-consensus</x:v>
+      </x:c>
       <x:c r="I32" s="1"/>
       <x:c r="J32" s="1"/>
       <x:c r="K32" s="1"/>
@@ -16837,12 +17246,24 @@
     <x:row r="33" ht="15" hidden="0">
       <x:c r="A33" s="1"/>
       <x:c r="B33" s="1"/>
-      <x:c r="C33" s="1"/>
-      <x:c r="D33" s="1"/>
-      <x:c r="E33" s="1"/>
-      <x:c r="F33" s="1"/>
-      <x:c r="G33" s="1"/>
-      <x:c r="H33" s="1"/>
+      <x:c r="C33" s="1" t="str">
+        <x:v>S027</x:v>
+      </x:c>
+      <x:c r="D33" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E33" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="F33" s="1" t="str">
+        <x:v>ADVFN</x:v>
+      </x:c>
+      <x:c r="G33" s="1" t="str">
+        <x:v>Serco Group market capitalisation</x:v>
+      </x:c>
+      <x:c r="H33" s="1" t="str">
+        <x:v>https://uk.advfn.com/stock-market/london/serco-SRP/financials</x:v>
+      </x:c>
       <x:c r="I33" s="1"/>
       <x:c r="J33" s="1"/>
       <x:c r="K33" s="1"/>
@@ -16865,12 +17286,24 @@
     <x:row r="34" ht="15" hidden="0">
       <x:c r="A34" s="1"/>
       <x:c r="B34" s="1"/>
-      <x:c r="C34" s="1"/>
-      <x:c r="D34" s="1"/>
-      <x:c r="E34" s="1"/>
-      <x:c r="F34" s="1"/>
-      <x:c r="G34" s="1"/>
-      <x:c r="H34" s="1"/>
+      <x:c r="C34" s="1" t="str">
+        <x:v>S028</x:v>
+      </x:c>
+      <x:c r="D34" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E34" s="1" t="str">
+        <x:v>2026-02-17</x:v>
+      </x:c>
+      <x:c r="F34" s="1" t="str">
+        <x:v>U.S. Securities and Exchange Commission</x:v>
+      </x:c>
+      <x:c r="G34" s="1" t="str">
+        <x:v>Leidos company facts</x:v>
+      </x:c>
+      <x:c r="H34" s="1" t="str">
+        <x:v>https://data.sec.gov/api/xbrl/companyfacts/CIK0001336920.json</x:v>
+      </x:c>
       <x:c r="I34" s="1"/>
       <x:c r="J34" s="1"/>
       <x:c r="K34" s="1"/>
@@ -16893,12 +17326,24 @@
     <x:row r="35" ht="15" hidden="0">
       <x:c r="A35" s="1"/>
       <x:c r="B35" s="1"/>
-      <x:c r="C35" s="1"/>
-      <x:c r="D35" s="1"/>
-      <x:c r="E35" s="1"/>
-      <x:c r="F35" s="1"/>
-      <x:c r="G35" s="1"/>
-      <x:c r="H35" s="1"/>
+      <x:c r="C35" s="1" t="str">
+        <x:v>S029</x:v>
+      </x:c>
+      <x:c r="D35" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E35" s="1" t="str">
+        <x:v>2026-08-06</x:v>
+      </x:c>
+      <x:c r="F35" s="1" t="str">
+        <x:v>U.S. Securities and Exchange Commission</x:v>
+      </x:c>
+      <x:c r="G35" s="1" t="str">
+        <x:v>CACI company facts</x:v>
+      </x:c>
+      <x:c r="H35" s="1" t="str">
+        <x:v>https://data.sec.gov/api/xbrl/companyfacts/CIK0000016058.json</x:v>
+      </x:c>
       <x:c r="I35" s="1"/>
       <x:c r="J35" s="1"/>
       <x:c r="K35" s="1"/>
@@ -16921,12 +17366,24 @@
     <x:row r="36" ht="15" hidden="0">
       <x:c r="A36" s="1"/>
       <x:c r="B36" s="1"/>
-      <x:c r="C36" s="1"/>
-      <x:c r="D36" s="1"/>
-      <x:c r="E36" s="1"/>
-      <x:c r="F36" s="1"/>
-      <x:c r="G36" s="1"/>
-      <x:c r="H36" s="1"/>
+      <x:c r="C36" s="1" t="str">
+        <x:v>S030</x:v>
+      </x:c>
+      <x:c r="D36" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E36" s="1" t="str">
+        <x:v>2026-05-22</x:v>
+      </x:c>
+      <x:c r="F36" s="1" t="str">
+        <x:v>U.S. Securities and Exchange Commission</x:v>
+      </x:c>
+      <x:c r="G36" s="1" t="str">
+        <x:v>Booz Allen Hamilton company facts</x:v>
+      </x:c>
+      <x:c r="H36" s="1" t="str">
+        <x:v>https://data.sec.gov/api/xbrl/companyfacts/CIK0001443646.json</x:v>
+      </x:c>
       <x:c r="I36" s="1"/>
       <x:c r="J36" s="1"/>
       <x:c r="K36" s="1"/>
@@ -16949,12 +17406,24 @@
     <x:row r="37" ht="15" hidden="0">
       <x:c r="A37" s="1"/>
       <x:c r="B37" s="1"/>
-      <x:c r="C37" s="1"/>
-      <x:c r="D37" s="1"/>
-      <x:c r="E37" s="1"/>
-      <x:c r="F37" s="1"/>
-      <x:c r="G37" s="1"/>
-      <x:c r="H37" s="1"/>
+      <x:c r="C37" s="1" t="str">
+        <x:v>S031</x:v>
+      </x:c>
+      <x:c r="D37" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E37" s="1" t="str">
+        <x:v>2026-03-16</x:v>
+      </x:c>
+      <x:c r="F37" s="1" t="str">
+        <x:v>U.S. Securities and Exchange Commission</x:v>
+      </x:c>
+      <x:c r="G37" s="1" t="str">
+        <x:v>SAIC company facts</x:v>
+      </x:c>
+      <x:c r="H37" s="1" t="str">
+        <x:v>https://data.sec.gov/api/xbrl/companyfacts/CIK0001571123.json</x:v>
+      </x:c>
       <x:c r="I37" s="1"/>
       <x:c r="J37" s="1"/>
       <x:c r="K37" s="1"/>
@@ -16977,12 +17446,24 @@
     <x:row r="38" ht="15" hidden="0">
       <x:c r="A38" s="1"/>
       <x:c r="B38" s="1"/>
-      <x:c r="C38" s="1"/>
-      <x:c r="D38" s="1"/>
-      <x:c r="E38" s="1"/>
-      <x:c r="F38" s="1"/>
-      <x:c r="G38" s="1"/>
-      <x:c r="H38" s="1"/>
+      <x:c r="C38" s="1" t="str">
+        <x:v>S032</x:v>
+      </x:c>
+      <x:c r="D38" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E38" s="1" t="str">
+        <x:v>2019-12-17</x:v>
+      </x:c>
+      <x:c r="F38" s="1" t="str">
+        <x:v>Leidos Holdings Inc.</x:v>
+      </x:c>
+      <x:c r="G38" s="1" t="str">
+        <x:v>Leidos to Acquire Dynetics</x:v>
+      </x:c>
+      <x:c r="H38" s="1" t="str">
+        <x:v>https://investors.leidos.com/news-and-events/news-releases/press-release-details/2019/Leidos-to-Acquire-Dynetics/default.aspx</x:v>
+      </x:c>
       <x:c r="I38" s="1"/>
       <x:c r="J38" s="1"/>
       <x:c r="K38" s="1"/>
@@ -17005,12 +17486,24 @@
     <x:row r="39" ht="15" hidden="0">
       <x:c r="A39" s="1"/>
       <x:c r="B39" s="1"/>
-      <x:c r="C39" s="1"/>
-      <x:c r="D39" s="1"/>
-      <x:c r="E39" s="1"/>
-      <x:c r="F39" s="1"/>
-      <x:c r="G39" s="1"/>
-      <x:c r="H39" s="1"/>
+      <x:c r="C39" s="1" t="str">
+        <x:v>S033</x:v>
+      </x:c>
+      <x:c r="D39" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E39" s="1" t="str">
+        <x:v>2024-09-16</x:v>
+      </x:c>
+      <x:c r="F39" s="1" t="str">
+        <x:v>CACI International Inc.</x:v>
+      </x:c>
+      <x:c r="G39" s="1" t="str">
+        <x:v>CACI to Purchase Azure Summit Technology</x:v>
+      </x:c>
+      <x:c r="H39" s="1" t="str">
+        <x:v>https://investor.caci.com/2024-09-16-CACI-Enters-into-Definitive-Agreement-to-Purchase-Azure-Summit-Technology</x:v>
+      </x:c>
       <x:c r="I39" s="1"/>
       <x:c r="J39" s="1"/>
       <x:c r="K39" s="1"/>
@@ -17033,12 +17526,24 @@
     <x:row r="40" ht="15" hidden="0">
       <x:c r="A40" s="1"/>
       <x:c r="B40" s="1"/>
-      <x:c r="C40" s="1"/>
-      <x:c r="D40" s="1"/>
-      <x:c r="E40" s="1"/>
-      <x:c r="F40" s="1"/>
-      <x:c r="G40" s="1"/>
-      <x:c r="H40" s="1"/>
+      <x:c r="C40" s="1" t="str">
+        <x:v>S034</x:v>
+      </x:c>
+      <x:c r="D40" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E40" s="1" t="str">
+        <x:v>2024-07-16</x:v>
+      </x:c>
+      <x:c r="F40" s="1" t="str">
+        <x:v>KBR Inc.</x:v>
+      </x:c>
+      <x:c r="G40" s="1" t="str">
+        <x:v>KBR to Acquire LinQuest</x:v>
+      </x:c>
+      <x:c r="H40" s="1" t="str">
+        <x:v>https://www.kbr.com/en/insights-news/press-release/kbr-acquire-linquest-expanding-technical-capabilities-across-air-space-and-digital-domains</x:v>
+      </x:c>
       <x:c r="I40" s="1"/>
       <x:c r="J40" s="1"/>
       <x:c r="K40" s="1"/>
@@ -17061,12 +17566,24 @@
     <x:row r="41" ht="15" hidden="0">
       <x:c r="A41" s="1"/>
       <x:c r="B41" s="1"/>
-      <x:c r="C41" s="1"/>
-      <x:c r="D41" s="1"/>
-      <x:c r="E41" s="1"/>
-      <x:c r="F41" s="1"/>
-      <x:c r="G41" s="1"/>
-      <x:c r="H41" s="1"/>
+      <x:c r="C41" s="1" t="str">
+        <x:v>S035</x:v>
+      </x:c>
+      <x:c r="D41" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E41" s="1" t="str">
+        <x:v>2022-02-15</x:v>
+      </x:c>
+      <x:c r="F41" s="1" t="str">
+        <x:v>Amentum</x:v>
+      </x:c>
+      <x:c r="G41" s="1" t="str">
+        <x:v>Amentum Completes Acquisition of PAE</x:v>
+      </x:c>
+      <x:c r="H41" s="1" t="str">
+        <x:v>https://www.amentum.com/news/amentum-completes-acquisition-of-pae/</x:v>
+      </x:c>
       <x:c r="I41" s="1"/>
       <x:c r="J41" s="1"/>
       <x:c r="K41" s="1"/>
@@ -17089,12 +17606,24 @@
     <x:row r="42" ht="15" hidden="0">
       <x:c r="A42" s="1"/>
       <x:c r="B42" s="1"/>
-      <x:c r="C42" s="1"/>
-      <x:c r="D42" s="1"/>
-      <x:c r="E42" s="1"/>
-      <x:c r="F42" s="1"/>
-      <x:c r="G42" s="1"/>
-      <x:c r="H42" s="1"/>
+      <x:c r="C42" s="1" t="str">
+        <x:v>S036</x:v>
+      </x:c>
+      <x:c r="D42" s="1" t="str">
+        <x:v>2026-09-16</x:v>
+      </x:c>
+      <x:c r="E42" s="1" t="str">
+        <x:v>2021-03-16</x:v>
+      </x:c>
+      <x:c r="F42" s="1" t="str">
+        <x:v>U.S. Securities and Exchange Commission</x:v>
+      </x:c>
+      <x:c r="G42" s="1" t="str">
+        <x:v>PAE company facts</x:v>
+      </x:c>
+      <x:c r="H42" s="1" t="str">
+        <x:v>https://data.sec.gov/api/xbrl/companyfacts/CIK0001720821.json</x:v>
+      </x:c>
       <x:c r="I42" s="1"/>
       <x:c r="J42" s="1"/>
       <x:c r="K42" s="1"/>
@@ -23603,6 +24132,1646 @@
     <x:mergeCell ref="A282:F282"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R937bd0bfe7244709"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4c1e2ae604b4960"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="23" customHeight="1">
+      <x:c r="A1" s="557" t="str">
+        <x:v>QinetiQ trading comparable companies</x:v>
+      </x:c>
+      <x:c r="B1" s="557"/>
+      <x:c r="C1" s="557"/>
+      <x:c r="D1" s="557"/>
+      <x:c r="E1" s="557"/>
+      <x:c r="F1" s="557"/>
+      <x:c r="G1" s="557"/>
+      <x:c r="H1" s="557"/>
+      <x:c r="I1" s="557"/>
+      <x:c r="J1" s="557"/>
+      <x:c r="K1" s="557"/>
+      <x:c r="L1" s="557"/>
+      <x:c r="M1" s="557"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="528" t="str">
+        <x:v>Purpose: value QinetiQ using current listed-company enterprise-value multiples as an independent market cross-check on the DCF. Market capitalisations are at 16 September 2026; financials use the latest completed annual period. £m for UK companies and $m for US companies, so no FX conversion is required to calculate multiples.</x:v>
+      </x:c>
+      <x:c r="B2" s="528"/>
+      <x:c r="C2" s="528"/>
+      <x:c r="D2" s="528"/>
+      <x:c r="E2" s="528"/>
+      <x:c r="F2" s="528"/>
+      <x:c r="G2" s="528"/>
+      <x:c r="H2" s="528"/>
+      <x:c r="I2" s="528"/>
+      <x:c r="J2" s="528"/>
+      <x:c r="K2" s="528"/>
+      <x:c r="L2" s="528"/>
+      <x:c r="M2" s="528"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="528"/>
+      <x:c r="B3" s="528"/>
+      <x:c r="C3" s="528"/>
+      <x:c r="D3" s="528"/>
+      <x:c r="E3" s="528"/>
+      <x:c r="F3" s="528"/>
+      <x:c r="G3" s="528"/>
+      <x:c r="H3" s="528"/>
+      <x:c r="I3" s="528"/>
+      <x:c r="J3" s="528"/>
+      <x:c r="K3" s="528"/>
+      <x:c r="L3" s="528"/>
+      <x:c r="M3" s="528"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="321"/>
+      <x:c r="B4" s="321"/>
+      <x:c r="C4" s="321"/>
+      <x:c r="D4" s="321"/>
+      <x:c r="E4" s="321"/>
+      <x:c r="F4" s="321"/>
+      <x:c r="G4" s="321"/>
+      <x:c r="H4" s="321"/>
+      <x:c r="I4" s="321"/>
+      <x:c r="J4" s="321"/>
+      <x:c r="K4" s="321"/>
+      <x:c r="L4" s="321"/>
+      <x:c r="M4" s="321"/>
+    </x:row>
+    <x:row r="5" ht="31" customHeight="1">
+      <x:c r="A5" s="534" t="str">
+        <x:v>Company</x:v>
+      </x:c>
+      <x:c r="B5" s="534" t="str">
+        <x:v>Peer group</x:v>
+      </x:c>
+      <x:c r="C5" s="534" t="str">
+        <x:v>CCY</x:v>
+      </x:c>
+      <x:c r="D5" s="534" t="str">
+        <x:v>Market cap</x:v>
+      </x:c>
+      <x:c r="E5" s="534" t="str">
+        <x:v>Debt</x:v>
+      </x:c>
+      <x:c r="F5" s="534" t="str">
+        <x:v>Cash</x:v>
+      </x:c>
+      <x:c r="G5" s="534" t="str">
+        <x:v>Net debt</x:v>
+      </x:c>
+      <x:c r="H5" s="534" t="str">
+        <x:v>Enterprise value</x:v>
+      </x:c>
+      <x:c r="I5" s="534" t="str">
+        <x:v>Revenue</x:v>
+      </x:c>
+      <x:c r="J5" s="534" t="str">
+        <x:v>Operating profit</x:v>
+      </x:c>
+      <x:c r="K5" s="534" t="str">
+        <x:v>EBIT margin</x:v>
+      </x:c>
+      <x:c r="L5" s="534" t="str">
+        <x:v>EV / revenue</x:v>
+      </x:c>
+      <x:c r="M5" s="534" t="str">
+        <x:v>EV / op. profit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="573" t="str">
+        <x:v>Babcock</x:v>
+      </x:c>
+      <x:c r="B6" s="573" t="str">
+        <x:v>UK defence / engineering</x:v>
+      </x:c>
+      <x:c r="C6" s="573" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
+      <x:c r="D6" s="469" t="n">
+        <x:v>4714.59</x:v>
+      </x:c>
+      <x:c r="E6" s="469" t="n">
+        <x:v>22.7</x:v>
+      </x:c>
+      <x:c r="F6" s="469" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="386" t="n">
+        <x:f>E6-F6</x:f>
+        <x:v>22.7</x:v>
+      </x:c>
+      <x:c r="H6" s="386" t="n">
+        <x:f>D6+G6</x:f>
+        <x:v>4737.29</x:v>
+      </x:c>
+      <x:c r="I6" s="469" t="n">
+        <x:v>5178</x:v>
+      </x:c>
+      <x:c r="J6" s="469" t="n">
+        <x:v>433</x:v>
+      </x:c>
+      <x:c r="K6" s="568" t="n">
+        <x:f>J6/I6</x:f>
+        <x:v>0.08362302047122441</x:v>
+      </x:c>
+      <x:c r="L6" s="566" t="n">
+        <x:f>H6/I6</x:f>
+        <x:v>0.9148879876400154</x:v>
+      </x:c>
+      <x:c r="M6" s="566" t="n">
+        <x:f>H6/J6</x:f>
+        <x:v>10.940623556581986</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="573" t="str">
+        <x:v>Chemring</x:v>
+      </x:c>
+      <x:c r="B7" s="573" t="str">
+        <x:v>UK defence / products</x:v>
+      </x:c>
+      <x:c r="C7" s="573" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
+      <x:c r="D7" s="469" t="n">
+        <x:v>1424.58</x:v>
+      </x:c>
+      <x:c r="E7" s="469" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="F7" s="469" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G7" s="386" t="n">
+        <x:f>E7-F7</x:f>
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H7" s="386" t="n">
+        <x:f>D7+G7</x:f>
+        <x:v>1513.58</x:v>
+      </x:c>
+      <x:c r="I7" s="469" t="n">
+        <x:v>497.5</x:v>
+      </x:c>
+      <x:c r="J7" s="469" t="n">
+        <x:v>73.5</x:v>
+      </x:c>
+      <x:c r="K7" s="568" t="n">
+        <x:f>J7/I7</x:f>
+        <x:v>0.14773869346733667</x:v>
+      </x:c>
+      <x:c r="L7" s="566" t="n">
+        <x:f>H7/I7</x:f>
+        <x:v>3.042371859296482</x:v>
+      </x:c>
+      <x:c r="M7" s="566" t="n">
+        <x:f>H7/J7</x:f>
+        <x:v>20.592925170068025</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="573" t="str">
+        <x:v>Cohort</x:v>
+      </x:c>
+      <x:c r="B8" s="573" t="str">
+        <x:v>UK defence / technology</x:v>
+      </x:c>
+      <x:c r="C8" s="573" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
+      <x:c r="D8" s="469" t="n">
+        <x:v>530.48</x:v>
+      </x:c>
+      <x:c r="E8" s="469" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="469" t="n">
+        <x:v>2.217</x:v>
+      </x:c>
+      <x:c r="G8" s="386" t="n">
+        <x:f>E8-F8</x:f>
+        <x:v>-2.217</x:v>
+      </x:c>
+      <x:c r="H8" s="386" t="n">
+        <x:f>D8+G8</x:f>
+        <x:v>528.263</x:v>
+      </x:c>
+      <x:c r="I8" s="469" t="n">
+        <x:v>306.4</x:v>
+      </x:c>
+      <x:c r="J8" s="469" t="n">
+        <x:v>36.3</x:v>
+      </x:c>
+      <x:c r="K8" s="568" t="n">
+        <x:f>J8/I8</x:f>
+        <x:v>0.11847258485639686</x:v>
+      </x:c>
+      <x:c r="L8" s="566" t="n">
+        <x:f>H8/I8</x:f>
+        <x:v>1.7240959530026112</x:v>
+      </x:c>
+      <x:c r="M8" s="566" t="n">
+        <x:f>H8/J8</x:f>
+        <x:v>14.55269972451791</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="573" t="str">
+        <x:v>Serco</x:v>
+      </x:c>
+      <x:c r="B9" s="573" t="str">
+        <x:v>Government services</x:v>
+      </x:c>
+      <x:c r="C9" s="573" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
+      <x:c r="D9" s="469" t="n">
+        <x:v>2411.872</x:v>
+      </x:c>
+      <x:c r="E9" s="469" t="n">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="F9" s="469" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="386" t="n">
+        <x:f>E9-F9</x:f>
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="H9" s="386" t="n">
+        <x:f>D9+G9</x:f>
+        <x:v>2617.872</x:v>
+      </x:c>
+      <x:c r="I9" s="469" t="n">
+        <x:v>4877</x:v>
+      </x:c>
+      <x:c r="J9" s="469" t="n">
+        <x:v>272</x:v>
+      </x:c>
+      <x:c r="K9" s="568" t="n">
+        <x:f>J9/I9</x:f>
+        <x:v>0.055771990978060286</x:v>
+      </x:c>
+      <x:c r="L9" s="566" t="n">
+        <x:f>H9/I9</x:f>
+        <x:v>0.536779167521017</x:v>
+      </x:c>
+      <x:c r="M9" s="566" t="n">
+        <x:f>H9/J9</x:f>
+        <x:v>9.624529411764705</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="573" t="str">
+        <x:v>Leidos</x:v>
+      </x:c>
+      <x:c r="B10" s="573" t="str">
+        <x:v>US defence / technology</x:v>
+      </x:c>
+      <x:c r="C10" s="573" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D10" s="469" t="n">
+        <x:v>16350.38</x:v>
+      </x:c>
+      <x:c r="E10" s="469" t="n">
+        <x:v>4648</x:v>
+      </x:c>
+      <x:c r="F10" s="469" t="n">
+        <x:v>1108</x:v>
+      </x:c>
+      <x:c r="G10" s="386" t="n">
+        <x:f>E10-F10</x:f>
+        <x:v>3540</x:v>
+      </x:c>
+      <x:c r="H10" s="386" t="n">
+        <x:f>D10+G10</x:f>
+        <x:v>19890.379999999997</x:v>
+      </x:c>
+      <x:c r="I10" s="469" t="n">
+        <x:v>17174</x:v>
+      </x:c>
+      <x:c r="J10" s="469" t="n">
+        <x:v>2109</x:v>
+      </x:c>
+      <x:c r="K10" s="568" t="n">
+        <x:f>J10/I10</x:f>
+        <x:v>0.12280190986374752</x:v>
+      </x:c>
+      <x:c r="L10" s="566" t="n">
+        <x:f>H10/I10</x:f>
+        <x:v>1.1581681611738672</x:v>
+      </x:c>
+      <x:c r="M10" s="566" t="n">
+        <x:f>H10/J10</x:f>
+        <x:v>9.431190137505926</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="573" t="str">
+        <x:v>CACI</x:v>
+      </x:c>
+      <x:c r="B11" s="573" t="str">
+        <x:v>US defence / intelligence</x:v>
+      </x:c>
+      <x:c r="C11" s="573" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D11" s="469" t="n">
+        <x:v>13977.692</x:v>
+      </x:c>
+      <x:c r="E11" s="469" t="n">
+        <x:v>4901.509</x:v>
+      </x:c>
+      <x:c r="F11" s="469" t="n">
+        <x:v>191.756</x:v>
+      </x:c>
+      <x:c r="G11" s="386" t="n">
+        <x:f>E11-F11</x:f>
+        <x:v>4709.753</x:v>
+      </x:c>
+      <x:c r="H11" s="386" t="n">
+        <x:f>D11+G11</x:f>
+        <x:v>18687.445</x:v>
+      </x:c>
+      <x:c r="I11" s="469" t="n">
+        <x:v>9567.779</x:v>
+      </x:c>
+      <x:c r="J11" s="469" t="n">
+        <x:v>919.815</x:v>
+      </x:c>
+      <x:c r="K11" s="568" t="n">
+        <x:f>J11/I11</x:f>
+        <x:v>0.0961367314190681</x:v>
+      </x:c>
+      <x:c r="L11" s="566" t="n">
+        <x:f>H11/I11</x:f>
+        <x:v>1.9531643655230748</x:v>
+      </x:c>
+      <x:c r="M11" s="566" t="n">
+        <x:f>H11/J11</x:f>
+        <x:v>20.316525605692448</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="573" t="str">
+        <x:v>Booz Allen Hamilton</x:v>
+      </x:c>
+      <x:c r="B12" s="573" t="str">
+        <x:v>US government technology</x:v>
+      </x:c>
+      <x:c r="C12" s="573" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D12" s="469" t="n">
+        <x:v>9468.833</x:v>
+      </x:c>
+      <x:c r="E12" s="469" t="n">
+        <x:v>3940</x:v>
+      </x:c>
+      <x:c r="F12" s="469" t="n">
+        <x:v>728</x:v>
+      </x:c>
+      <x:c r="G12" s="386" t="n">
+        <x:f>E12-F12</x:f>
+        <x:v>3212</x:v>
+      </x:c>
+      <x:c r="H12" s="386" t="n">
+        <x:f>D12+G12</x:f>
+        <x:v>12680.833</x:v>
+      </x:c>
+      <x:c r="I12" s="469" t="n">
+        <x:v>11217</x:v>
+      </x:c>
+      <x:c r="J12" s="469" t="n">
+        <x:v>1033</x:v>
+      </x:c>
+      <x:c r="K12" s="568" t="n">
+        <x:f>J12/I12</x:f>
+        <x:v>0.09209235981100115</x:v>
+      </x:c>
+      <x:c r="L12" s="566" t="n">
+        <x:f>H12/I12</x:f>
+        <x:v>1.1305012926807525</x:v>
+      </x:c>
+      <x:c r="M12" s="566" t="n">
+        <x:f>H12/J12</x:f>
+        <x:v>12.275733785091965</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="573" t="str">
+        <x:v>SAIC</x:v>
+      </x:c>
+      <x:c r="B13" s="573" t="str">
+        <x:v>US government technology</x:v>
+      </x:c>
+      <x:c r="C13" s="573" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="D13" s="469" t="n">
+        <x:v>5535.516</x:v>
+      </x:c>
+      <x:c r="E13" s="469" t="n">
+        <x:v>2487</x:v>
+      </x:c>
+      <x:c r="F13" s="469" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="G13" s="386" t="n">
+        <x:f>E13-F13</x:f>
+        <x:v>2305</x:v>
+      </x:c>
+      <x:c r="H13" s="386" t="n">
+        <x:f>D13+G13</x:f>
+        <x:v>7840.516</x:v>
+      </x:c>
+      <x:c r="I13" s="469" t="n">
+        <x:v>7262</x:v>
+      </x:c>
+      <x:c r="J13" s="469" t="n">
+        <x:v>521</x:v>
+      </x:c>
+      <x:c r="K13" s="568" t="n">
+        <x:f>J13/I13</x:f>
+        <x:v>0.07174332139906361</x:v>
+      </x:c>
+      <x:c r="L13" s="566" t="n">
+        <x:f>H13/I13</x:f>
+        <x:v>1.0796634535940512</x:v>
+      </x:c>
+      <x:c r="M13" s="566" t="n">
+        <x:f>H13/J13</x:f>
+        <x:v>15.048975047984644</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="366"/>
+      <x:c r="B14" s="366"/>
+      <x:c r="C14" s="366"/>
+      <x:c r="D14" s="386"/>
+      <x:c r="E14" s="386"/>
+      <x:c r="F14" s="386"/>
+      <x:c r="G14" s="386"/>
+      <x:c r="H14" s="386"/>
+      <x:c r="I14" s="386"/>
+      <x:c r="J14" s="386"/>
+      <x:c r="K14" s="568"/>
+      <x:c r="L14" s="566"/>
+      <x:c r="M14" s="566"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="574" t="str">
+        <x:v>QinetiQ</x:v>
+      </x:c>
+      <x:c r="B15" s="574" t="str">
+        <x:v>Subject company</x:v>
+      </x:c>
+      <x:c r="C15" s="574" t="str">
+        <x:v>GBP</x:v>
+      </x:c>
+      <x:c r="D15" s="575" t="n">
+        <x:v>2434.72</x:v>
+      </x:c>
+      <x:c r="E15" s="575" t="n">
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="F15" s="575" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="576" t="n">
+        <x:f>E15-F15</x:f>
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="H15" s="576" t="n">
+        <x:f>D15+G15</x:f>
+        <x:v>2593.8199999999997</x:v>
+      </x:c>
+      <x:c r="I15" s="575" t="n">
+        <x:v>1922.6</x:v>
+      </x:c>
+      <x:c r="J15" s="575" t="n">
+        <x:v>217.9</x:v>
+      </x:c>
+      <x:c r="K15" s="577" t="n">
+        <x:f>J15/I15</x:f>
+        <x:v>0.11333610735462396</x:v>
+      </x:c>
+      <x:c r="L15" s="578" t="n">
+        <x:f>H15/I15</x:f>
+        <x:v>1.3491209820035368</x:v>
+      </x:c>
+      <x:c r="M15" s="578" t="n">
+        <x:f>H15/J15</x:f>
+        <x:v>11.903717301514455</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="321"/>
+      <x:c r="B16" s="321"/>
+      <x:c r="C16" s="321"/>
+      <x:c r="D16" s="321"/>
+      <x:c r="E16" s="321"/>
+      <x:c r="F16" s="321"/>
+      <x:c r="G16" s="321"/>
+      <x:c r="H16" s="321"/>
+      <x:c r="I16" s="321"/>
+      <x:c r="J16" s="321"/>
+      <x:c r="K16" s="321"/>
+      <x:c r="L16" s="321"/>
+      <x:c r="M16" s="321"/>
+    </x:row>
+    <x:row r="17" ht="23" customHeight="1">
+      <x:c r="A17" s="557" t="str">
+        <x:v>Peer multiple range</x:v>
+      </x:c>
+      <x:c r="B17" s="557"/>
+      <x:c r="C17" s="557"/>
+      <x:c r="D17" s="557"/>
+      <x:c r="E17" s="557"/>
+      <x:c r="F17" s="557"/>
+      <x:c r="G17" s="321"/>
+      <x:c r="H17" s="321"/>
+      <x:c r="I17" s="321"/>
+      <x:c r="J17" s="321"/>
+      <x:c r="K17" s="321"/>
+      <x:c r="L17" s="321"/>
+      <x:c r="M17" s="321"/>
+    </x:row>
+    <x:row r="18" ht="31" customHeight="1">
+      <x:c r="A18" s="534" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B18" s="534" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="C18" s="534" t="str">
+        <x:v>Median</x:v>
+      </x:c>
+      <x:c r="D18" s="534" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E18" s="321"/>
+      <x:c r="F18" s="321"/>
+      <x:c r="G18" s="321"/>
+      <x:c r="H18" s="321"/>
+      <x:c r="I18" s="321"/>
+      <x:c r="J18" s="321"/>
+      <x:c r="K18" s="321"/>
+      <x:c r="L18" s="321"/>
+      <x:c r="M18" s="321"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="321" t="str">
+        <x:v>EV / revenue</x:v>
+      </x:c>
+      <x:c r="B19" s="559" t="n">
+        <x:f>MIN(L6:L13)</x:f>
+        <x:v>0.536779167521017</x:v>
+      </x:c>
+      <x:c r="C19" s="565" t="n">
+        <x:f>MEDIAN(L6:L13)</x:f>
+        <x:v>1.1443347269273099</x:v>
+      </x:c>
+      <x:c r="D19" s="559" t="n">
+        <x:f>MAX(L6:L13)</x:f>
+        <x:v>3.042371859296482</x:v>
+      </x:c>
+      <x:c r="E19" s="321"/>
+      <x:c r="F19" s="321"/>
+      <x:c r="G19" s="321"/>
+      <x:c r="H19" s="321"/>
+      <x:c r="I19" s="321"/>
+      <x:c r="J19" s="321"/>
+      <x:c r="K19" s="321"/>
+      <x:c r="L19" s="321"/>
+      <x:c r="M19" s="321"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="321" t="str">
+        <x:v>EV / operating profit</x:v>
+      </x:c>
+      <x:c r="B20" s="559" t="n">
+        <x:f>MIN(M6:M13)</x:f>
+        <x:v>9.431190137505926</x:v>
+      </x:c>
+      <x:c r="C20" s="565" t="n">
+        <x:f>MEDIAN(M6:M13)</x:f>
+        <x:v>13.414216754804936</x:v>
+      </x:c>
+      <x:c r="D20" s="559" t="n">
+        <x:f>MAX(M6:M13)</x:f>
+        <x:v>20.592925170068025</x:v>
+      </x:c>
+      <x:c r="E20" s="321"/>
+      <x:c r="F20" s="321"/>
+      <x:c r="G20" s="321"/>
+      <x:c r="H20" s="321"/>
+      <x:c r="I20" s="321"/>
+      <x:c r="J20" s="321"/>
+      <x:c r="K20" s="321"/>
+      <x:c r="L20" s="321"/>
+      <x:c r="M20" s="321"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="321"/>
+      <x:c r="B21" s="321"/>
+      <x:c r="C21" s="321"/>
+      <x:c r="D21" s="321"/>
+      <x:c r="E21" s="321"/>
+      <x:c r="F21" s="321"/>
+      <x:c r="G21" s="321"/>
+      <x:c r="H21" s="321"/>
+      <x:c r="I21" s="321"/>
+      <x:c r="J21" s="321"/>
+      <x:c r="K21" s="321"/>
+      <x:c r="L21" s="321"/>
+      <x:c r="M21" s="321"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="321"/>
+      <x:c r="B22" s="321"/>
+      <x:c r="C22" s="321"/>
+      <x:c r="D22" s="321"/>
+      <x:c r="E22" s="321"/>
+      <x:c r="F22" s="321"/>
+      <x:c r="G22" s="321"/>
+      <x:c r="H22" s="321"/>
+      <x:c r="I22" s="321"/>
+      <x:c r="J22" s="321"/>
+      <x:c r="K22" s="321"/>
+      <x:c r="L22" s="321"/>
+      <x:c r="M22" s="321"/>
+    </x:row>
+    <x:row r="23" ht="23" customHeight="1">
+      <x:c r="A23" s="557" t="str">
+        <x:v>Implied QinetiQ valuation</x:v>
+      </x:c>
+      <x:c r="B23" s="557"/>
+      <x:c r="C23" s="557"/>
+      <x:c r="D23" s="557"/>
+      <x:c r="E23" s="557"/>
+      <x:c r="F23" s="557"/>
+      <x:c r="G23" s="557"/>
+      <x:c r="H23" s="557"/>
+      <x:c r="I23" s="557"/>
+      <x:c r="J23" s="321"/>
+      <x:c r="K23" s="321"/>
+      <x:c r="L23" s="321"/>
+      <x:c r="M23" s="321"/>
+    </x:row>
+    <x:row r="24" ht="31" customHeight="1">
+      <x:c r="A24" s="534" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="B24" s="534" t="str">
+        <x:v>Peer median</x:v>
+      </x:c>
+      <x:c r="C24" s="534" t="str">
+        <x:v>QinetiQ metric</x:v>
+      </x:c>
+      <x:c r="D24" s="534" t="str">
+        <x:v>Implied EV</x:v>
+      </x:c>
+      <x:c r="E24" s="534" t="str">
+        <x:v>Less: net debt</x:v>
+      </x:c>
+      <x:c r="F24" s="534" t="str">
+        <x:v>Implied equity value</x:v>
+      </x:c>
+      <x:c r="G24" s="534" t="str">
+        <x:v>Diluted shares</x:v>
+      </x:c>
+      <x:c r="H24" s="534" t="str">
+        <x:v>Value / share</x:v>
+      </x:c>
+      <x:c r="I24" s="534" t="str">
+        <x:v>Vs current price</x:v>
+      </x:c>
+      <x:c r="J24" s="321"/>
+      <x:c r="K24" s="321"/>
+      <x:c r="L24" s="321"/>
+      <x:c r="M24" s="321"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="366" t="str">
+        <x:v>EV / revenue</x:v>
+      </x:c>
+      <x:c r="B25" s="566" t="n">
+        <x:f>$C$19</x:f>
+        <x:v>1.1443347269273099</x:v>
+      </x:c>
+      <x:c r="C25" s="386" t="n">
+        <x:f>$I$15</x:f>
+        <x:v>1922.6</x:v>
+      </x:c>
+      <x:c r="D25" s="386" t="n">
+        <x:f>B25*C25</x:f>
+        <x:v>2200.0979459904456</x:v>
+      </x:c>
+      <x:c r="E25" s="386" t="n">
+        <x:f>$G$15</x:f>
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="F25" s="386" t="n">
+        <x:f>D25-E25</x:f>
+        <x:v>2040.9979459904457</x:v>
+      </x:c>
+      <x:c r="G25" s="386" t="n">
+        <x:f>Forecast!$B$106</x:f>
+        <x:v>522.1</x:v>
+      </x:c>
+      <x:c r="H25" s="613" t="n">
+        <x:f>F25/G25</x:f>
+        <x:v>3.9092088603532766</x:v>
+      </x:c>
+      <x:c r="I25" s="568" t="n">
+        <x:f>H25/($D$15/Forecast!$B$106)-1</x:f>
+        <x:v>-0.1617114304764219</x:v>
+      </x:c>
+      <x:c r="J25" s="321"/>
+      <x:c r="K25" s="321"/>
+      <x:c r="L25" s="321"/>
+      <x:c r="M25" s="321"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="370" t="str">
+        <x:v>EV / operating profit</x:v>
+      </x:c>
+      <x:c r="B26" s="569" t="n">
+        <x:f>$C$20</x:f>
+        <x:v>13.414216754804936</x:v>
+      </x:c>
+      <x:c r="C26" s="488" t="n">
+        <x:f>$J$15</x:f>
+        <x:v>217.9</x:v>
+      </x:c>
+      <x:c r="D26" s="488" t="n">
+        <x:f>B26*C26</x:f>
+        <x:v>2922.9578308719956</x:v>
+      </x:c>
+      <x:c r="E26" s="488" t="n">
+        <x:f>$G$15</x:f>
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="F26" s="488" t="n">
+        <x:f>D26-E26</x:f>
+        <x:v>2763.8578308719957</x:v>
+      </x:c>
+      <x:c r="G26" s="488" t="n">
+        <x:f>Forecast!$B$106</x:f>
+        <x:v>522.1</x:v>
+      </x:c>
+      <x:c r="H26" s="614" t="n">
+        <x:f>F26/G26</x:f>
+        <x:v>5.2937326774027875</x:v>
+      </x:c>
+      <x:c r="I26" s="571" t="n">
+        <x:f>H26/($D$15/Forecast!$B$106)-1</x:f>
+        <x:v>0.13518508529604878</x:v>
+      </x:c>
+      <x:c r="J26" s="321"/>
+      <x:c r="K26" s="321"/>
+      <x:c r="L26" s="321"/>
+      <x:c r="M26" s="321"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="321"/>
+      <x:c r="B27" s="321"/>
+      <x:c r="C27" s="321"/>
+      <x:c r="D27" s="321"/>
+      <x:c r="E27" s="321"/>
+      <x:c r="F27" s="321"/>
+      <x:c r="G27" s="321"/>
+      <x:c r="H27" s="321"/>
+      <x:c r="I27" s="321"/>
+      <x:c r="J27" s="321"/>
+      <x:c r="K27" s="321"/>
+      <x:c r="L27" s="321"/>
+      <x:c r="M27" s="321"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="321"/>
+      <x:c r="B28" s="321"/>
+      <x:c r="C28" s="321"/>
+      <x:c r="D28" s="321"/>
+      <x:c r="E28" s="321"/>
+      <x:c r="F28" s="321"/>
+      <x:c r="G28" s="321"/>
+      <x:c r="H28" s="321"/>
+      <x:c r="I28" s="321"/>
+      <x:c r="J28" s="321"/>
+      <x:c r="K28" s="321"/>
+      <x:c r="L28" s="321"/>
+      <x:c r="M28" s="321"/>
+    </x:row>
+    <x:row r="29" ht="23" customHeight="1">
+      <x:c r="A29" s="557" t="str">
+        <x:v>Valuation cross-check (£ per share)</x:v>
+      </x:c>
+      <x:c r="B29" s="557"/>
+      <x:c r="C29" s="557"/>
+      <x:c r="D29" s="557"/>
+      <x:c r="E29" s="557"/>
+      <x:c r="F29" s="321"/>
+      <x:c r="G29" s="321"/>
+      <x:c r="H29" s="321"/>
+      <x:c r="I29" s="321"/>
+      <x:c r="J29" s="321"/>
+      <x:c r="K29" s="321"/>
+      <x:c r="L29" s="321"/>
+      <x:c r="M29" s="321"/>
+    </x:row>
+    <x:row r="30" ht="31" customHeight="1">
+      <x:c r="A30" s="534" t="str">
+        <x:v>Current price</x:v>
+      </x:c>
+      <x:c r="B30" s="534" t="str">
+        <x:v>Trading: revenue</x:v>
+      </x:c>
+      <x:c r="C30" s="534" t="str">
+        <x:v>Trading: op. profit</x:v>
+      </x:c>
+      <x:c r="D30" s="534" t="str">
+        <x:v>Base DCF</x:v>
+      </x:c>
+      <x:c r="E30" s="534" t="str">
+        <x:v>Restructuring DCF</x:v>
+      </x:c>
+      <x:c r="F30" s="321"/>
+      <x:c r="G30" s="321"/>
+      <x:c r="H30" s="321"/>
+      <x:c r="I30" s="321"/>
+      <x:c r="J30" s="321"/>
+      <x:c r="K30" s="321"/>
+      <x:c r="L30" s="321"/>
+      <x:c r="M30" s="321"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="615" t="n">
+        <x:f>$D$15/Forecast!$B$106</x:f>
+        <x:v>4.663321202834705</x:v>
+      </x:c>
+      <x:c r="B31" s="615" t="n">
+        <x:f>$H$25</x:f>
+        <x:v>3.9092088603532766</x:v>
+      </x:c>
+      <x:c r="C31" s="615" t="n">
+        <x:f>$H$26</x:f>
+        <x:v>5.2937326774027875</x:v>
+      </x:c>
+      <x:c r="D31" s="615" t="n">
+        <x:f>Forecast!$B$107</x:f>
+        <x:v>5.5089682185956175</x:v>
+      </x:c>
+      <x:c r="E31" s="615" t="n">
+        <x:f>Forecast!$B$173</x:f>
+        <x:v>5.519558386657466</x:v>
+      </x:c>
+      <x:c r="F31" s="321"/>
+      <x:c r="G31" s="321"/>
+      <x:c r="H31" s="321"/>
+      <x:c r="I31" s="321"/>
+      <x:c r="J31" s="321"/>
+      <x:c r="K31" s="321"/>
+      <x:c r="L31" s="321"/>
+      <x:c r="M31" s="321"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="321"/>
+      <x:c r="B32" s="321"/>
+      <x:c r="C32" s="321"/>
+      <x:c r="D32" s="321"/>
+      <x:c r="E32" s="321"/>
+      <x:c r="F32" s="321"/>
+      <x:c r="G32" s="321"/>
+      <x:c r="H32" s="321"/>
+      <x:c r="I32" s="321"/>
+      <x:c r="J32" s="321"/>
+      <x:c r="K32" s="321"/>
+      <x:c r="L32" s="321"/>
+      <x:c r="M32" s="321"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="321"/>
+      <x:c r="B33" s="321"/>
+      <x:c r="C33" s="321"/>
+      <x:c r="D33" s="321"/>
+      <x:c r="E33" s="321"/>
+      <x:c r="F33" s="321"/>
+      <x:c r="G33" s="321"/>
+      <x:c r="H33" s="321"/>
+      <x:c r="I33" s="321"/>
+      <x:c r="J33" s="321"/>
+      <x:c r="K33" s="321"/>
+      <x:c r="L33" s="321"/>
+      <x:c r="M33" s="321"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="528" t="str">
+        <x:v>Interpretation: the 1.14x revenue median implies £3.91 per share, while the 13.41x operating-profit median implies £5.29. QinetiQ's higher margin makes the operating-profit method the more meaningful trading cross-check; it is below but close to the £5.51 base DCF. Babcock uses normalised underlying profit before the one-off Type 31 charge; UK peers otherwise use underlying/adjusted profit and US peers use GAAP operating income.</x:v>
+      </x:c>
+      <x:c r="B34" s="528"/>
+      <x:c r="C34" s="528"/>
+      <x:c r="D34" s="528"/>
+      <x:c r="E34" s="528"/>
+      <x:c r="F34" s="528"/>
+      <x:c r="G34" s="528"/>
+      <x:c r="H34" s="528"/>
+      <x:c r="I34" s="528"/>
+      <x:c r="J34" s="528"/>
+      <x:c r="K34" s="528"/>
+      <x:c r="L34" s="528"/>
+      <x:c r="M34" s="528"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="528"/>
+      <x:c r="B35" s="528"/>
+      <x:c r="C35" s="528"/>
+      <x:c r="D35" s="528"/>
+      <x:c r="E35" s="528"/>
+      <x:c r="F35" s="528"/>
+      <x:c r="G35" s="528"/>
+      <x:c r="H35" s="528"/>
+      <x:c r="I35" s="528"/>
+      <x:c r="J35" s="528"/>
+      <x:c r="K35" s="528"/>
+      <x:c r="L35" s="528"/>
+      <x:c r="M35" s="528"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:M1"/>
+    <x:mergeCell ref="A2:M3"/>
+    <x:mergeCell ref="A17:F17"/>
+    <x:mergeCell ref="A23:I23"/>
+    <x:mergeCell ref="A29:E29"/>
+    <x:mergeCell ref="A34:M35"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="45" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="23" customHeight="1">
+      <x:c r="A1" s="557" t="str">
+        <x:v>QinetiQ precedent transactions</x:v>
+      </x:c>
+      <x:c r="B1" s="557"/>
+      <x:c r="C1" s="557"/>
+      <x:c r="D1" s="557"/>
+      <x:c r="E1" s="557"/>
+      <x:c r="F1" s="557"/>
+      <x:c r="G1" s="557"/>
+      <x:c r="H1" s="557"/>
+      <x:c r="I1" s="557"/>
+      <x:c r="J1" s="557"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="528" t="str">
+        <x:v>Purpose: test the US-disposal sale multiple against prices paid for control of comparable defence, intelligence and government-technology assets. Precedent prices include control premiums and expected synergies, so the output is an upside reference and negotiation range rather than an automatic base-case assumption.</x:v>
+      </x:c>
+      <x:c r="B2" s="528"/>
+      <x:c r="C2" s="528"/>
+      <x:c r="D2" s="528"/>
+      <x:c r="E2" s="528"/>
+      <x:c r="F2" s="528"/>
+      <x:c r="G2" s="528"/>
+      <x:c r="H2" s="528"/>
+      <x:c r="I2" s="528"/>
+      <x:c r="J2" s="528"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="528"/>
+      <x:c r="B3" s="528"/>
+      <x:c r="C3" s="528"/>
+      <x:c r="D3" s="528"/>
+      <x:c r="E3" s="528"/>
+      <x:c r="F3" s="528"/>
+      <x:c r="G3" s="528"/>
+      <x:c r="H3" s="528"/>
+      <x:c r="I3" s="528"/>
+      <x:c r="J3" s="528"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="321"/>
+      <x:c r="B4" s="321"/>
+      <x:c r="C4" s="321"/>
+      <x:c r="D4" s="321"/>
+      <x:c r="E4" s="321"/>
+      <x:c r="F4" s="321"/>
+      <x:c r="G4" s="321"/>
+      <x:c r="H4" s="321"/>
+      <x:c r="I4" s="321"/>
+      <x:c r="J4" s="321"/>
+    </x:row>
+    <x:row r="5" ht="31" customHeight="1">
+      <x:c r="A5" s="534" t="str">
+        <x:v>Target</x:v>
+      </x:c>
+      <x:c r="B5" s="534" t="str">
+        <x:v>Acquirer</x:v>
+      </x:c>
+      <x:c r="C5" s="534" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="D5" s="534" t="str">
+        <x:v>Enterprise value ($m)</x:v>
+      </x:c>
+      <x:c r="E5" s="534" t="str">
+        <x:v>Revenue ($m)</x:v>
+      </x:c>
+      <x:c r="F5" s="534" t="str">
+        <x:v>EBITDA ($m)</x:v>
+      </x:c>
+      <x:c r="G5" s="534" t="str">
+        <x:v>EV / revenue</x:v>
+      </x:c>
+      <x:c r="H5" s="534" t="str">
+        <x:v>EV / EBITDA</x:v>
+      </x:c>
+      <x:c r="I5" s="534" t="str">
+        <x:v>Reported multiple</x:v>
+      </x:c>
+      <x:c r="J5" s="534" t="str">
+        <x:v>Relevance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="573" t="str">
+        <x:v>Avantus Federal</x:v>
+      </x:c>
+      <x:c r="B6" s="573" t="str">
+        <x:v>QinetiQ</x:v>
+      </x:c>
+      <x:c r="C6" s="573" t="str">
+        <x:v>Aug-2022</x:v>
+      </x:c>
+      <x:c r="D6" s="469" t="n">
+        <x:v>590</x:v>
+      </x:c>
+      <x:c r="E6" s="469" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="F6" s="469" t="n">
+        <x:v>35.5</x:v>
+      </x:c>
+      <x:c r="G6" s="566" t="n">
+        <x:f>D6/E6</x:f>
+        <x:v>1.9798657718120805</x:v>
+      </x:c>
+      <x:c r="H6" s="566" t="n">
+        <x:f>D6/F6</x:f>
+        <x:v>16.619718309859156</x:v>
+      </x:c>
+      <x:c r="I6" s="473"/>
+      <x:c r="J6" s="612" t="str">
+        <x:v>Direct QinetiQ US cyber / intelligence deal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="573" t="str">
+        <x:v>Dynetics</x:v>
+      </x:c>
+      <x:c r="B7" s="573" t="str">
+        <x:v>Leidos</x:v>
+      </x:c>
+      <x:c r="C7" s="573" t="str">
+        <x:v>Dec-2019</x:v>
+      </x:c>
+      <x:c r="D7" s="469" t="n">
+        <x:v>1650</x:v>
+      </x:c>
+      <x:c r="E7" s="469" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="F7" s="469"/>
+      <x:c r="G7" s="566" t="n">
+        <x:f>D7/E7</x:f>
+        <x:v>1.65</x:v>
+      </x:c>
+      <x:c r="H7" s="566"/>
+      <x:c r="I7" s="473"/>
+      <x:c r="J7" s="612" t="str">
+        <x:v>Defence technology, space and engineering</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="573" t="str">
+        <x:v>Azure Summit Technology</x:v>
+      </x:c>
+      <x:c r="B8" s="573" t="str">
+        <x:v>CACI</x:v>
+      </x:c>
+      <x:c r="C8" s="573" t="str">
+        <x:v>Sep-2024</x:v>
+      </x:c>
+      <x:c r="D8" s="469" t="n">
+        <x:v>1275</x:v>
+      </x:c>
+      <x:c r="E8" s="469" t="n">
+        <x:v>440</x:v>
+      </x:c>
+      <x:c r="F8" s="469" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="G8" s="566" t="n">
+        <x:f>D8/E8</x:f>
+        <x:v>2.897727272727273</x:v>
+      </x:c>
+      <x:c r="H8" s="566" t="n">
+        <x:f>D8/F8</x:f>
+        <x:v>11.590909090909092</x:v>
+      </x:c>
+      <x:c r="I8" s="473"/>
+      <x:c r="J8" s="612" t="str">
+        <x:v>Higher-growth RF / electronic-warfare technology</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="573" t="str">
+        <x:v>LinQuest</x:v>
+      </x:c>
+      <x:c r="B9" s="573" t="str">
+        <x:v>KBR</x:v>
+      </x:c>
+      <x:c r="C9" s="573" t="str">
+        <x:v>Jul-2024</x:v>
+      </x:c>
+      <x:c r="D9" s="469" t="n">
+        <x:v>737</x:v>
+      </x:c>
+      <x:c r="E9" s="469"/>
+      <x:c r="F9" s="469"/>
+      <x:c r="G9" s="566"/>
+      <x:c r="H9" s="566"/>
+      <x:c r="I9" s="473" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="J9" s="612" t="str">
+        <x:v>National-security space and digital integration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="573" t="str">
+        <x:v>PAE</x:v>
+      </x:c>
+      <x:c r="B10" s="573" t="str">
+        <x:v>Amentum</x:v>
+      </x:c>
+      <x:c r="C10" s="573" t="str">
+        <x:v>Oct-2021</x:v>
+      </x:c>
+      <x:c r="D10" s="469" t="n">
+        <x:v>1900</x:v>
+      </x:c>
+      <x:c r="E10" s="469" t="n">
+        <x:v>2714.628</x:v>
+      </x:c>
+      <x:c r="F10" s="469"/>
+      <x:c r="G10" s="566" t="n">
+        <x:f>D10/E10</x:f>
+        <x:v>0.699911737446162</x:v>
+      </x:c>
+      <x:c r="H10" s="566"/>
+      <x:c r="I10" s="473"/>
+      <x:c r="J10" s="612" t="str">
+        <x:v>Lower-margin government-services reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="366"/>
+      <x:c r="B11" s="366"/>
+      <x:c r="C11" s="366"/>
+      <x:c r="D11" s="366"/>
+      <x:c r="E11" s="366"/>
+      <x:c r="F11" s="366"/>
+      <x:c r="G11" s="566"/>
+      <x:c r="H11" s="566"/>
+      <x:c r="I11" s="566"/>
+      <x:c r="J11" s="366"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="600" t="str">
+        <x:v>Median of disclosed EV / revenue multiples</x:v>
+      </x:c>
+      <x:c r="B12" s="600"/>
+      <x:c r="C12" s="600"/>
+      <x:c r="D12" s="600"/>
+      <x:c r="E12" s="600"/>
+      <x:c r="F12" s="600"/>
+      <x:c r="G12" s="601" t="n">
+        <x:f>MEDIAN(G6:G10)</x:f>
+        <x:v>1.8149328859060403</x:v>
+      </x:c>
+      <x:c r="H12" s="569"/>
+      <x:c r="I12" s="569"/>
+      <x:c r="J12" s="370"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="321"/>
+      <x:c r="B13" s="321"/>
+      <x:c r="C13" s="321"/>
+      <x:c r="D13" s="321"/>
+      <x:c r="E13" s="321"/>
+      <x:c r="F13" s="321"/>
+      <x:c r="G13" s="321"/>
+      <x:c r="H13" s="321"/>
+      <x:c r="I13" s="321"/>
+      <x:c r="J13" s="321"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="321"/>
+      <x:c r="B14" s="321"/>
+      <x:c r="C14" s="321"/>
+      <x:c r="D14" s="321"/>
+      <x:c r="E14" s="321"/>
+      <x:c r="F14" s="321"/>
+      <x:c r="G14" s="321"/>
+      <x:c r="H14" s="321"/>
+      <x:c r="I14" s="321"/>
+      <x:c r="J14" s="321"/>
+    </x:row>
+    <x:row r="15" ht="23" customHeight="1">
+      <x:c r="A15" s="557" t="str">
+        <x:v>US-disposal implication</x:v>
+      </x:c>
+      <x:c r="B15" s="557"/>
+      <x:c r="C15" s="557"/>
+      <x:c r="D15" s="321"/>
+      <x:c r="E15" s="321"/>
+      <x:c r="F15" s="321"/>
+      <x:c r="G15" s="321"/>
+      <x:c r="H15" s="321"/>
+      <x:c r="I15" s="321"/>
+      <x:c r="J15" s="321"/>
+    </x:row>
+    <x:row r="16" ht="31" customHeight="1">
+      <x:c r="A16" s="534" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B16" s="534" t="str">
+        <x:v>Existing disposal case</x:v>
+      </x:c>
+      <x:c r="C16" s="534" t="str">
+        <x:v>Precedent-median reference</x:v>
+      </x:c>
+      <x:c r="D16" s="321"/>
+      <x:c r="E16" s="321"/>
+      <x:c r="F16" s="321"/>
+      <x:c r="G16" s="321"/>
+      <x:c r="H16" s="321"/>
+      <x:c r="I16" s="321"/>
+      <x:c r="J16" s="321"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="366" t="str">
+        <x:v>Sale EV / revenue</x:v>
+      </x:c>
+      <x:c r="B17" s="602" t="n">
+        <x:f>Forecast!$B$199</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" s="603" t="n">
+        <x:f>$G$12</x:f>
+        <x:v>1.8149328859060403</x:v>
+      </x:c>
+      <x:c r="D17" s="321"/>
+      <x:c r="E17" s="321"/>
+      <x:c r="F17" s="321"/>
+      <x:c r="G17" s="321"/>
+      <x:c r="H17" s="321"/>
+      <x:c r="I17" s="321"/>
+      <x:c r="J17" s="321"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="366" t="str">
+        <x:v>FY26 US revenue (£m)</x:v>
+      </x:c>
+      <x:c r="B18" s="604" t="n">
+        <x:f>Forecast!$B$193</x:f>
+        <x:v>290.7</x:v>
+      </x:c>
+      <x:c r="C18" s="605" t="n">
+        <x:f>B18</x:f>
+        <x:v>290.7</x:v>
+      </x:c>
+      <x:c r="D18" s="321"/>
+      <x:c r="E18" s="321"/>
+      <x:c r="F18" s="321"/>
+      <x:c r="G18" s="321"/>
+      <x:c r="H18" s="321"/>
+      <x:c r="I18" s="321"/>
+      <x:c r="J18" s="321"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="366" t="str">
+        <x:v>Gross proceeds (£m)</x:v>
+      </x:c>
+      <x:c r="B19" s="604" t="n">
+        <x:f>B17*B18</x:f>
+        <x:v>290.7</x:v>
+      </x:c>
+      <x:c r="C19" s="605" t="n">
+        <x:f>C17*C18</x:f>
+        <x:v>527.6009899328859</x:v>
+      </x:c>
+      <x:c r="D19" s="321"/>
+      <x:c r="E19" s="321"/>
+      <x:c r="F19" s="321"/>
+      <x:c r="G19" s="321"/>
+      <x:c r="H19" s="321"/>
+      <x:c r="I19" s="321"/>
+      <x:c r="J19" s="321"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="366" t="str">
+        <x:v>Proceeds leakage</x:v>
+      </x:c>
+      <x:c r="B20" s="606" t="n">
+        <x:f>Forecast!$B$201</x:f>
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C20" s="607" t="n">
+        <x:f>B20</x:f>
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D20" s="321"/>
+      <x:c r="E20" s="321"/>
+      <x:c r="F20" s="321"/>
+      <x:c r="G20" s="321"/>
+      <x:c r="H20" s="321"/>
+      <x:c r="I20" s="321"/>
+      <x:c r="J20" s="321"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="366" t="str">
+        <x:v>Net proceeds (£m)</x:v>
+      </x:c>
+      <x:c r="B21" s="604" t="n">
+        <x:f>B19*(1-B20)</x:f>
+        <x:v>261.63</x:v>
+      </x:c>
+      <x:c r="C21" s="605" t="n">
+        <x:f>C19*(1-C20)</x:f>
+        <x:v>474.84089093959733</x:v>
+      </x:c>
+      <x:c r="D21" s="321"/>
+      <x:c r="E21" s="321"/>
+      <x:c r="F21" s="321"/>
+      <x:c r="G21" s="321"/>
+      <x:c r="H21" s="321"/>
+      <x:c r="I21" s="321"/>
+      <x:c r="J21" s="321"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="366" t="str">
+        <x:v>Retained-business EV (£m)</x:v>
+      </x:c>
+      <x:c r="B22" s="604" t="n">
+        <x:f>Forecast!$B$249</x:f>
+        <x:v>2739.112270378971</x:v>
+      </x:c>
+      <x:c r="C22" s="605" t="n">
+        <x:f>B22</x:f>
+        <x:v>2739.112270378971</x:v>
+      </x:c>
+      <x:c r="D22" s="321"/>
+      <x:c r="E22" s="321"/>
+      <x:c r="F22" s="321"/>
+      <x:c r="G22" s="321"/>
+      <x:c r="H22" s="321"/>
+      <x:c r="I22" s="321"/>
+      <x:c r="J22" s="321"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="366" t="str">
+        <x:v>Less: group net debt (£m)</x:v>
+      </x:c>
+      <x:c r="B23" s="604" t="n">
+        <x:f>Forecast!$B$104</x:f>
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="C23" s="605" t="n">
+        <x:f>B23</x:f>
+        <x:v>159.1</x:v>
+      </x:c>
+      <x:c r="D23" s="321"/>
+      <x:c r="E23" s="321"/>
+      <x:c r="F23" s="321"/>
+      <x:c r="G23" s="321"/>
+      <x:c r="H23" s="321"/>
+      <x:c r="I23" s="321"/>
+      <x:c r="J23" s="321"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="366" t="str">
+        <x:v>Equity value (£m)</x:v>
+      </x:c>
+      <x:c r="B24" s="604" t="n">
+        <x:f>B22+B21-B23</x:f>
+        <x:v>2841.6422703789713</x:v>
+      </x:c>
+      <x:c r="C24" s="605" t="n">
+        <x:f>C22+C21-C23</x:f>
+        <x:v>3054.8531613185683</x:v>
+      </x:c>
+      <x:c r="D24" s="321"/>
+      <x:c r="E24" s="321"/>
+      <x:c r="F24" s="321"/>
+      <x:c r="G24" s="321"/>
+      <x:c r="H24" s="321"/>
+      <x:c r="I24" s="321"/>
+      <x:c r="J24" s="321"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="366" t="str">
+        <x:v>Diluted shares (m)</x:v>
+      </x:c>
+      <x:c r="B25" s="604" t="n">
+        <x:f>Forecast!$B$106</x:f>
+        <x:v>522.1</x:v>
+      </x:c>
+      <x:c r="C25" s="605" t="n">
+        <x:f>B25</x:f>
+        <x:v>522.1</x:v>
+      </x:c>
+      <x:c r="D25" s="321"/>
+      <x:c r="E25" s="321"/>
+      <x:c r="F25" s="321"/>
+      <x:c r="G25" s="321"/>
+      <x:c r="H25" s="321"/>
+      <x:c r="I25" s="321"/>
+      <x:c r="J25" s="321"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="608" t="str">
+        <x:v>Implied value / share (£)</x:v>
+      </x:c>
+      <x:c r="B26" s="616" t="n">
+        <x:f>B24/B25</x:f>
+        <x:v>5.442716472666101</x:v>
+      </x:c>
+      <x:c r="C26" s="613" t="n">
+        <x:f>C24/C25</x:f>
+        <x:v>5.851088223172894</x:v>
+      </x:c>
+      <x:c r="D26" s="321"/>
+      <x:c r="E26" s="321"/>
+      <x:c r="F26" s="321"/>
+      <x:c r="G26" s="321"/>
+      <x:c r="H26" s="321"/>
+      <x:c r="I26" s="321"/>
+      <x:c r="J26" s="321"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="608" t="str">
+        <x:v>Difference vs base DCF (£/share)</x:v>
+      </x:c>
+      <x:c r="B27" s="616" t="n">
+        <x:f>B26-Forecast!$B$107</x:f>
+        <x:v>-0.06625174592951666</x:v>
+      </x:c>
+      <x:c r="C27" s="613" t="n">
+        <x:f>C26-Forecast!$B$107</x:f>
+        <x:v>0.34212000457727676</x:v>
+      </x:c>
+      <x:c r="D27" s="321"/>
+      <x:c r="E27" s="321"/>
+      <x:c r="F27" s="321"/>
+      <x:c r="G27" s="321"/>
+      <x:c r="H27" s="321"/>
+      <x:c r="I27" s="321"/>
+      <x:c r="J27" s="321"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="370" t="str">
+        <x:v>Break-even sale multiple</x:v>
+      </x:c>
+      <x:c r="B28" s="610" t="n">
+        <x:f>Forecast!$B$203</x:f>
+        <x:v>1.1322097486901377</x:v>
+      </x:c>
+      <x:c r="C28" s="611" t="n">
+        <x:f>B28</x:f>
+        <x:v>1.1322097486901377</x:v>
+      </x:c>
+      <x:c r="D28" s="321"/>
+      <x:c r="E28" s="321"/>
+      <x:c r="F28" s="321"/>
+      <x:c r="G28" s="321"/>
+      <x:c r="H28" s="321"/>
+      <x:c r="I28" s="321"/>
+      <x:c r="J28" s="321"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="321"/>
+      <x:c r="B29" s="321"/>
+      <x:c r="C29" s="321"/>
+      <x:c r="D29" s="321"/>
+      <x:c r="E29" s="321"/>
+      <x:c r="F29" s="321"/>
+      <x:c r="G29" s="321"/>
+      <x:c r="H29" s="321"/>
+      <x:c r="I29" s="321"/>
+      <x:c r="J29" s="321"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="321"/>
+      <x:c r="B30" s="321"/>
+      <x:c r="C30" s="321"/>
+      <x:c r="D30" s="321"/>
+      <x:c r="E30" s="321"/>
+      <x:c r="F30" s="321"/>
+      <x:c r="G30" s="321"/>
+      <x:c r="H30" s="321"/>
+      <x:c r="I30" s="321"/>
+      <x:c r="J30" s="321"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="528" t="str">
+        <x:v>Interpretation: disclosed transaction multiples have a 1.81x revenue median, compared with the model's 1.00x assumption and approximately 1.13x break-even price. At the median, the disposal case would imply about £5.85 per share. The median is not adopted as the base case because Avantus and Azure Summit had stronger growth, differentiated technology and strategic scarcity, while all precedent prices may include control and synergy value. The evidence shows that 1.00x is conservative and that a sale becomes value-creating above roughly 1.13x after the 10% proceeds allowance.</x:v>
+      </x:c>
+      <x:c r="B31" s="528"/>
+      <x:c r="C31" s="528"/>
+      <x:c r="D31" s="528"/>
+      <x:c r="E31" s="528"/>
+      <x:c r="F31" s="528"/>
+      <x:c r="G31" s="528"/>
+      <x:c r="H31" s="528"/>
+      <x:c r="I31" s="528"/>
+      <x:c r="J31" s="528"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="528"/>
+      <x:c r="B32" s="528"/>
+      <x:c r="C32" s="528"/>
+      <x:c r="D32" s="528"/>
+      <x:c r="E32" s="528"/>
+      <x:c r="F32" s="528"/>
+      <x:c r="G32" s="528"/>
+      <x:c r="H32" s="528"/>
+      <x:c r="I32" s="528"/>
+      <x:c r="J32" s="528"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="528"/>
+      <x:c r="B33" s="528"/>
+      <x:c r="C33" s="528"/>
+      <x:c r="D33" s="528"/>
+      <x:c r="E33" s="528"/>
+      <x:c r="F33" s="528"/>
+      <x:c r="G33" s="528"/>
+      <x:c r="H33" s="528"/>
+      <x:c r="I33" s="528"/>
+      <x:c r="J33" s="528"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J3"/>
+    <x:mergeCell ref="A12:F12"/>
+    <x:mergeCell ref="A15:C15"/>
+    <x:mergeCell ref="A31:J33"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add final valuation synthesis and recommendation
</commit_message>
<xml_diff>
--- a/model/QinetiQ_Valuation_Model.xlsx
+++ b/model/QinetiQ_Valuation_Model.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R864877b2e1ea4973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="Ra785ac3e09a547bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="R12e7e3ba42c24885"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="R6dddc7574af34fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R35651bbadb6f4be7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="Rdc47e0d8d3ab4457"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="7" r:id="R83a5855761034028"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedents" sheetId="8" r:id="Ra09e5cb618034833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Re151fe722fd642ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Summary" sheetId="2" r:id="R1477f7ec3af84079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments" sheetId="3" r:id="R447788eddd354bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statements" sheetId="4" r:id="Rc96e2bdd590b44a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="Rf7537ce27c754283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="6" r:id="Re27600e50b5940d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading Comps" sheetId="7" r:id="Rbffaaa56d37148b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedents" sheetId="8" r:id="R310d49c5576d4386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="9" r:id="Rfe3713f3052344a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -902,7 +903,7 @@
     <x:numFmt numFmtId="210" formatCode="0.000x"/>
     <x:numFmt numFmtId="211" formatCode="£0.00;[Red](£0.00);-"/>
   </x:numFmts>
-  <x:fonts count="34">
+  <x:fonts count="35">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -1093,8 +1094,13 @@
       <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="2"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="51">
+  <x:fills count="57">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1346,6 +1352,36 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="22">
     <x:border diagonalUp="0" diagonalDown="0"/>
@@ -1544,7 +1580,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="617">
+  <x:cellXfs count="683">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -3394,6 +3430,204 @@
       <x:alignment horizontal="general" vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="209" fontId="27" fillId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="52" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="53" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="53" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="27" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="34" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="54" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="25" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="171" fontId="27" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="34" fillId="55" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="27" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="26" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="54" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="26" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -3467,6 +3701,178 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:t>Implied value per share (£)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Value / share</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Valuation Summary'!$H$17:$H$22</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Valuation Summary'!$I$17:$I$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="600">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="675">
+                <a:latin typeface="Arial"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8e898de52fe2410a"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3922,7 +4328,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="1" t="str">
-        <x:v>0.8</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
@@ -3986,7 +4392,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="D12" s="1" t="str">
-        <x:v>Trading comparables and precedent transactions complete</x:v>
+        <x:v>Final valuation synthesis and strategic recommendation complete</x:v>
       </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
@@ -24132,7 +24538,7 @@
     <x:mergeCell ref="A282:F282"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4c1e2ae604b4960"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6f9450f46424572"/>
 </x:worksheet>
 </file>
 
@@ -25774,4 +26180,1068 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="3" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="23" customHeight="1">
+      <x:c r="A1" s="660" t="str">
+        <x:v>QinetiQ valuation summary and strategic recommendation</x:v>
+      </x:c>
+      <x:c r="B1" s="660"/>
+      <x:c r="C1" s="660"/>
+      <x:c r="D1" s="660"/>
+      <x:c r="E1" s="660"/>
+      <x:c r="F1" s="660"/>
+      <x:c r="G1" s="660"/>
+      <x:c r="H1" s="660"/>
+      <x:c r="I1" s="660"/>
+      <x:c r="J1" s="660"/>
+      <x:c r="K1" s="660"/>
+      <x:c r="L1" s="660"/>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="622" t="str">
+        <x:v>The core valuation uses the operating-profit trading comparable and the two retain-case DCFs. Precedent transactions are used only to assess conditional US sale upside. Research date: 16 September 2026.</x:v>
+      </x:c>
+      <x:c r="B2" s="622"/>
+      <x:c r="C2" s="622"/>
+      <x:c r="D2" s="622"/>
+      <x:c r="E2" s="622"/>
+      <x:c r="F2" s="622"/>
+      <x:c r="G2" s="622"/>
+      <x:c r="H2" s="622"/>
+      <x:c r="I2" s="622"/>
+      <x:c r="J2" s="622"/>
+      <x:c r="K2" s="622"/>
+      <x:c r="L2" s="622"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="622"/>
+      <x:c r="B3" s="622"/>
+      <x:c r="C3" s="622"/>
+      <x:c r="D3" s="622"/>
+      <x:c r="E3" s="622"/>
+      <x:c r="F3" s="622"/>
+      <x:c r="G3" s="622"/>
+      <x:c r="H3" s="622"/>
+      <x:c r="I3" s="622"/>
+      <x:c r="J3" s="622"/>
+      <x:c r="K3" s="622"/>
+      <x:c r="L3" s="622"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="321"/>
+      <x:c r="B4" s="321"/>
+      <x:c r="C4" s="321"/>
+      <x:c r="D4" s="321"/>
+      <x:c r="E4" s="321"/>
+      <x:c r="F4" s="321"/>
+      <x:c r="G4" s="321"/>
+      <x:c r="H4" s="321"/>
+      <x:c r="I4" s="321"/>
+      <x:c r="J4" s="321"/>
+      <x:c r="K4" s="321"/>
+      <x:c r="L4" s="321"/>
+    </x:row>
+    <x:row r="5" ht="23" customHeight="1">
+      <x:c r="A5" s="660" t="str">
+        <x:v>Valuation conclusion</x:v>
+      </x:c>
+      <x:c r="B5" s="660"/>
+      <x:c r="C5" s="660"/>
+      <x:c r="D5" s="660"/>
+      <x:c r="E5" s="660"/>
+      <x:c r="F5" s="660"/>
+      <x:c r="G5" s="321"/>
+      <x:c r="H5" s="321"/>
+      <x:c r="I5" s="321"/>
+      <x:c r="J5" s="321"/>
+      <x:c r="K5" s="321"/>
+      <x:c r="L5" s="321"/>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="628" t="str">
+        <x:v>Metric</x:v>
+      </x:c>
+      <x:c r="B6" s="628" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C6" s="628" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+      <x:c r="D6" s="321"/>
+      <x:c r="E6" s="321"/>
+      <x:c r="F6" s="321"/>
+      <x:c r="G6" s="321"/>
+      <x:c r="H6" s="321"/>
+      <x:c r="I6" s="321"/>
+      <x:c r="J6" s="321"/>
+      <x:c r="K6" s="321"/>
+      <x:c r="L6" s="321"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="366" t="str">
+        <x:v>Current share price</x:v>
+      </x:c>
+      <x:c r="B7" s="661" t="n">
+        <x:f>'Trading Comps'!A31</x:f>
+        <x:v>4.663321202834705</x:v>
+      </x:c>
+      <x:c r="C7" s="366" t="str">
+        <x:v>Research-date market price</x:v>
+      </x:c>
+      <x:c r="D7" s="321"/>
+      <x:c r="E7" s="321"/>
+      <x:c r="F7" s="321"/>
+      <x:c r="G7" s="321"/>
+      <x:c r="H7" s="321"/>
+      <x:c r="I7" s="321"/>
+      <x:c r="J7" s="321"/>
+      <x:c r="K7" s="321"/>
+      <x:c r="L7" s="321"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="366" t="str">
+        <x:v>Core valuation low</x:v>
+      </x:c>
+      <x:c r="B8" s="661" t="n">
+        <x:f>MIN('Trading Comps'!H26,Forecast!B107,Forecast!B173)</x:f>
+        <x:v>5.2937326774027875</x:v>
+      </x:c>
+      <x:c r="C8" s="366" t="str">
+        <x:v>Operating-profit trading value</x:v>
+      </x:c>
+      <x:c r="D8" s="321"/>
+      <x:c r="E8" s="321"/>
+      <x:c r="F8" s="321"/>
+      <x:c r="G8" s="321"/>
+      <x:c r="H8" s="321"/>
+      <x:c r="I8" s="321"/>
+      <x:c r="J8" s="321"/>
+      <x:c r="K8" s="321"/>
+      <x:c r="L8" s="321"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="366" t="str">
+        <x:v>Core valuation high</x:v>
+      </x:c>
+      <x:c r="B9" s="661" t="n">
+        <x:f>MAX('Trading Comps'!H26,Forecast!B107,Forecast!B173)</x:f>
+        <x:v>5.519558386657466</x:v>
+      </x:c>
+      <x:c r="C9" s="366" t="str">
+        <x:v>Highest retain-case DCF</x:v>
+      </x:c>
+      <x:c r="D9" s="321"/>
+      <x:c r="E9" s="321"/>
+      <x:c r="F9" s="321"/>
+      <x:c r="G9" s="321"/>
+      <x:c r="H9" s="321"/>
+      <x:c r="I9" s="321"/>
+      <x:c r="J9" s="321"/>
+      <x:c r="K9" s="321"/>
+      <x:c r="L9" s="321"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="662" t="str">
+        <x:v>Illustrative central value</x:v>
+      </x:c>
+      <x:c r="B10" s="663" t="n">
+        <x:f>SUM(E17:E22)</x:f>
+        <x:v>5.403997990014664</x:v>
+      </x:c>
+      <x:c r="C10" s="662" t="str">
+        <x:v>50% EBIT comps; 25% base DCF; 25% restructuring DCF</x:v>
+      </x:c>
+      <x:c r="D10" s="321"/>
+      <x:c r="E10" s="321"/>
+      <x:c r="F10" s="321"/>
+      <x:c r="G10" s="321"/>
+      <x:c r="H10" s="321"/>
+      <x:c r="I10" s="321"/>
+      <x:c r="J10" s="321"/>
+      <x:c r="K10" s="321"/>
+      <x:c r="L10" s="321"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="662" t="str">
+        <x:v>Central-value upside</x:v>
+      </x:c>
+      <x:c r="B11" s="664" t="n">
+        <x:f>B10/B7-1</x:f>
+        <x:v>0.15883031748482646</x:v>
+      </x:c>
+      <x:c r="C11" s="662" t="str">
+        <x:v>Upside to the research-date price</x:v>
+      </x:c>
+      <x:c r="D11" s="321"/>
+      <x:c r="E11" s="321"/>
+      <x:c r="F11" s="321"/>
+      <x:c r="G11" s="321"/>
+      <x:c r="H11" s="321"/>
+      <x:c r="I11" s="321"/>
+      <x:c r="J11" s="321"/>
+      <x:c r="K11" s="321"/>
+      <x:c r="L11" s="321"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="366" t="str">
+        <x:v>Conditional sale upside</x:v>
+      </x:c>
+      <x:c r="B12" s="661" t="n">
+        <x:f>Precedents!C26</x:f>
+        <x:v>5.851088223172894</x:v>
+      </x:c>
+      <x:c r="C12" s="366" t="str">
+        <x:v>US disposal at the precedent revenue median</x:v>
+      </x:c>
+      <x:c r="D12" s="321"/>
+      <x:c r="E12" s="321"/>
+      <x:c r="F12" s="321"/>
+      <x:c r="G12" s="321"/>
+      <x:c r="H12" s="321"/>
+      <x:c r="I12" s="321"/>
+      <x:c r="J12" s="321"/>
+      <x:c r="K12" s="321"/>
+      <x:c r="L12" s="321"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="370" t="str">
+        <x:v>Downside cross-check</x:v>
+      </x:c>
+      <x:c r="B13" s="665" t="n">
+        <x:f>'Trading Comps'!H25</x:f>
+        <x:v>3.9092088603532766</x:v>
+      </x:c>
+      <x:c r="C13" s="370" t="str">
+        <x:v>Revenue-multiple result; affected by peer margin differences</x:v>
+      </x:c>
+      <x:c r="D13" s="321"/>
+      <x:c r="E13" s="321"/>
+      <x:c r="F13" s="321"/>
+      <x:c r="G13" s="321"/>
+      <x:c r="H13" s="321"/>
+      <x:c r="I13" s="321"/>
+      <x:c r="J13" s="321"/>
+      <x:c r="K13" s="321"/>
+      <x:c r="L13" s="321"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="321"/>
+      <x:c r="B14" s="321"/>
+      <x:c r="C14" s="321"/>
+      <x:c r="D14" s="321"/>
+      <x:c r="E14" s="321"/>
+      <x:c r="F14" s="321"/>
+      <x:c r="G14" s="321"/>
+      <x:c r="H14" s="321"/>
+      <x:c r="I14" s="321"/>
+      <x:c r="J14" s="321"/>
+      <x:c r="K14" s="321"/>
+      <x:c r="L14" s="321"/>
+    </x:row>
+    <x:row r="15" ht="23" customHeight="1">
+      <x:c r="A15" s="660" t="str">
+        <x:v>Valuation triangulation</x:v>
+      </x:c>
+      <x:c r="B15" s="660"/>
+      <x:c r="C15" s="660"/>
+      <x:c r="D15" s="660"/>
+      <x:c r="E15" s="660"/>
+      <x:c r="F15" s="660"/>
+      <x:c r="G15" s="321"/>
+      <x:c r="H15" s="321"/>
+      <x:c r="I15" s="321"/>
+      <x:c r="J15" s="321"/>
+      <x:c r="K15" s="321"/>
+      <x:c r="L15" s="321"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="628" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="B16" s="628" t="str">
+        <x:v>Value / share</x:v>
+      </x:c>
+      <x:c r="C16" s="628" t="str">
+        <x:v>Vs current price</x:v>
+      </x:c>
+      <x:c r="D16" s="628" t="str">
+        <x:v>Weight</x:v>
+      </x:c>
+      <x:c r="E16" s="628" t="str">
+        <x:v>Weighted value</x:v>
+      </x:c>
+      <x:c r="F16" s="628" t="str">
+        <x:v>Role in conclusion</x:v>
+      </x:c>
+      <x:c r="G16" s="321"/>
+      <x:c r="H16" s="666" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="I16" s="666" t="str">
+        <x:v>Value / share</x:v>
+      </x:c>
+      <x:c r="J16" s="321"/>
+      <x:c r="K16" s="321"/>
+      <x:c r="L16" s="321"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="366" t="str">
+        <x:v>Revenue comps</x:v>
+      </x:c>
+      <x:c r="B17" s="661" t="n">
+        <x:f>'Trading Comps'!H25</x:f>
+        <x:v>3.9092088603532766</x:v>
+      </x:c>
+      <x:c r="C17" s="472" t="n">
+        <x:f>B17/$B$7-1</x:f>
+        <x:v>-0.1617114304764219</x:v>
+      </x:c>
+      <x:c r="D17" s="568" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="483" t="n">
+        <x:f>B17*D17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="366" t="str">
+        <x:v>Downside cross-check</x:v>
+      </x:c>
+      <x:c r="G17" s="321"/>
+      <x:c r="H17" s="666" t="str">
+        <x:v>Revenue comps</x:v>
+      </x:c>
+      <x:c r="I17" s="666" t="n">
+        <x:f>B17</x:f>
+        <x:v>3.9092088603532766</x:v>
+      </x:c>
+      <x:c r="J17" s="321"/>
+      <x:c r="K17" s="321"/>
+      <x:c r="L17" s="321"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="366" t="str">
+        <x:v>Operating-profit comps</x:v>
+      </x:c>
+      <x:c r="B18" s="661" t="n">
+        <x:f>'Trading Comps'!H26</x:f>
+        <x:v>5.2937326774027875</x:v>
+      </x:c>
+      <x:c r="C18" s="472" t="n">
+        <x:f>B18/$B$7-1</x:f>
+        <x:v>0.13518508529604878</x:v>
+      </x:c>
+      <x:c r="D18" s="568" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E18" s="483" t="n">
+        <x:f>B18*D18</x:f>
+        <x:v>2.6468663387013938</x:v>
+      </x:c>
+      <x:c r="F18" s="366" t="str">
+        <x:v>Core market evidence</x:v>
+      </x:c>
+      <x:c r="G18" s="321"/>
+      <x:c r="H18" s="666" t="str">
+        <x:v>EBIT comps</x:v>
+      </x:c>
+      <x:c r="I18" s="666" t="n">
+        <x:f>B18</x:f>
+        <x:v>5.2937326774027875</x:v>
+      </x:c>
+      <x:c r="J18" s="321"/>
+      <x:c r="K18" s="321"/>
+      <x:c r="L18" s="321"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="366" t="str">
+        <x:v>Base DCF</x:v>
+      </x:c>
+      <x:c r="B19" s="661" t="n">
+        <x:f>Forecast!B107</x:f>
+        <x:v>5.5089682185956175</x:v>
+      </x:c>
+      <x:c r="C19" s="472" t="n">
+        <x:f>B19/$B$7-1</x:f>
+        <x:v>0.18134007480481218</x:v>
+      </x:c>
+      <x:c r="D19" s="568" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E19" s="483" t="n">
+        <x:f>B19*D19</x:f>
+        <x:v>1.3772420546489044</x:v>
+      </x:c>
+      <x:c r="F19" s="366" t="str">
+        <x:v>Core intrinsic value</x:v>
+      </x:c>
+      <x:c r="G19" s="321"/>
+      <x:c r="H19" s="666" t="str">
+        <x:v>Base DCF</x:v>
+      </x:c>
+      <x:c r="I19" s="666" t="n">
+        <x:f>B19</x:f>
+        <x:v>5.5089682185956175</x:v>
+      </x:c>
+      <x:c r="J19" s="321"/>
+      <x:c r="K19" s="321"/>
+      <x:c r="L19" s="321"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="366" t="str">
+        <x:v>Restructuring DCF</x:v>
+      </x:c>
+      <x:c r="B20" s="661" t="n">
+        <x:f>Forecast!B173</x:f>
+        <x:v>5.519558386657466</x:v>
+      </x:c>
+      <x:c r="C20" s="472" t="n">
+        <x:f>B20/$B$7-1</x:f>
+        <x:v>0.18361102454239653</x:v>
+      </x:c>
+      <x:c r="D20" s="568" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="E20" s="483" t="n">
+        <x:f>B20*D20</x:f>
+        <x:v>1.3798895966643665</x:v>
+      </x:c>
+      <x:c r="F20" s="366" t="str">
+        <x:v>Core strategic alternative</x:v>
+      </x:c>
+      <x:c r="G20" s="321"/>
+      <x:c r="H20" s="666" t="str">
+        <x:v>Restructuring</x:v>
+      </x:c>
+      <x:c r="I20" s="666" t="n">
+        <x:f>B20</x:f>
+        <x:v>5.519558386657466</x:v>
+      </x:c>
+      <x:c r="J20" s="321"/>
+      <x:c r="K20" s="321"/>
+      <x:c r="L20" s="321"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="366" t="str">
+        <x:v>US disposal at 1.00x</x:v>
+      </x:c>
+      <x:c r="B21" s="661" t="n">
+        <x:f>Forecast!B255</x:f>
+        <x:v>5.442716472666101</x:v>
+      </x:c>
+      <x:c r="C21" s="472" t="n">
+        <x:f>B21/$B$7-1</x:f>
+        <x:v>0.16713308732789467</x:v>
+      </x:c>
+      <x:c r="D21" s="568" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="483" t="n">
+        <x:f>B21*D21</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="366" t="str">
+        <x:v>Conservative sale case</x:v>
+      </x:c>
+      <x:c r="G21" s="321"/>
+      <x:c r="H21" s="666" t="str">
+        <x:v>Disposal 1.0x</x:v>
+      </x:c>
+      <x:c r="I21" s="666" t="n">
+        <x:f>B21</x:f>
+        <x:v>5.442716472666101</x:v>
+      </x:c>
+      <x:c r="J21" s="321"/>
+      <x:c r="K21" s="321"/>
+      <x:c r="L21" s="321"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="366" t="str">
+        <x:v>US disposal at precedent median</x:v>
+      </x:c>
+      <x:c r="B22" s="661" t="n">
+        <x:f>Precedents!C26</x:f>
+        <x:v>5.851088223172894</x:v>
+      </x:c>
+      <x:c r="C22" s="472" t="n">
+        <x:f>B22/$B$7-1</x:f>
+        <x:v>0.2547040979326447</x:v>
+      </x:c>
+      <x:c r="D22" s="568" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="483" t="n">
+        <x:f>B22*D22</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="366" t="str">
+        <x:v>Conditional transaction upside</x:v>
+      </x:c>
+      <x:c r="G22" s="321"/>
+      <x:c r="H22" s="666" t="str">
+        <x:v>Disposal median</x:v>
+      </x:c>
+      <x:c r="I22" s="666" t="n">
+        <x:f>B22</x:f>
+        <x:v>5.851088223172894</x:v>
+      </x:c>
+      <x:c r="J22" s="321"/>
+      <x:c r="K22" s="321"/>
+      <x:c r="L22" s="321"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="667" t="str">
+        <x:v>Illustrative central value</x:v>
+      </x:c>
+      <x:c r="B23" s="668"/>
+      <x:c r="C23" s="667"/>
+      <x:c r="D23" s="667"/>
+      <x:c r="E23" s="668" t="n">
+        <x:f>SUM(E17:E22)</x:f>
+        <x:v>5.403997990014664</x:v>
+      </x:c>
+      <x:c r="F23" s="667" t="str">
+        <x:v>50% market evidence; 50% DCF evidence</x:v>
+      </x:c>
+      <x:c r="G23" s="321"/>
+      <x:c r="H23" s="321"/>
+      <x:c r="I23" s="321"/>
+      <x:c r="J23" s="321"/>
+      <x:c r="K23" s="321"/>
+      <x:c r="L23" s="321"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="321"/>
+      <x:c r="B24" s="321"/>
+      <x:c r="C24" s="321"/>
+      <x:c r="D24" s="321"/>
+      <x:c r="E24" s="321"/>
+      <x:c r="F24" s="321"/>
+      <x:c r="G24" s="321"/>
+      <x:c r="H24" s="321"/>
+      <x:c r="I24" s="321"/>
+      <x:c r="J24" s="321"/>
+      <x:c r="K24" s="321"/>
+      <x:c r="L24" s="321"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="321"/>
+      <x:c r="B25" s="321"/>
+      <x:c r="C25" s="321"/>
+      <x:c r="D25" s="321"/>
+      <x:c r="E25" s="321"/>
+      <x:c r="F25" s="321"/>
+      <x:c r="G25" s="321"/>
+      <x:c r="H25" s="321"/>
+      <x:c r="I25" s="321"/>
+      <x:c r="J25" s="321"/>
+      <x:c r="K25" s="321"/>
+      <x:c r="L25" s="321"/>
+    </x:row>
+    <x:row r="26" ht="23" customHeight="1">
+      <x:c r="A26" s="660" t="str">
+        <x:v>US sale decision</x:v>
+      </x:c>
+      <x:c r="B26" s="660"/>
+      <x:c r="C26" s="660"/>
+      <x:c r="D26" s="660"/>
+      <x:c r="E26" s="660"/>
+      <x:c r="F26" s="660"/>
+      <x:c r="G26" s="321"/>
+      <x:c r="H26" s="321"/>
+      <x:c r="I26" s="321"/>
+      <x:c r="J26" s="321"/>
+      <x:c r="K26" s="321"/>
+      <x:c r="L26" s="321"/>
+    </x:row>
+    <x:row r="27" ht="30" customHeight="1">
+      <x:c r="A27" s="628" t="str">
+        <x:v>Sale EV / revenue</x:v>
+      </x:c>
+      <x:c r="B27" s="628" t="str">
+        <x:v>Value / share</x:v>
+      </x:c>
+      <x:c r="C27" s="628" t="str">
+        <x:v>Vs base DCF</x:v>
+      </x:c>
+      <x:c r="D27" s="628" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+      <x:c r="E27" s="321"/>
+      <x:c r="F27" s="321"/>
+      <x:c r="G27" s="321"/>
+      <x:c r="H27" s="321"/>
+      <x:c r="I27" s="321"/>
+      <x:c r="J27" s="321"/>
+      <x:c r="K27" s="321"/>
+      <x:c r="L27" s="321"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="669" t="n">
+        <x:f>Forecast!B199</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B28" s="670" t="n">
+        <x:f>Forecast!B255</x:f>
+        <x:v>5.442716472666101</x:v>
+      </x:c>
+      <x:c r="C28" s="670" t="n">
+        <x:f>B28-Forecast!$B$107</x:f>
+        <x:v>-0.06625174592951666</x:v>
+      </x:c>
+      <x:c r="D28" s="671" t="str">
+        <x:v>Reject: below standalone value</x:v>
+      </x:c>
+      <x:c r="E28" s="321"/>
+      <x:c r="F28" s="321"/>
+      <x:c r="G28" s="321"/>
+      <x:c r="H28" s="321"/>
+      <x:c r="I28" s="321"/>
+      <x:c r="J28" s="321"/>
+      <x:c r="K28" s="321"/>
+      <x:c r="L28" s="321"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="672" t="n">
+        <x:f>Forecast!B203</x:f>
+        <x:v>1.1322097486901377</x:v>
+      </x:c>
+      <x:c r="B29" s="673" t="n">
+        <x:f>Forecast!B107</x:f>
+        <x:v>5.5089682185956175</x:v>
+      </x:c>
+      <x:c r="C29" s="673" t="n">
+        <x:f>B29-Forecast!$B$107</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="674" t="str">
+        <x:v>Economic break-even only</x:v>
+      </x:c>
+      <x:c r="E29" s="321"/>
+      <x:c r="F29" s="321"/>
+      <x:c r="G29" s="321"/>
+      <x:c r="H29" s="321"/>
+      <x:c r="I29" s="321"/>
+      <x:c r="J29" s="321"/>
+      <x:c r="K29" s="321"/>
+      <x:c r="L29" s="321"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="675" t="n">
+        <x:f>1.25</x:f>
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="B30" s="676" t="n">
+        <x:f>(Forecast!$B$249+Forecast!$B$193*A30*(1-Forecast!$B$201)-Forecast!$B$104)/Forecast!$B$106</x:f>
+        <x:v>5.567994197239937</x:v>
+      </x:c>
+      <x:c r="C30" s="676" t="n">
+        <x:f>B30-Forecast!$B$107</x:f>
+        <x:v>0.059025978644319466</x:v>
+      </x:c>
+      <x:c r="D30" s="677" t="str">
+        <x:v>Minimum discussion point; limited value creation</x:v>
+      </x:c>
+      <x:c r="E30" s="321"/>
+      <x:c r="F30" s="321"/>
+      <x:c r="G30" s="321"/>
+      <x:c r="H30" s="321"/>
+      <x:c r="I30" s="321"/>
+      <x:c r="J30" s="321"/>
+      <x:c r="K30" s="321"/>
+      <x:c r="L30" s="321"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="675" t="n">
+        <x:f>1.50</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="B31" s="676" t="n">
+        <x:f>(Forecast!$B$249+Forecast!$B$193*A31*(1-Forecast!$B$201)-Forecast!$B$104)/Forecast!$B$106</x:f>
+        <x:v>5.693271921813774</x:v>
+      </x:c>
+      <x:c r="C31" s="676" t="n">
+        <x:f>B31-Forecast!$B$107</x:f>
+        <x:v>0.18430370321815648</x:v>
+      </x:c>
+      <x:c r="D31" s="677" t="str">
+        <x:v>Preferred level with a stronger risk buffer</x:v>
+      </x:c>
+      <x:c r="E31" s="321"/>
+      <x:c r="F31" s="321"/>
+      <x:c r="G31" s="321"/>
+      <x:c r="H31" s="321"/>
+      <x:c r="I31" s="321"/>
+      <x:c r="J31" s="321"/>
+      <x:c r="K31" s="321"/>
+      <x:c r="L31" s="321"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="678" t="n">
+        <x:f>Precedents!G12</x:f>
+        <x:v>1.8149328859060403</x:v>
+      </x:c>
+      <x:c r="B32" s="679" t="n">
+        <x:f>Precedents!C26</x:f>
+        <x:v>5.851088223172894</x:v>
+      </x:c>
+      <x:c r="C32" s="679" t="n">
+        <x:f>B32-Forecast!$B$107</x:f>
+        <x:v>0.34212000457727676</x:v>
+      </x:c>
+      <x:c r="D32" s="680" t="str">
+        <x:v>Conditional precedent-median upside</x:v>
+      </x:c>
+      <x:c r="E32" s="321"/>
+      <x:c r="F32" s="321"/>
+      <x:c r="G32" s="321"/>
+      <x:c r="H32" s="321"/>
+      <x:c r="I32" s="321"/>
+      <x:c r="J32" s="321"/>
+      <x:c r="K32" s="321"/>
+      <x:c r="L32" s="321"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="321"/>
+      <x:c r="B33" s="321"/>
+      <x:c r="C33" s="321"/>
+      <x:c r="D33" s="321"/>
+      <x:c r="E33" s="321"/>
+      <x:c r="F33" s="321"/>
+      <x:c r="G33" s="321"/>
+      <x:c r="H33" s="321"/>
+      <x:c r="I33" s="321"/>
+      <x:c r="J33" s="321"/>
+      <x:c r="K33" s="321"/>
+      <x:c r="L33" s="321"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="321"/>
+      <x:c r="B34" s="321"/>
+      <x:c r="C34" s="321"/>
+      <x:c r="D34" s="321"/>
+      <x:c r="E34" s="321"/>
+      <x:c r="F34" s="321"/>
+      <x:c r="G34" s="321"/>
+      <x:c r="H34" s="321"/>
+      <x:c r="I34" s="321"/>
+      <x:c r="J34" s="321"/>
+      <x:c r="K34" s="321"/>
+      <x:c r="L34" s="321"/>
+    </x:row>
+    <x:row r="35" ht="28" customHeight="1">
+      <x:c r="A35" s="651" t="str">
+        <x:v>Recommendation: continue improving the US operation while maintaining a competitive sale process. Do not sell near 1.00x revenue. Treat 1.13x as mathematical break-even, not a target. Require at least approximately 1.25x, with a price closer to 1.50x preferable after considering tax, separation costs, stranded overhead and transaction certainty. If bids remain below that range, retaining the business is more defensible.</x:v>
+      </x:c>
+      <x:c r="B35" s="651"/>
+      <x:c r="C35" s="651"/>
+      <x:c r="D35" s="651"/>
+      <x:c r="E35" s="651"/>
+      <x:c r="F35" s="651"/>
+      <x:c r="G35" s="651"/>
+      <x:c r="H35" s="651"/>
+      <x:c r="I35" s="651"/>
+      <x:c r="J35" s="651"/>
+      <x:c r="K35" s="651"/>
+      <x:c r="L35" s="651"/>
+    </x:row>
+    <x:row r="36" ht="28" customHeight="1">
+      <x:c r="A36" s="651"/>
+      <x:c r="B36" s="651"/>
+      <x:c r="C36" s="651"/>
+      <x:c r="D36" s="651"/>
+      <x:c r="E36" s="651"/>
+      <x:c r="F36" s="651"/>
+      <x:c r="G36" s="651"/>
+      <x:c r="H36" s="651"/>
+      <x:c r="I36" s="651"/>
+      <x:c r="J36" s="651"/>
+      <x:c r="K36" s="651"/>
+      <x:c r="L36" s="651"/>
+    </x:row>
+    <x:row r="37" ht="28" customHeight="1">
+      <x:c r="A37" s="651"/>
+      <x:c r="B37" s="651"/>
+      <x:c r="C37" s="651"/>
+      <x:c r="D37" s="651"/>
+      <x:c r="E37" s="651"/>
+      <x:c r="F37" s="651"/>
+      <x:c r="G37" s="651"/>
+      <x:c r="H37" s="651"/>
+      <x:c r="I37" s="651"/>
+      <x:c r="J37" s="651"/>
+      <x:c r="K37" s="651"/>
+      <x:c r="L37" s="651"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="321"/>
+      <x:c r="B38" s="321"/>
+      <x:c r="C38" s="321"/>
+      <x:c r="D38" s="321"/>
+      <x:c r="E38" s="321"/>
+      <x:c r="F38" s="321"/>
+      <x:c r="G38" s="321"/>
+      <x:c r="H38" s="321"/>
+      <x:c r="I38" s="321"/>
+      <x:c r="J38" s="321"/>
+      <x:c r="K38" s="321"/>
+      <x:c r="L38" s="321"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="321"/>
+      <x:c r="B39" s="321"/>
+      <x:c r="C39" s="321"/>
+      <x:c r="D39" s="321"/>
+      <x:c r="E39" s="321"/>
+      <x:c r="F39" s="321"/>
+      <x:c r="G39" s="321"/>
+      <x:c r="H39" s="321"/>
+      <x:c r="I39" s="321"/>
+      <x:c r="J39" s="321"/>
+      <x:c r="K39" s="321"/>
+      <x:c r="L39" s="321"/>
+    </x:row>
+    <x:row r="40" ht="23" customHeight="1">
+      <x:c r="A40" s="660" t="str">
+        <x:v>Main risks</x:v>
+      </x:c>
+      <x:c r="B40" s="660"/>
+      <x:c r="C40" s="660"/>
+      <x:c r="D40" s="660"/>
+      <x:c r="E40" s="660"/>
+      <x:c r="F40" s="660"/>
+      <x:c r="G40" s="660"/>
+      <x:c r="H40" s="660"/>
+      <x:c r="I40" s="660"/>
+      <x:c r="J40" s="660"/>
+      <x:c r="K40" s="660"/>
+      <x:c r="L40" s="660"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="608" t="str">
+        <x:v>Terminal value</x:v>
+      </x:c>
+      <x:c r="B41" s="681" t="str">
+        <x:v>Approximately 74% of base enterprise value comes from terminal value.</x:v>
+      </x:c>
+      <x:c r="C41" s="681"/>
+      <x:c r="D41" s="681"/>
+      <x:c r="E41" s="681"/>
+      <x:c r="F41" s="681"/>
+      <x:c r="G41" s="681"/>
+      <x:c r="H41" s="681"/>
+      <x:c r="I41" s="681"/>
+      <x:c r="J41" s="681"/>
+      <x:c r="K41" s="681"/>
+      <x:c r="L41" s="681"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="608" t="str">
+        <x:v>US execution</x:v>
+      </x:c>
+      <x:c r="B42" s="681" t="str">
+        <x:v>Global Solutions has volatile margins and weaker contracted-revenue visibility.</x:v>
+      </x:c>
+      <x:c r="C42" s="681"/>
+      <x:c r="D42" s="681"/>
+      <x:c r="E42" s="681"/>
+      <x:c r="F42" s="681"/>
+      <x:c r="G42" s="681"/>
+      <x:c r="H42" s="681"/>
+      <x:c r="I42" s="681"/>
+      <x:c r="J42" s="681"/>
+      <x:c r="K42" s="681"/>
+      <x:c r="L42" s="681"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="608" t="str">
+        <x:v>Transaction deductions</x:v>
+      </x:c>
+      <x:c r="B43" s="681" t="str">
+        <x:v>Tax, fees, separation costs and stranded overhead may exceed the 10% allowance.</x:v>
+      </x:c>
+      <x:c r="C43" s="681"/>
+      <x:c r="D43" s="681"/>
+      <x:c r="E43" s="681"/>
+      <x:c r="F43" s="681"/>
+      <x:c r="G43" s="681"/>
+      <x:c r="H43" s="681"/>
+      <x:c r="I43" s="681"/>
+      <x:c r="J43" s="681"/>
+      <x:c r="K43" s="681"/>
+      <x:c r="L43" s="681"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="608" t="str">
+        <x:v>Comparable differences</x:v>
+      </x:c>
+      <x:c r="B44" s="681" t="str">
+        <x:v>Peers have different margins, business mixes and accounting definitions.</x:v>
+      </x:c>
+      <x:c r="C44" s="681"/>
+      <x:c r="D44" s="681"/>
+      <x:c r="E44" s="681"/>
+      <x:c r="F44" s="681"/>
+      <x:c r="G44" s="681"/>
+      <x:c r="H44" s="681"/>
+      <x:c r="I44" s="681"/>
+      <x:c r="J44" s="681"/>
+      <x:c r="K44" s="681"/>
+      <x:c r="L44" s="681"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="608" t="str">
+        <x:v>Precedent premiums</x:v>
+      </x:c>
+      <x:c r="B45" s="681" t="str">
+        <x:v>Historical deals include control premiums, synergies and stronger assets.</x:v>
+      </x:c>
+      <x:c r="C45" s="681"/>
+      <x:c r="D45" s="681"/>
+      <x:c r="E45" s="681"/>
+      <x:c r="F45" s="681"/>
+      <x:c r="G45" s="681"/>
+      <x:c r="H45" s="681"/>
+      <x:c r="I45" s="681"/>
+      <x:c r="J45" s="681"/>
+      <x:c r="K45" s="681"/>
+      <x:c r="L45" s="681"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="682" t="str">
+        <x:v>Market-date sensitivity</x:v>
+      </x:c>
+      <x:c r="B46" s="499" t="str">
+        <x:v>Share prices and WACC inputs should be refreshed before presenting the conclusion.</x:v>
+      </x:c>
+      <x:c r="C46" s="499"/>
+      <x:c r="D46" s="499"/>
+      <x:c r="E46" s="499"/>
+      <x:c r="F46" s="499"/>
+      <x:c r="G46" s="499"/>
+      <x:c r="H46" s="499"/>
+      <x:c r="I46" s="499"/>
+      <x:c r="J46" s="499"/>
+      <x:c r="K46" s="499"/>
+      <x:c r="L46" s="499"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="321"/>
+      <x:c r="B47" s="321"/>
+      <x:c r="C47" s="321"/>
+      <x:c r="D47" s="321"/>
+      <x:c r="E47" s="321"/>
+      <x:c r="F47" s="321"/>
+      <x:c r="G47" s="321"/>
+      <x:c r="H47" s="321"/>
+      <x:c r="I47" s="321"/>
+      <x:c r="J47" s="321"/>
+      <x:c r="K47" s="321"/>
+      <x:c r="L47" s="321"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="321"/>
+      <x:c r="B48" s="321"/>
+      <x:c r="C48" s="321"/>
+      <x:c r="D48" s="321"/>
+      <x:c r="E48" s="321"/>
+      <x:c r="F48" s="321"/>
+      <x:c r="G48" s="321"/>
+      <x:c r="H48" s="321"/>
+      <x:c r="I48" s="321"/>
+      <x:c r="J48" s="321"/>
+      <x:c r="K48" s="321"/>
+      <x:c r="L48" s="321"/>
+    </x:row>
+    <x:row r="49" ht="28" customHeight="1">
+      <x:c r="A49" s="622" t="str">
+        <x:v>Interview answer: I triangulated the valuation rather than relying on one method. The EBIT trading comparable implied £5.29 per share, while the base and restructuring DCFs implied £5.51 and £5.52. This produced a core range of £5.29-£5.52 and a central reference of about £5.40. For the US business, 1.13x revenue is only mathematical break-even. I would continue improving the operation while running a sale process and would prefer a bid closer to 1.50x revenue before recommending disposal.</x:v>
+      </x:c>
+      <x:c r="B49" s="622"/>
+      <x:c r="C49" s="622"/>
+      <x:c r="D49" s="622"/>
+      <x:c r="E49" s="622"/>
+      <x:c r="F49" s="622"/>
+      <x:c r="G49" s="622"/>
+      <x:c r="H49" s="622"/>
+      <x:c r="I49" s="622"/>
+      <x:c r="J49" s="622"/>
+      <x:c r="K49" s="622"/>
+      <x:c r="L49" s="622"/>
+    </x:row>
+    <x:row r="50" ht="28" customHeight="1">
+      <x:c r="A50" s="622"/>
+      <x:c r="B50" s="622"/>
+      <x:c r="C50" s="622"/>
+      <x:c r="D50" s="622"/>
+      <x:c r="E50" s="622"/>
+      <x:c r="F50" s="622"/>
+      <x:c r="G50" s="622"/>
+      <x:c r="H50" s="622"/>
+      <x:c r="I50" s="622"/>
+      <x:c r="J50" s="622"/>
+      <x:c r="K50" s="622"/>
+      <x:c r="L50" s="622"/>
+    </x:row>
+    <x:row r="51" ht="28" customHeight="1">
+      <x:c r="A51" s="622"/>
+      <x:c r="B51" s="622"/>
+      <x:c r="C51" s="622"/>
+      <x:c r="D51" s="622"/>
+      <x:c r="E51" s="622"/>
+      <x:c r="F51" s="622"/>
+      <x:c r="G51" s="622"/>
+      <x:c r="H51" s="622"/>
+      <x:c r="I51" s="622"/>
+      <x:c r="J51" s="622"/>
+      <x:c r="K51" s="622"/>
+      <x:c r="L51" s="622"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L3"/>
+    <x:mergeCell ref="A5:F5"/>
+    <x:mergeCell ref="A15:F15"/>
+    <x:mergeCell ref="A23:D23"/>
+    <x:mergeCell ref="A26:F26"/>
+    <x:mergeCell ref="A35:L37"/>
+    <x:mergeCell ref="A40:L40"/>
+    <x:mergeCell ref="B41:L41"/>
+    <x:mergeCell ref="B42:L42"/>
+    <x:mergeCell ref="B43:L43"/>
+    <x:mergeCell ref="B44:L44"/>
+    <x:mergeCell ref="B45:L45"/>
+    <x:mergeCell ref="B46:L46"/>
+    <x:mergeCell ref="A49:L51"/>
+    <x:mergeCell ref="C6:F6"/>
+    <x:mergeCell ref="C7:F7"/>
+    <x:mergeCell ref="C8:F8"/>
+    <x:mergeCell ref="C9:F9"/>
+    <x:mergeCell ref="C10:F10"/>
+    <x:mergeCell ref="C11:F11"/>
+    <x:mergeCell ref="C12:F12"/>
+    <x:mergeCell ref="C13:F13"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf636d44ecd0b462d"/>
+</x:worksheet>
 </file>
</xml_diff>